<commit_message>
Actualizacion automatica de datos Asana y KPI 2026-06-18 20:37 UTC
</commit_message>
<xml_diff>
--- a/data/50001490 - ZITRON PERU METRO LIMA PV04-PV05.xlsx
+++ b/data/50001490 - ZITRON PERU METRO LIMA PV04-PV05.xlsx
@@ -3347,7 +3347,7 @@
       </c>
       <c r="C31" s="9"/>
       <c r="D31" s="8">
-        <v>46139.543415625</v>
+        <v>46191.83935533564</v>
       </c>
       <c r="E31" s="9" t="s">
         <v>118</v>
@@ -3392,9 +3392,11 @@
       <c r="B32" s="5">
         <v>46073.69994704861</v>
       </c>
-      <c r="C32" s="6"/>
+      <c r="C32" s="5">
+        <v>46191.839348587964</v>
+      </c>
       <c r="D32" s="5">
-        <v>46182.683637118054</v>
+        <v>46191.83935060185</v>
       </c>
       <c r="E32" s="6" t="s">
         <v>121</v>
@@ -3516,9 +3518,11 @@
       <c r="B34" s="5">
         <v>46073.69994769676</v>
       </c>
-      <c r="C34" s="6"/>
+      <c r="C34" s="5">
+        <v>46191.83755203703</v>
+      </c>
       <c r="D34" s="5">
-        <v>46182.68363659723</v>
+        <v>46191.83755358796</v>
       </c>
       <c r="E34" s="6" t="s">
         <v>130</v>
@@ -3758,9 +3762,11 @@
       <c r="B38" s="5">
         <v>46073.69994892361</v>
       </c>
-      <c r="C38" s="6"/>
+      <c r="C38" s="5">
+        <v>46191.836712743054</v>
+      </c>
       <c r="D38" s="5">
-        <v>46182.67567175926</v>
+        <v>46191.83671528935</v>
       </c>
       <c r="E38" s="6" t="s">
         <v>142</v>
@@ -4553,9 +4559,11 @@
       <c r="B51" s="8">
         <v>46077.579487986106</v>
       </c>
-      <c r="C51" s="9"/>
+      <c r="C51" s="8">
+        <v>46191.83738681713</v>
+      </c>
       <c r="D51" s="8">
-        <v>46182.68337946759</v>
+        <v>46191.83738863426</v>
       </c>
       <c r="E51" s="9" t="s">
         <v>183</v>
@@ -4901,9 +4909,11 @@
       <c r="B57" s="8">
         <v>46139.543413900465</v>
       </c>
-      <c r="C57" s="9"/>
+      <c r="C57" s="8">
+        <v>46191.840089791665</v>
+      </c>
       <c r="D57" s="8">
-        <v>46185.72120696759</v>
+        <v>46191.84009155093</v>
       </c>
       <c r="E57" s="9" t="s">
         <v>198</v>
@@ -4964,9 +4974,11 @@
       <c r="B58" s="5">
         <v>46139.543700821756</v>
       </c>
-      <c r="C58" s="6"/>
+      <c r="C58" s="5">
+        <v>46191.839869421296</v>
+      </c>
       <c r="D58" s="5">
-        <v>46177.56878042824</v>
+        <v>46191.83987099537</v>
       </c>
       <c r="E58" s="6" t="s">
         <v>116</v>
@@ -5017,9 +5029,11 @@
       <c r="B59" s="8">
         <v>46139.54378479166</v>
       </c>
-      <c r="C59" s="9"/>
+      <c r="C59" s="8">
+        <v>46191.83995417824</v>
+      </c>
       <c r="D59" s="8">
-        <v>46177.16872760416</v>
+        <v>46191.83995613426</v>
       </c>
       <c r="E59" s="9" t="s">
         <v>205</v>
@@ -5957,7 +5971,7 @@
       </c>
       <c r="C75" s="9"/>
       <c r="D75" s="8">
-        <v>46134.17255372685</v>
+        <v>46191.8375600463</v>
       </c>
       <c r="E75" s="9" t="s">
         <v>264</v>

</xml_diff>

<commit_message>
Actualizacion automatica de datos Asana y KPI 2026-06-22 14:51 UTC
</commit_message>
<xml_diff>
--- a/data/50001490 - ZITRON PERU METRO LIMA PV04-PV05.xlsx
+++ b/data/50001490 - ZITRON PERU METRO LIMA PV04-PV05.xlsx
@@ -5389,7 +5389,7 @@
       </c>
       <c r="C65" s="9"/>
       <c r="D65" s="8">
-        <v>46077.627563472226</v>
+        <v>46195.6020638426</v>
       </c>
       <c r="E65" s="9" t="s">
         <v>228</v>
@@ -5434,9 +5434,11 @@
       <c r="B66" s="5">
         <v>46073.69994689815</v>
       </c>
-      <c r="C66" s="6"/>
+      <c r="C66" s="5">
+        <v>46195.60205410879</v>
+      </c>
       <c r="D66" s="5">
-        <v>46132.578650428244</v>
+        <v>46195.60205646991</v>
       </c>
       <c r="E66" s="6" t="s">
         <v>231</v>
@@ -5499,7 +5501,7 @@
       </c>
       <c r="C67" s="9"/>
       <c r="D67" s="8">
-        <v>46092.503911493055</v>
+        <v>46195.60206259259</v>
       </c>
       <c r="E67" s="9" t="s">
         <v>236</v>
@@ -5798,7 +5800,7 @@
       </c>
       <c r="C72" s="6"/>
       <c r="D72" s="5">
-        <v>46077.631060694446</v>
+        <v>46195.604225717594</v>
       </c>
       <c r="E72" s="6" t="s">
         <v>228</v>
@@ -6032,9 +6034,11 @@
       <c r="B76" s="5">
         <v>46073.69994708333</v>
       </c>
-      <c r="C76" s="6"/>
+      <c r="C76" s="5">
+        <v>46195.603957824074</v>
+      </c>
       <c r="D76" s="5">
-        <v>46148.25044650463</v>
+        <v>46195.603959687505</v>
       </c>
       <c r="E76" s="6" t="s">
         <v>267</v>
@@ -6095,9 +6099,11 @@
       <c r="B77" s="8">
         <v>46076.88127923611</v>
       </c>
-      <c r="C77" s="9"/>
+      <c r="C77" s="8">
+        <v>46195.60421921297</v>
+      </c>
       <c r="D77" s="8">
-        <v>46128.661488854166</v>
+        <v>46195.60422127315</v>
       </c>
       <c r="E77" s="9" t="s">
         <v>270</v>
@@ -6158,9 +6164,11 @@
       <c r="B78" s="5">
         <v>46077.57961084491</v>
       </c>
-      <c r="C78" s="6"/>
+      <c r="C78" s="5">
+        <v>46195.60466336805</v>
+      </c>
       <c r="D78" s="5">
-        <v>46174.651739594905</v>
+        <v>46195.60466490741</v>
       </c>
       <c r="E78" s="6" t="s">
         <v>273</v>
@@ -6396,7 +6404,7 @@
       </c>
       <c r="C82" s="6"/>
       <c r="D82" s="5">
-        <v>46150.168837708334</v>
+        <v>46195.60396552083</v>
       </c>
       <c r="E82" s="6" t="s">
         <v>284</v>
@@ -6585,7 +6593,7 @@
       </c>
       <c r="C85" s="9"/>
       <c r="D85" s="8">
-        <v>46133.18400270834</v>
+        <v>46195.60422616898</v>
       </c>
       <c r="E85" s="9" t="s">
         <v>295</v>
@@ -6884,7 +6892,7 @@
       </c>
       <c r="C90" s="6"/>
       <c r="D90" s="5">
-        <v>46160.25052104167</v>
+        <v>46195.604670092594</v>
       </c>
       <c r="E90" s="6" t="s">
         <v>274</v>

</xml_diff>

<commit_message>
Actualizacion automatica de datos Asana y KPI 2026-06-25 15:07 UTC
</commit_message>
<xml_diff>
--- a/data/50001490 - ZITRON PERU METRO LIMA PV04-PV05.xlsx
+++ b/data/50001490 - ZITRON PERU METRO LIMA PV04-PV05.xlsx
@@ -6404,7 +6404,7 @@
       </c>
       <c r="C82" s="6"/>
       <c r="D82" s="5">
-        <v>46197.58394950231</v>
+        <v>46198.59349042824</v>
       </c>
       <c r="E82" s="6" t="s">
         <v>284</v>
@@ -6467,7 +6467,7 @@
       </c>
       <c r="C83" s="9"/>
       <c r="D83" s="8">
-        <v>46197.583529641204</v>
+        <v>46198.592367060184</v>
       </c>
       <c r="E83" s="9" t="s">
         <v>288</v>
@@ -6530,7 +6530,7 @@
       </c>
       <c r="C84" s="6"/>
       <c r="D84" s="5">
-        <v>46197.583207523145</v>
+        <v>46198.59272494213</v>
       </c>
       <c r="E84" s="6" t="s">
         <v>291</v>

</xml_diff>

<commit_message>
Actualizacion automatica de datos Asana y KPI 2026-06-26 21:10 UTC
</commit_message>
<xml_diff>
--- a/data/50001490 - ZITRON PERU METRO LIMA PV04-PV05.xlsx
+++ b/data/50001490 - ZITRON PERU METRO LIMA PV04-PV05.xlsx
@@ -5436,7 +5436,7 @@
       </c>
       <c r="C66" s="6"/>
       <c r="D66" s="5">
-        <v>46198.822638171296</v>
+        <v>46199.82444644676</v>
       </c>
       <c r="E66" s="6" t="s">
         <v>231</v>
@@ -5845,7 +5845,7 @@
       </c>
       <c r="C73" s="9"/>
       <c r="D73" s="8">
-        <v>46198.8234224537</v>
+        <v>46199.830143969906</v>
       </c>
       <c r="E73" s="9" t="s">
         <v>259</v>
@@ -5971,7 +5971,7 @@
       </c>
       <c r="C75" s="9"/>
       <c r="D75" s="8">
-        <v>46198.823039097224</v>
+        <v>46199.82646660879</v>
       </c>
       <c r="E75" s="9" t="s">
         <v>264</v>

</xml_diff>

<commit_message>
Actualizacion automatica de datos Asana y KPI 2026-07-02 19:30 UTC
</commit_message>
<xml_diff>
--- a/data/50001490 - ZITRON PERU METRO LIMA PV04-PV05.xlsx
+++ b/data/50001490 - ZITRON PERU METRO LIMA PV04-PV05.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1207" uniqueCount="337">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1218" uniqueCount="339">
   <si>
     <t xml:space="preserve">50001490-ZITRON PERU METRO DE LIMA PV04-PV05 </t>
   </si>
@@ -631,6 +631,18 @@
     <t xml:space="preserve">Fabricacion externa OT 4204 - 4205 </t>
   </si>
   <si>
+    <t>1216239551129098</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Control de calidad  fabricacion externa </t>
+  </si>
+  <si>
+    <t>Nicolás López</t>
+  </si>
+  <si>
+    <t>nicolas.lopez@zitron.com</t>
+  </si>
+  <si>
     <t>1213380177588299</t>
   </si>
   <si>
@@ -722,12 +734,6 @@
   </si>
   <si>
     <t>Control de calidad compras materiales a codigo // compras locale aprovisionamiento</t>
-  </si>
-  <si>
-    <t>Nicolás López</t>
-  </si>
-  <si>
-    <t>nicolas.lopez@zitron.com</t>
   </si>
   <si>
     <t>Bodega:,Preparación Materiales</t>
@@ -1545,7 +1551,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:U98"/>
+  <dimension ref="A1:U99"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="10.4" customWidth="1"/>
@@ -4913,7 +4919,7 @@
         <v>46191.840089791665</v>
       </c>
       <c r="D57" s="8">
-        <v>46191.84009155093</v>
+        <v>46205.80892784722</v>
       </c>
       <c r="E57" s="9" t="s">
         <v>198</v>
@@ -5082,24 +5088,28 @@
         <v>206</v>
       </c>
       <c r="B60" s="5">
-        <v>46073.69994815972</v>
+        <v>46205.80892462963</v>
       </c>
       <c r="C60" s="6"/>
       <c r="D60" s="5">
-        <v>46129.586425601854</v>
+        <v>46205.80976949074</v>
       </c>
       <c r="E60" s="6" t="s">
         <v>207</v>
       </c>
       <c r="F60" s="6" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G60" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="H60" s="6"/>
+        <v>208</v>
+      </c>
+      <c r="H60" s="6" t="s">
+        <v>209</v>
+      </c>
       <c r="I60" s="6"/>
-      <c r="J60" s="6"/>
+      <c r="J60" s="5">
+        <v>46205</v>
+      </c>
       <c r="K60" s="6" t="s">
         <v>26</v>
       </c>
@@ -5107,13 +5117,13 @@
         <v>26</v>
       </c>
       <c r="M60" s="6" t="s">
-        <v>0</v>
+        <v>26</v>
       </c>
       <c r="N60" s="6" t="s">
-        <v>26</v>
+        <v>198</v>
       </c>
       <c r="O60" s="6" t="s">
-        <v>208</v>
+        <v>26</v>
       </c>
       <c r="P60" s="6" t="s">
         <v>26</v>
@@ -5126,84 +5136,66 @@
     </row>
     <row r="61" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A61" s="7" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="B61" s="8">
-        <v>46073.6999484375</v>
-      </c>
-      <c r="C61" s="8">
-        <v>46099.54242106482</v>
-      </c>
+        <v>46073.69994815972</v>
+      </c>
+      <c r="C61" s="9"/>
       <c r="D61" s="8">
-        <v>46099.54242268519</v>
+        <v>46129.586425601854</v>
       </c>
       <c r="E61" s="9" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="F61" s="9" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="G61" s="9" t="s">
-        <v>211</v>
-      </c>
-      <c r="H61" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="H61" s="9"/>
+      <c r="I61" s="9"/>
+      <c r="J61" s="9"/>
+      <c r="K61" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="L61" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="M61" s="9" t="s">
+        <v>0</v>
+      </c>
+      <c r="N61" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="O61" s="9" t="s">
         <v>212</v>
       </c>
-      <c r="I61" s="8">
-        <v>46003</v>
-      </c>
-      <c r="J61" s="8">
-        <v>46009</v>
-      </c>
-      <c r="K61" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="L61" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="M61" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="N61" s="9" t="s">
-        <v>207</v>
-      </c>
-      <c r="O61" s="9" t="s">
-        <v>74</v>
-      </c>
       <c r="P61" s="9" t="s">
-        <v>213</v>
-      </c>
-      <c r="Q61" s="8">
-        <v>46003</v>
-      </c>
-      <c r="R61" s="8">
-        <v>46010</v>
-      </c>
-      <c r="S61" s="10" t="s">
-        <v>31</v>
-      </c>
-      <c r="T61" s="9">
-        <v>1</v>
-      </c>
-      <c r="U61" s="11" t="s">
-        <v>32</v>
-      </c>
+        <v>26</v>
+      </c>
+      <c r="Q61" s="9"/>
+      <c r="R61" s="9"/>
+      <c r="S61" s="9"/>
+      <c r="T61" s="9"/>
+      <c r="U61" s="9"/>
     </row>
     <row r="62" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A62" s="4" t="s">
+        <v>213</v>
+      </c>
+      <c r="B62" s="5">
+        <v>46073.6999484375</v>
+      </c>
+      <c r="C62" s="5">
+        <v>46099.54242106482</v>
+      </c>
+      <c r="D62" s="5">
+        <v>46099.54242268519</v>
+      </c>
+      <c r="E62" s="6" t="s">
         <v>214</v>
-      </c>
-      <c r="B62" s="5">
-        <v>46073.699946249995</v>
-      </c>
-      <c r="C62" s="5">
-        <v>46129.586253912035</v>
-      </c>
-      <c r="D62" s="5">
-        <v>46129.58626813657</v>
-      </c>
-      <c r="E62" s="6" t="s">
-        <v>213</v>
       </c>
       <c r="F62" s="6" t="s">
         <v>26</v>
@@ -5215,10 +5207,10 @@
         <v>216</v>
       </c>
       <c r="I62" s="5">
-        <v>46058</v>
+        <v>46003</v>
       </c>
       <c r="J62" s="5">
-        <v>46064</v>
+        <v>46009</v>
       </c>
       <c r="K62" s="6" t="s">
         <v>26</v>
@@ -5230,19 +5222,19 @@
         <v>26</v>
       </c>
       <c r="N62" s="6" t="s">
-        <v>207</v>
+        <v>211</v>
       </c>
       <c r="O62" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="P62" s="6" t="s">
         <v>217</v>
       </c>
-      <c r="P62" s="6" t="s">
-        <v>218</v>
-      </c>
       <c r="Q62" s="5">
-        <v>46058</v>
+        <v>46003</v>
       </c>
       <c r="R62" s="5">
-        <v>46064</v>
+        <v>46010</v>
       </c>
       <c r="S62" s="10" t="s">
         <v>31</v>
@@ -5256,32 +5248,34 @@
     </row>
     <row r="63" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A63" s="7" t="s">
+        <v>218</v>
+      </c>
+      <c r="B63" s="8">
+        <v>46073.699946249995</v>
+      </c>
+      <c r="C63" s="8">
+        <v>46129.586253912035</v>
+      </c>
+      <c r="D63" s="8">
+        <v>46129.58626813657</v>
+      </c>
+      <c r="E63" s="9" t="s">
+        <v>217</v>
+      </c>
+      <c r="F63" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="G63" s="9" t="s">
         <v>219</v>
       </c>
-      <c r="B63" s="8">
-        <v>46092.494241736116</v>
-      </c>
-      <c r="C63" s="8">
-        <v>46129.58641790509</v>
-      </c>
-      <c r="D63" s="8">
-        <v>46139.54817715278</v>
-      </c>
-      <c r="E63" s="9" t="s">
-        <v>115</v>
-      </c>
-      <c r="F63" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="G63" s="9" t="s">
-        <v>215</v>
-      </c>
       <c r="H63" s="9" t="s">
-        <v>216</v>
-      </c>
-      <c r="I63" s="9"/>
+        <v>220</v>
+      </c>
+      <c r="I63" s="8">
+        <v>46058</v>
+      </c>
       <c r="J63" s="8">
-        <v>46065</v>
+        <v>46064</v>
       </c>
       <c r="K63" s="9" t="s">
         <v>26</v>
@@ -5293,19 +5287,19 @@
         <v>26</v>
       </c>
       <c r="N63" s="9" t="s">
-        <v>207</v>
+        <v>211</v>
       </c>
       <c r="O63" s="9" t="s">
-        <v>213</v>
+        <v>221</v>
       </c>
       <c r="P63" s="9" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="Q63" s="8">
-        <v>46065</v>
+        <v>46058</v>
       </c>
       <c r="R63" s="8">
-        <v>46065</v>
+        <v>46064</v>
       </c>
       <c r="S63" s="10" t="s">
         <v>31</v>
@@ -5319,90 +5313,96 @@
     </row>
     <row r="64" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A64" s="4" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="B64" s="5">
-        <v>46092.49428590278</v>
-      </c>
-      <c r="C64" s="6"/>
+        <v>46092.494241736116</v>
+      </c>
+      <c r="C64" s="5">
+        <v>46129.58641790509</v>
+      </c>
       <c r="D64" s="5">
-        <v>46154.16811805556</v>
+        <v>46139.54817715278</v>
       </c>
       <c r="E64" s="6" t="s">
-        <v>222</v>
+        <v>115</v>
       </c>
       <c r="F64" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G64" s="6" t="s">
-        <v>223</v>
+        <v>219</v>
       </c>
       <c r="H64" s="6" t="s">
+        <v>220</v>
+      </c>
+      <c r="I64" s="6"/>
+      <c r="J64" s="5">
+        <v>46065</v>
+      </c>
+      <c r="K64" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="L64" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="M64" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="N64" s="6" t="s">
+        <v>211</v>
+      </c>
+      <c r="O64" s="6" t="s">
+        <v>217</v>
+      </c>
+      <c r="P64" s="6" t="s">
         <v>224</v>
       </c>
-      <c r="I64" s="5">
-        <v>46154</v>
-      </c>
-      <c r="J64" s="5">
-        <v>46154</v>
-      </c>
-      <c r="K64" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="L64" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="M64" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="N64" s="6" t="s">
-        <v>207</v>
-      </c>
-      <c r="O64" s="6" t="s">
-        <v>225</v>
-      </c>
-      <c r="P64" s="6" t="s">
-        <v>226</v>
-      </c>
       <c r="Q64" s="5">
-        <v>46154</v>
+        <v>46065</v>
       </c>
       <c r="R64" s="5">
-        <v>46154</v>
-      </c>
-      <c r="S64" s="11" t="s">
-        <v>128</v>
+        <v>46065</v>
+      </c>
+      <c r="S64" s="10" t="s">
+        <v>31</v>
       </c>
       <c r="T64" s="6">
-        <v>0</v>
-      </c>
-      <c r="U64" s="10" t="s">
-        <v>58</v>
+        <v>1</v>
+      </c>
+      <c r="U64" s="11" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="65" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A65" s="7" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="B65" s="8">
-        <v>46073.69994662037</v>
+        <v>46092.49428590278</v>
       </c>
       <c r="C65" s="9"/>
       <c r="D65" s="8">
-        <v>46198.821161875</v>
+        <v>46154.16811805556</v>
       </c>
       <c r="E65" s="9" t="s">
+        <v>226</v>
+      </c>
+      <c r="F65" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="G65" s="9" t="s">
+        <v>227</v>
+      </c>
+      <c r="H65" s="9" t="s">
         <v>228</v>
       </c>
-      <c r="F65" s="9" t="s">
-        <v>25</v>
-      </c>
-      <c r="G65" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="H65" s="9"/>
-      <c r="I65" s="9"/>
-      <c r="J65" s="9"/>
+      <c r="I65" s="8">
+        <v>46154</v>
+      </c>
+      <c r="J65" s="8">
+        <v>46154</v>
+      </c>
       <c r="K65" s="9" t="s">
         <v>26</v>
       </c>
@@ -5410,138 +5410,132 @@
         <v>26</v>
       </c>
       <c r="M65" s="9" t="s">
-        <v>0</v>
+        <v>26</v>
       </c>
       <c r="N65" s="9" t="s">
-        <v>26</v>
+        <v>211</v>
       </c>
       <c r="O65" s="9" t="s">
         <v>229</v>
       </c>
       <c r="P65" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="Q65" s="9"/>
-      <c r="R65" s="9"/>
-      <c r="S65" s="9"/>
-      <c r="T65" s="9"/>
-      <c r="U65" s="9"/>
+        <v>230</v>
+      </c>
+      <c r="Q65" s="8">
+        <v>46154</v>
+      </c>
+      <c r="R65" s="8">
+        <v>46154</v>
+      </c>
+      <c r="S65" s="11" t="s">
+        <v>128</v>
+      </c>
+      <c r="T65" s="9">
+        <v>0</v>
+      </c>
+      <c r="U65" s="10" t="s">
+        <v>58</v>
+      </c>
     </row>
     <row r="66" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A66" s="4" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="B66" s="5">
-        <v>46073.69994689815</v>
+        <v>46073.69994662037</v>
       </c>
       <c r="C66" s="6"/>
       <c r="D66" s="5">
-        <v>46199.82444644676</v>
+        <v>46198.821161875</v>
       </c>
       <c r="E66" s="6" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="F66" s="6" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="G66" s="6" t="s">
-        <v>232</v>
-      </c>
-      <c r="H66" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="H66" s="6"/>
+      <c r="I66" s="6"/>
+      <c r="J66" s="6"/>
+      <c r="K66" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="L66" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="M66" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="N66" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="O66" s="6" t="s">
         <v>233</v>
       </c>
-      <c r="I66" s="5">
-        <v>46063</v>
-      </c>
-      <c r="J66" s="5">
-        <v>46064</v>
-      </c>
-      <c r="K66" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="L66" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="M66" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="N66" s="6" t="s">
-        <v>228</v>
-      </c>
-      <c r="O66" s="6" t="s">
-        <v>171</v>
-      </c>
       <c r="P66" s="6" t="s">
-        <v>234</v>
-      </c>
-      <c r="Q66" s="5">
-        <v>46063</v>
-      </c>
-      <c r="R66" s="5">
-        <v>46065</v>
-      </c>
-      <c r="S66" s="10" t="s">
-        <v>31</v>
-      </c>
-      <c r="T66" s="6">
-        <v>0</v>
-      </c>
-      <c r="U66" s="12" t="s">
-        <v>201</v>
-      </c>
+        <v>26</v>
+      </c>
+      <c r="Q66" s="6"/>
+      <c r="R66" s="6"/>
+      <c r="S66" s="6"/>
+      <c r="T66" s="6"/>
+      <c r="U66" s="6"/>
     </row>
     <row r="67" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A67" s="7" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="B67" s="8">
-        <v>46073.69994719907</v>
+        <v>46073.69994689815</v>
       </c>
       <c r="C67" s="9"/>
       <c r="D67" s="8">
-        <v>46198.8211615162</v>
+        <v>46199.82444644676</v>
       </c>
       <c r="E67" s="9" t="s">
+        <v>235</v>
+      </c>
+      <c r="F67" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="G67" s="9" t="s">
         <v>236</v>
       </c>
-      <c r="F67" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="G67" s="9" t="s">
+      <c r="H67" s="9" t="s">
         <v>237</v>
       </c>
-      <c r="H67" s="9" t="s">
+      <c r="I67" s="8">
+        <v>46063</v>
+      </c>
+      <c r="J67" s="8">
+        <v>46064</v>
+      </c>
+      <c r="K67" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="L67" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="M67" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="N67" s="9" t="s">
+        <v>232</v>
+      </c>
+      <c r="O67" s="9" t="s">
+        <v>171</v>
+      </c>
+      <c r="P67" s="9" t="s">
         <v>238</v>
       </c>
-      <c r="I67" s="8">
+      <c r="Q67" s="8">
+        <v>46063</v>
+      </c>
+      <c r="R67" s="8">
         <v>46065</v>
-      </c>
-      <c r="J67" s="8">
-        <v>46066</v>
-      </c>
-      <c r="K67" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="L67" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="M67" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="N67" s="9" t="s">
-        <v>228</v>
-      </c>
-      <c r="O67" s="9" t="s">
-        <v>231</v>
-      </c>
-      <c r="P67" s="9" t="s">
-        <v>239</v>
-      </c>
-      <c r="Q67" s="8">
-        <v>46065</v>
-      </c>
-      <c r="R67" s="8">
-        <v>46066</v>
       </c>
       <c r="S67" s="10" t="s">
         <v>31</v>
@@ -5549,172 +5543,172 @@
       <c r="T67" s="9">
         <v>0</v>
       </c>
-      <c r="U67" s="10" t="s">
-        <v>58</v>
+      <c r="U67" s="12" t="s">
+        <v>201</v>
       </c>
     </row>
     <row r="68" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A68" s="4" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="B68" s="5">
-        <v>46073.69994748842</v>
+        <v>46073.69994719907</v>
       </c>
       <c r="C68" s="6"/>
       <c r="D68" s="5">
-        <v>46077.62916171296</v>
+        <v>46198.8211615162</v>
       </c>
       <c r="E68" s="6" t="s">
+        <v>240</v>
+      </c>
+      <c r="F68" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="G68" s="6" t="s">
+        <v>208</v>
+      </c>
+      <c r="H68" s="6" t="s">
+        <v>209</v>
+      </c>
+      <c r="I68" s="5">
+        <v>46065</v>
+      </c>
+      <c r="J68" s="5">
+        <v>46066</v>
+      </c>
+      <c r="K68" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="L68" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="M68" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="N68" s="6" t="s">
+        <v>232</v>
+      </c>
+      <c r="O68" s="6" t="s">
+        <v>235</v>
+      </c>
+      <c r="P68" s="6" t="s">
         <v>241</v>
       </c>
-      <c r="F68" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="G68" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="H68" s="6"/>
-      <c r="I68" s="6"/>
-      <c r="J68" s="6"/>
-      <c r="K68" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="L68" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="M68" s="6" t="s">
+      <c r="Q68" s="5">
+        <v>46065</v>
+      </c>
+      <c r="R68" s="5">
+        <v>46066</v>
+      </c>
+      <c r="S68" s="10" t="s">
+        <v>31</v>
+      </c>
+      <c r="T68" s="6">
         <v>0</v>
       </c>
-      <c r="N68" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="O68" s="6" t="s">
-        <v>242</v>
-      </c>
-      <c r="P68" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="Q68" s="6"/>
-      <c r="R68" s="6"/>
-      <c r="S68" s="6"/>
-      <c r="T68" s="6"/>
-      <c r="U68" s="6"/>
+      <c r="U68" s="10" t="s">
+        <v>58</v>
+      </c>
     </row>
     <row r="69" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A69" s="7" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="B69" s="8">
-        <v>46073.69994777778</v>
+        <v>46073.69994748842</v>
       </c>
       <c r="C69" s="9"/>
       <c r="D69" s="8">
-        <v>46092.50399041666</v>
+        <v>46077.62916171296</v>
       </c>
       <c r="E69" s="9" t="s">
+        <v>243</v>
+      </c>
+      <c r="F69" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="G69" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="H69" s="9"/>
+      <c r="I69" s="9"/>
+      <c r="J69" s="9"/>
+      <c r="K69" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="L69" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="M69" s="9" t="s">
+        <v>0</v>
+      </c>
+      <c r="N69" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="O69" s="9" t="s">
         <v>244</v>
       </c>
-      <c r="F69" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="G69" s="9" t="s">
-        <v>245</v>
-      </c>
-      <c r="H69" s="9" t="s">
-        <v>246</v>
-      </c>
-      <c r="I69" s="8">
-        <v>46069</v>
-      </c>
-      <c r="J69" s="8">
-        <v>46077</v>
-      </c>
-      <c r="K69" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="L69" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="M69" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="N69" s="9" t="s">
-        <v>241</v>
-      </c>
-      <c r="O69" s="9" t="s">
-        <v>236</v>
-      </c>
       <c r="P69" s="9" t="s">
-        <v>247</v>
-      </c>
-      <c r="Q69" s="8">
-        <v>46069</v>
-      </c>
-      <c r="R69" s="8">
-        <v>46077</v>
-      </c>
-      <c r="S69" s="10" t="s">
-        <v>31</v>
-      </c>
-      <c r="T69" s="9">
-        <v>0</v>
-      </c>
-      <c r="U69" s="10" t="s">
-        <v>58</v>
-      </c>
+        <v>26</v>
+      </c>
+      <c r="Q69" s="9"/>
+      <c r="R69" s="9"/>
+      <c r="S69" s="9"/>
+      <c r="T69" s="9"/>
+      <c r="U69" s="9"/>
     </row>
     <row r="70" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A70" s="4" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
       <c r="B70" s="5">
-        <v>46073.699948113426</v>
+        <v>46073.69994777778</v>
       </c>
       <c r="C70" s="6"/>
       <c r="D70" s="5">
-        <v>46129.58642229167</v>
+        <v>46092.50399041666</v>
       </c>
       <c r="E70" s="6" t="s">
+        <v>246</v>
+      </c>
+      <c r="F70" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="G70" s="6" t="s">
+        <v>247</v>
+      </c>
+      <c r="H70" s="6" t="s">
+        <v>248</v>
+      </c>
+      <c r="I70" s="5">
+        <v>46069</v>
+      </c>
+      <c r="J70" s="5">
+        <v>46077</v>
+      </c>
+      <c r="K70" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="L70" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="M70" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="N70" s="6" t="s">
+        <v>243</v>
+      </c>
+      <c r="O70" s="6" t="s">
+        <v>240</v>
+      </c>
+      <c r="P70" s="6" t="s">
         <v>249</v>
       </c>
-      <c r="F70" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="G70" s="6" t="s">
-        <v>245</v>
-      </c>
-      <c r="H70" s="6" t="s">
-        <v>246</v>
-      </c>
-      <c r="I70" s="5">
-        <v>46078</v>
-      </c>
-      <c r="J70" s="5">
-        <v>46106</v>
-      </c>
-      <c r="K70" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="L70" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="M70" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="N70" s="6" t="s">
-        <v>241</v>
-      </c>
-      <c r="O70" s="6" t="s">
-        <v>250</v>
-      </c>
-      <c r="P70" s="6" t="s">
-        <v>251</v>
-      </c>
       <c r="Q70" s="5">
-        <v>46078</v>
+        <v>46069</v>
       </c>
       <c r="R70" s="5">
-        <v>46106</v>
+        <v>46077</v>
       </c>
       <c r="S70" s="10" t="s">
         <v>31</v>
@@ -5728,56 +5722,56 @@
     </row>
     <row r="71" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A71" s="7" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="B71" s="8">
-        <v>46073.69994846065</v>
+        <v>46073.699948113426</v>
       </c>
       <c r="C71" s="9"/>
       <c r="D71" s="8">
-        <v>46129.5864233912</v>
+        <v>46129.58642229167</v>
       </c>
       <c r="E71" s="9" t="s">
+        <v>251</v>
+      </c>
+      <c r="F71" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="G71" s="9" t="s">
+        <v>247</v>
+      </c>
+      <c r="H71" s="9" t="s">
+        <v>248</v>
+      </c>
+      <c r="I71" s="8">
+        <v>46078</v>
+      </c>
+      <c r="J71" s="8">
+        <v>46106</v>
+      </c>
+      <c r="K71" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="L71" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="M71" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="N71" s="9" t="s">
+        <v>243</v>
+      </c>
+      <c r="O71" s="9" t="s">
+        <v>252</v>
+      </c>
+      <c r="P71" s="9" t="s">
         <v>253</v>
       </c>
-      <c r="F71" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="G71" s="9" t="s">
-        <v>237</v>
-      </c>
-      <c r="H71" s="9" t="s">
-        <v>238</v>
-      </c>
-      <c r="I71" s="8">
-        <v>46107</v>
-      </c>
-      <c r="J71" s="8">
-        <v>46108</v>
-      </c>
-      <c r="K71" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="L71" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="M71" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="N71" s="9" t="s">
-        <v>241</v>
-      </c>
-      <c r="O71" s="9" t="s">
-        <v>254</v>
-      </c>
-      <c r="P71" s="9" t="s">
-        <v>255</v>
-      </c>
       <c r="Q71" s="8">
-        <v>46107</v>
+        <v>46078</v>
       </c>
       <c r="R71" s="8">
-        <v>46108</v>
+        <v>46106</v>
       </c>
       <c r="S71" s="10" t="s">
         <v>31</v>
@@ -5791,27 +5785,33 @@
     </row>
     <row r="72" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A72" s="4" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="B72" s="5">
-        <v>46073.699948865746</v>
+        <v>46073.69994846065</v>
       </c>
       <c r="C72" s="6"/>
       <c r="D72" s="5">
-        <v>46195.604225717594</v>
+        <v>46129.5864233912</v>
       </c>
       <c r="E72" s="6" t="s">
-        <v>228</v>
+        <v>255</v>
       </c>
       <c r="F72" s="6" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G72" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="H72" s="6"/>
-      <c r="I72" s="6"/>
-      <c r="J72" s="6"/>
+        <v>208</v>
+      </c>
+      <c r="H72" s="6" t="s">
+        <v>209</v>
+      </c>
+      <c r="I72" s="5">
+        <v>46107</v>
+      </c>
+      <c r="J72" s="5">
+        <v>46108</v>
+      </c>
       <c r="K72" s="6" t="s">
         <v>26</v>
       </c>
@@ -5819,138 +5819,132 @@
         <v>26</v>
       </c>
       <c r="M72" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="N72" s="6" t="s">
+        <v>243</v>
+      </c>
+      <c r="O72" s="6" t="s">
+        <v>256</v>
+      </c>
+      <c r="P72" s="6" t="s">
+        <v>257</v>
+      </c>
+      <c r="Q72" s="5">
+        <v>46107</v>
+      </c>
+      <c r="R72" s="5">
+        <v>46108</v>
+      </c>
+      <c r="S72" s="10" t="s">
+        <v>31</v>
+      </c>
+      <c r="T72" s="6">
         <v>0</v>
       </c>
-      <c r="N72" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="O72" s="6" t="s">
-        <v>257</v>
-      </c>
-      <c r="P72" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="Q72" s="6"/>
-      <c r="R72" s="6"/>
-      <c r="S72" s="6"/>
-      <c r="T72" s="6"/>
-      <c r="U72" s="6"/>
+      <c r="U72" s="10" t="s">
+        <v>58</v>
+      </c>
     </row>
     <row r="73" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A73" s="7" t="s">
         <v>258</v>
       </c>
       <c r="B73" s="8">
-        <v>46073.69995097222</v>
+        <v>46073.699948865746</v>
       </c>
       <c r="C73" s="9"/>
       <c r="D73" s="8">
-        <v>46199.830143969906</v>
+        <v>46195.604225717594</v>
       </c>
       <c r="E73" s="9" t="s">
+        <v>232</v>
+      </c>
+      <c r="F73" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="G73" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="H73" s="9"/>
+      <c r="I73" s="9"/>
+      <c r="J73" s="9"/>
+      <c r="K73" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="L73" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="M73" s="9" t="s">
+        <v>0</v>
+      </c>
+      <c r="N73" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="O73" s="9" t="s">
         <v>259</v>
       </c>
-      <c r="F73" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="G73" s="9" t="s">
-        <v>232</v>
-      </c>
-      <c r="H73" s="9" t="s">
-        <v>233</v>
-      </c>
-      <c r="I73" s="8">
-        <v>46097</v>
-      </c>
-      <c r="J73" s="8">
-        <v>46098</v>
-      </c>
-      <c r="K73" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="L73" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="M73" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="N73" s="9" t="s">
-        <v>228</v>
-      </c>
-      <c r="O73" s="9" t="s">
-        <v>148</v>
-      </c>
       <c r="P73" s="9" t="s">
-        <v>260</v>
-      </c>
-      <c r="Q73" s="8">
-        <v>46097</v>
-      </c>
-      <c r="R73" s="8">
-        <v>46098</v>
-      </c>
-      <c r="S73" s="10" t="s">
-        <v>31</v>
-      </c>
-      <c r="T73" s="9">
-        <v>0</v>
-      </c>
-      <c r="U73" s="10" t="s">
-        <v>58</v>
-      </c>
+        <v>26</v>
+      </c>
+      <c r="Q73" s="9"/>
+      <c r="R73" s="9"/>
+      <c r="S73" s="9"/>
+      <c r="T73" s="9"/>
+      <c r="U73" s="9"/>
     </row>
     <row r="74" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A74" s="4" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="B74" s="5">
-        <v>46073.69994640046</v>
+        <v>46073.69995097222</v>
       </c>
       <c r="C74" s="6"/>
       <c r="D74" s="5">
-        <v>46121.187778182866</v>
+        <v>46199.830143969906</v>
       </c>
       <c r="E74" s="6" t="s">
-        <v>56</v>
+        <v>261</v>
       </c>
       <c r="F74" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G74" s="6" t="s">
+        <v>236</v>
+      </c>
+      <c r="H74" s="6" t="s">
+        <v>237</v>
+      </c>
+      <c r="I74" s="5">
+        <v>46097</v>
+      </c>
+      <c r="J74" s="5">
+        <v>46098</v>
+      </c>
+      <c r="K74" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="L74" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="M74" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="N74" s="6" t="s">
         <v>232</v>
       </c>
-      <c r="H74" s="6" t="s">
-        <v>233</v>
-      </c>
-      <c r="I74" s="5">
-        <v>46119</v>
-      </c>
-      <c r="J74" s="5">
-        <v>46120</v>
-      </c>
-      <c r="K74" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="L74" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="M74" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="N74" s="6" t="s">
-        <v>228</v>
-      </c>
       <c r="O74" s="6" t="s">
-        <v>139</v>
+        <v>148</v>
       </c>
       <c r="P74" s="6" t="s">
         <v>262</v>
       </c>
       <c r="Q74" s="5">
-        <v>46119</v>
+        <v>46097</v>
       </c>
       <c r="R74" s="5">
-        <v>46120</v>
+        <v>46098</v>
       </c>
       <c r="S74" s="10" t="s">
         <v>31</v>
@@ -5967,53 +5961,53 @@
         <v>263</v>
       </c>
       <c r="B75" s="8">
-        <v>46073.699946782406</v>
+        <v>46073.69994640046</v>
       </c>
       <c r="C75" s="9"/>
       <c r="D75" s="8">
-        <v>46199.82646660879</v>
+        <v>46121.187778182866</v>
       </c>
       <c r="E75" s="9" t="s">
+        <v>56</v>
+      </c>
+      <c r="F75" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="G75" s="9" t="s">
+        <v>236</v>
+      </c>
+      <c r="H75" s="9" t="s">
+        <v>237</v>
+      </c>
+      <c r="I75" s="8">
+        <v>46119</v>
+      </c>
+      <c r="J75" s="8">
+        <v>46120</v>
+      </c>
+      <c r="K75" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="L75" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="M75" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="N75" s="9" t="s">
+        <v>232</v>
+      </c>
+      <c r="O75" s="9" t="s">
+        <v>139</v>
+      </c>
+      <c r="P75" s="9" t="s">
         <v>264</v>
       </c>
-      <c r="F75" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="G75" s="9" t="s">
-        <v>232</v>
-      </c>
-      <c r="H75" s="9" t="s">
-        <v>233</v>
-      </c>
-      <c r="I75" s="8">
-        <v>46132</v>
-      </c>
-      <c r="J75" s="8">
-        <v>46133</v>
-      </c>
-      <c r="K75" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="L75" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="M75" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="N75" s="9" t="s">
-        <v>228</v>
-      </c>
-      <c r="O75" s="9" t="s">
-        <v>130</v>
-      </c>
-      <c r="P75" s="9" t="s">
-        <v>265</v>
-      </c>
       <c r="Q75" s="8">
-        <v>46132</v>
+        <v>46119</v>
       </c>
       <c r="R75" s="8">
-        <v>46133</v>
+        <v>46120</v>
       </c>
       <c r="S75" s="10" t="s">
         <v>31</v>
@@ -6027,126 +6021,124 @@
     </row>
     <row r="76" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A76" s="4" t="s">
+        <v>265</v>
+      </c>
+      <c r="B76" s="5">
+        <v>46073.699946782406</v>
+      </c>
+      <c r="C76" s="6"/>
+      <c r="D76" s="5">
+        <v>46199.82646660879</v>
+      </c>
+      <c r="E76" s="6" t="s">
         <v>266</v>
       </c>
-      <c r="B76" s="5">
-        <v>46073.69994708333</v>
-      </c>
-      <c r="C76" s="5">
-        <v>46195.603957824074</v>
-      </c>
-      <c r="D76" s="5">
-        <v>46195.603959687505</v>
-      </c>
-      <c r="E76" s="6" t="s">
+      <c r="F76" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="G76" s="6" t="s">
+        <v>236</v>
+      </c>
+      <c r="H76" s="6" t="s">
+        <v>237</v>
+      </c>
+      <c r="I76" s="5">
+        <v>46132</v>
+      </c>
+      <c r="J76" s="5">
+        <v>46133</v>
+      </c>
+      <c r="K76" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="L76" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="M76" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="N76" s="6" t="s">
+        <v>232</v>
+      </c>
+      <c r="O76" s="6" t="s">
+        <v>130</v>
+      </c>
+      <c r="P76" s="6" t="s">
         <v>267</v>
       </c>
-      <c r="F76" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="G76" s="6" t="s">
-        <v>232</v>
-      </c>
-      <c r="H76" s="6" t="s">
-        <v>233</v>
-      </c>
-      <c r="I76" s="5">
-        <v>46147</v>
-      </c>
-      <c r="J76" s="5">
-        <v>46148</v>
-      </c>
-      <c r="K76" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="L76" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="M76" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="N76" s="6" t="s">
-        <v>228</v>
-      </c>
-      <c r="O76" s="6" t="s">
-        <v>157</v>
-      </c>
-      <c r="P76" s="6" t="s">
-        <v>268</v>
-      </c>
       <c r="Q76" s="5">
-        <v>46147</v>
+        <v>46132</v>
       </c>
       <c r="R76" s="5">
-        <v>46148</v>
-      </c>
-      <c r="S76" s="11" t="s">
-        <v>128</v>
+        <v>46133</v>
+      </c>
+      <c r="S76" s="10" t="s">
+        <v>31</v>
       </c>
       <c r="T76" s="6">
         <v>0</v>
       </c>
-      <c r="U76" s="12" t="s">
-        <v>201</v>
+      <c r="U76" s="10" t="s">
+        <v>58</v>
       </c>
     </row>
     <row r="77" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A77" s="7" t="s">
+        <v>268</v>
+      </c>
+      <c r="B77" s="8">
+        <v>46073.69994708333</v>
+      </c>
+      <c r="C77" s="8">
+        <v>46195.603957824074</v>
+      </c>
+      <c r="D77" s="8">
+        <v>46195.603959687505</v>
+      </c>
+      <c r="E77" s="9" t="s">
         <v>269</v>
       </c>
-      <c r="B77" s="8">
-        <v>46076.88127923611</v>
-      </c>
-      <c r="C77" s="8">
-        <v>46195.60421921297</v>
-      </c>
-      <c r="D77" s="8">
-        <v>46195.60422127315</v>
-      </c>
-      <c r="E77" s="9" t="s">
+      <c r="F77" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="G77" s="9" t="s">
+        <v>236</v>
+      </c>
+      <c r="H77" s="9" t="s">
+        <v>237</v>
+      </c>
+      <c r="I77" s="8">
+        <v>46147</v>
+      </c>
+      <c r="J77" s="8">
+        <v>46148</v>
+      </c>
+      <c r="K77" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="L77" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="M77" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="N77" s="9" t="s">
+        <v>232</v>
+      </c>
+      <c r="O77" s="9" t="s">
+        <v>157</v>
+      </c>
+      <c r="P77" s="9" t="s">
         <v>270</v>
       </c>
-      <c r="F77" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="G77" s="9" t="s">
-        <v>232</v>
-      </c>
-      <c r="H77" s="9" t="s">
-        <v>233</v>
-      </c>
-      <c r="I77" s="8">
-        <v>46121</v>
-      </c>
-      <c r="J77" s="8">
-        <v>46122</v>
-      </c>
-      <c r="K77" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="L77" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="M77" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="N77" s="9" t="s">
-        <v>228</v>
-      </c>
-      <c r="O77" s="9" t="s">
-        <v>180</v>
-      </c>
-      <c r="P77" s="9" t="s">
-        <v>271</v>
-      </c>
       <c r="Q77" s="8">
-        <v>46121</v>
+        <v>46147</v>
       </c>
       <c r="R77" s="8">
-        <v>46122</v>
-      </c>
-      <c r="S77" s="10" t="s">
-        <v>31</v>
+        <v>46148</v>
+      </c>
+      <c r="S77" s="11" t="s">
+        <v>128</v>
       </c>
       <c r="T77" s="9">
         <v>0</v>
@@ -6157,58 +6149,58 @@
     </row>
     <row r="78" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A78" s="4" t="s">
+        <v>271</v>
+      </c>
+      <c r="B78" s="5">
+        <v>46076.88127923611</v>
+      </c>
+      <c r="C78" s="5">
+        <v>46195.60421921297</v>
+      </c>
+      <c r="D78" s="5">
+        <v>46195.60422127315</v>
+      </c>
+      <c r="E78" s="6" t="s">
         <v>272</v>
       </c>
-      <c r="B78" s="5">
-        <v>46077.57961084491</v>
-      </c>
-      <c r="C78" s="5">
-        <v>46195.60466336805</v>
-      </c>
-      <c r="D78" s="5">
-        <v>46195.60466490741</v>
-      </c>
-      <c r="E78" s="6" t="s">
+      <c r="F78" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="G78" s="6" t="s">
+        <v>236</v>
+      </c>
+      <c r="H78" s="6" t="s">
+        <v>237</v>
+      </c>
+      <c r="I78" s="5">
+        <v>46121</v>
+      </c>
+      <c r="J78" s="5">
+        <v>46122</v>
+      </c>
+      <c r="K78" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="L78" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="M78" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="N78" s="6" t="s">
+        <v>232</v>
+      </c>
+      <c r="O78" s="6" t="s">
+        <v>180</v>
+      </c>
+      <c r="P78" s="6" t="s">
         <v>273</v>
       </c>
-      <c r="F78" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="G78" s="6" t="s">
-        <v>232</v>
-      </c>
-      <c r="H78" s="6" t="s">
-        <v>233</v>
-      </c>
-      <c r="I78" s="5">
-        <v>46104</v>
-      </c>
-      <c r="J78" s="5">
-        <v>46105</v>
-      </c>
-      <c r="K78" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="L78" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="M78" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="N78" s="6" t="s">
-        <v>228</v>
-      </c>
-      <c r="O78" s="6" t="s">
-        <v>195</v>
-      </c>
-      <c r="P78" s="6" t="s">
-        <v>274</v>
-      </c>
       <c r="Q78" s="5">
-        <v>46104</v>
+        <v>46121</v>
       </c>
       <c r="R78" s="5">
-        <v>46105</v>
+        <v>46122</v>
       </c>
       <c r="S78" s="10" t="s">
         <v>31</v>
@@ -6216,62 +6208,64 @@
       <c r="T78" s="6">
         <v>0</v>
       </c>
-      <c r="U78" s="10" t="s">
-        <v>58</v>
+      <c r="U78" s="12" t="s">
+        <v>201</v>
       </c>
     </row>
     <row r="79" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A79" s="7" t="s">
+        <v>274</v>
+      </c>
+      <c r="B79" s="8">
+        <v>46077.57961084491</v>
+      </c>
+      <c r="C79" s="8">
+        <v>46195.60466336805</v>
+      </c>
+      <c r="D79" s="8">
+        <v>46195.60466490741</v>
+      </c>
+      <c r="E79" s="9" t="s">
         <v>275</v>
       </c>
-      <c r="B79" s="8">
-        <v>46077.57965403935</v>
-      </c>
-      <c r="C79" s="9"/>
-      <c r="D79" s="8">
-        <v>46182.692112696765</v>
-      </c>
-      <c r="E79" s="9" t="s">
-        <v>188</v>
-      </c>
       <c r="F79" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G79" s="9" t="s">
+        <v>236</v>
+      </c>
+      <c r="H79" s="9" t="s">
+        <v>237</v>
+      </c>
+      <c r="I79" s="8">
+        <v>46104</v>
+      </c>
+      <c r="J79" s="8">
+        <v>46105</v>
+      </c>
+      <c r="K79" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="L79" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="M79" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="N79" s="9" t="s">
         <v>232</v>
       </c>
-      <c r="H79" s="9" t="s">
-        <v>233</v>
-      </c>
-      <c r="I79" s="8">
-        <v>46098</v>
-      </c>
-      <c r="J79" s="8">
-        <v>46099</v>
-      </c>
-      <c r="K79" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="L79" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="M79" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="N79" s="9" t="s">
-        <v>228</v>
-      </c>
       <c r="O79" s="9" t="s">
-        <v>187</v>
+        <v>195</v>
       </c>
       <c r="P79" s="9" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="Q79" s="8">
-        <v>46098</v>
+        <v>46104</v>
       </c>
       <c r="R79" s="8">
-        <v>46099</v>
+        <v>46105</v>
       </c>
       <c r="S79" s="10" t="s">
         <v>31</v>
@@ -6285,27 +6279,33 @@
     </row>
     <row r="80" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A80" s="4" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="B80" s="5">
-        <v>46073.69994733796</v>
+        <v>46077.57965403935</v>
       </c>
       <c r="C80" s="6"/>
       <c r="D80" s="5">
-        <v>46078.621237141204</v>
+        <v>46182.692112696765</v>
       </c>
       <c r="E80" s="6" t="s">
-        <v>277</v>
+        <v>188</v>
       </c>
       <c r="F80" s="6" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G80" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="H80" s="6"/>
-      <c r="I80" s="6"/>
-      <c r="J80" s="6"/>
+        <v>236</v>
+      </c>
+      <c r="H80" s="6" t="s">
+        <v>237</v>
+      </c>
+      <c r="I80" s="5">
+        <v>46098</v>
+      </c>
+      <c r="J80" s="5">
+        <v>46099</v>
+      </c>
       <c r="K80" s="6" t="s">
         <v>26</v>
       </c>
@@ -6313,141 +6313,135 @@
         <v>26</v>
       </c>
       <c r="M80" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="N80" s="6" t="s">
+        <v>232</v>
+      </c>
+      <c r="O80" s="6" t="s">
+        <v>187</v>
+      </c>
+      <c r="P80" s="6" t="s">
+        <v>276</v>
+      </c>
+      <c r="Q80" s="5">
+        <v>46098</v>
+      </c>
+      <c r="R80" s="5">
+        <v>46099</v>
+      </c>
+      <c r="S80" s="10" t="s">
+        <v>31</v>
+      </c>
+      <c r="T80" s="6">
         <v>0</v>
       </c>
-      <c r="N80" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="O80" s="6" t="s">
-        <v>278</v>
-      </c>
-      <c r="P80" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="Q80" s="6"/>
-      <c r="R80" s="6"/>
-      <c r="S80" s="6"/>
-      <c r="T80" s="6"/>
-      <c r="U80" s="6"/>
+      <c r="U80" s="10" t="s">
+        <v>58</v>
+      </c>
     </row>
     <row r="81" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A81" s="7" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="B81" s="8">
-        <v>46073.69994759259</v>
+        <v>46073.69994733796</v>
       </c>
       <c r="C81" s="9"/>
       <c r="D81" s="8">
-        <v>46128.16821587963</v>
+        <v>46078.621237141204</v>
       </c>
       <c r="E81" s="9" t="s">
+        <v>279</v>
+      </c>
+      <c r="F81" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="G81" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="H81" s="9"/>
+      <c r="I81" s="9"/>
+      <c r="J81" s="9"/>
+      <c r="K81" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="L81" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="M81" s="9" t="s">
+        <v>0</v>
+      </c>
+      <c r="N81" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="O81" s="9" t="s">
         <v>280</v>
       </c>
-      <c r="F81" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="G81" s="9" t="s">
-        <v>281</v>
-      </c>
-      <c r="H81" s="9" t="s">
-        <v>281</v>
-      </c>
-      <c r="I81" s="8">
-        <v>46111</v>
-      </c>
-      <c r="J81" s="8">
-        <v>46128</v>
-      </c>
-      <c r="K81" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="L81" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="M81" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="N81" s="9" t="s">
-        <v>277</v>
-      </c>
-      <c r="O81" s="9" t="s">
-        <v>253</v>
-      </c>
       <c r="P81" s="9" t="s">
-        <v>282</v>
-      </c>
-      <c r="Q81" s="8">
-        <v>46111</v>
-      </c>
-      <c r="R81" s="8">
-        <v>46119</v>
-      </c>
-      <c r="S81" s="10" t="s">
-        <v>31</v>
-      </c>
-      <c r="T81" s="9">
-        <v>0</v>
-      </c>
-      <c r="U81" s="10" t="s">
-        <v>58</v>
-      </c>
+        <v>26</v>
+      </c>
+      <c r="Q81" s="9"/>
+      <c r="R81" s="9"/>
+      <c r="S81" s="9"/>
+      <c r="T81" s="9"/>
+      <c r="U81" s="9"/>
     </row>
     <row r="82" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A82" s="4" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="B82" s="5">
-        <v>46073.69994784722</v>
+        <v>46073.69994759259</v>
       </c>
       <c r="C82" s="6"/>
       <c r="D82" s="5">
-        <v>46198.59349042824</v>
+        <v>46128.16821587963</v>
       </c>
       <c r="E82" s="6" t="s">
+        <v>282</v>
+      </c>
+      <c r="F82" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="G82" s="6" t="s">
+        <v>283</v>
+      </c>
+      <c r="H82" s="6" t="s">
+        <v>283</v>
+      </c>
+      <c r="I82" s="5">
+        <v>46111</v>
+      </c>
+      <c r="J82" s="5">
+        <v>46128</v>
+      </c>
+      <c r="K82" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="L82" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="M82" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="N82" s="6" t="s">
+        <v>279</v>
+      </c>
+      <c r="O82" s="6" t="s">
+        <v>255</v>
+      </c>
+      <c r="P82" s="6" t="s">
         <v>284</v>
       </c>
-      <c r="F82" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="G82" s="6" t="s">
-        <v>281</v>
-      </c>
-      <c r="H82" s="6" t="s">
-        <v>281</v>
-      </c>
-      <c r="I82" s="5">
-        <v>46149</v>
-      </c>
-      <c r="J82" s="5">
-        <v>46150</v>
-      </c>
-      <c r="K82" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="L82" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="M82" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="N82" s="6" t="s">
-        <v>277</v>
-      </c>
-      <c r="O82" s="6" t="s">
-        <v>285</v>
-      </c>
-      <c r="P82" s="6" t="s">
-        <v>286</v>
-      </c>
       <c r="Q82" s="5">
-        <v>46149</v>
+        <v>46111</v>
       </c>
       <c r="R82" s="5">
-        <v>46150</v>
-      </c>
-      <c r="S82" s="11" t="s">
-        <v>128</v>
+        <v>46119</v>
+      </c>
+      <c r="S82" s="10" t="s">
+        <v>31</v>
       </c>
       <c r="T82" s="6">
         <v>0</v>
@@ -6458,59 +6452,59 @@
     </row>
     <row r="83" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A83" s="7" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
       <c r="B83" s="8">
-        <v>46073.69994813658</v>
+        <v>46073.69994784722</v>
       </c>
       <c r="C83" s="9"/>
       <c r="D83" s="8">
-        <v>46198.592367060184</v>
+        <v>46198.59349042824</v>
       </c>
       <c r="E83" s="9" t="s">
+        <v>286</v>
+      </c>
+      <c r="F83" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="G83" s="9" t="s">
+        <v>283</v>
+      </c>
+      <c r="H83" s="9" t="s">
+        <v>283</v>
+      </c>
+      <c r="I83" s="8">
+        <v>46149</v>
+      </c>
+      <c r="J83" s="8">
+        <v>46150</v>
+      </c>
+      <c r="K83" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="L83" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="M83" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="N83" s="9" t="s">
+        <v>279</v>
+      </c>
+      <c r="O83" s="9" t="s">
+        <v>287</v>
+      </c>
+      <c r="P83" s="9" t="s">
         <v>288</v>
       </c>
-      <c r="F83" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="G83" s="9" t="s">
-        <v>281</v>
-      </c>
-      <c r="H83" s="9" t="s">
-        <v>281</v>
-      </c>
-      <c r="I83" s="8">
-        <v>46134</v>
-      </c>
-      <c r="J83" s="8">
-        <v>46135</v>
-      </c>
-      <c r="K83" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="L83" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="M83" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="N83" s="9" t="s">
-        <v>277</v>
-      </c>
-      <c r="O83" s="9" t="s">
-        <v>289</v>
-      </c>
-      <c r="P83" s="9" t="s">
-        <v>286</v>
-      </c>
       <c r="Q83" s="8">
-        <v>46134</v>
+        <v>46149</v>
       </c>
       <c r="R83" s="8">
-        <v>46135</v>
-      </c>
-      <c r="S83" s="10" t="s">
-        <v>31</v>
+        <v>46150</v>
+      </c>
+      <c r="S83" s="11" t="s">
+        <v>128</v>
       </c>
       <c r="T83" s="9">
         <v>0</v>
@@ -6521,62 +6515,62 @@
     </row>
     <row r="84" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A84" s="4" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="B84" s="5">
-        <v>46073.699948368056</v>
+        <v>46073.69994813658</v>
       </c>
       <c r="C84" s="6"/>
       <c r="D84" s="5">
-        <v>46198.59272494213</v>
+        <v>46198.592367060184</v>
       </c>
       <c r="E84" s="6" t="s">
+        <v>290</v>
+      </c>
+      <c r="F84" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="G84" s="6" t="s">
+        <v>283</v>
+      </c>
+      <c r="H84" s="6" t="s">
+        <v>283</v>
+      </c>
+      <c r="I84" s="5">
+        <v>46134</v>
+      </c>
+      <c r="J84" s="5">
+        <v>46135</v>
+      </c>
+      <c r="K84" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="L84" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="M84" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="N84" s="6" t="s">
+        <v>279</v>
+      </c>
+      <c r="O84" s="6" t="s">
         <v>291</v>
       </c>
-      <c r="F84" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="G84" s="6" t="s">
-        <v>281</v>
-      </c>
-      <c r="H84" s="6" t="s">
-        <v>281</v>
-      </c>
-      <c r="I84" s="5">
-        <v>46136</v>
-      </c>
-      <c r="J84" s="5">
-        <v>46139</v>
-      </c>
-      <c r="K84" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="L84" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="M84" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="N84" s="6" t="s">
-        <v>277</v>
-      </c>
-      <c r="O84" s="6" t="s">
-        <v>292</v>
-      </c>
       <c r="P84" s="6" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="Q84" s="5">
-        <v>46136</v>
+        <v>46134</v>
       </c>
       <c r="R84" s="5">
-        <v>46139</v>
-      </c>
-      <c r="S84" s="12" t="s">
-        <v>293</v>
+        <v>46135</v>
+      </c>
+      <c r="S84" s="10" t="s">
+        <v>31</v>
       </c>
       <c r="T84" s="6">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="U84" s="10" t="s">
         <v>58</v>
@@ -6584,62 +6578,62 @@
     </row>
     <row r="85" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A85" s="7" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="B85" s="8">
-        <v>46076.88137268518</v>
+        <v>46073.699948368056</v>
       </c>
       <c r="C85" s="9"/>
       <c r="D85" s="8">
-        <v>46195.60422616898</v>
+        <v>46198.59272494213</v>
       </c>
       <c r="E85" s="9" t="s">
+        <v>293</v>
+      </c>
+      <c r="F85" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="G85" s="9" t="s">
+        <v>283</v>
+      </c>
+      <c r="H85" s="9" t="s">
+        <v>283</v>
+      </c>
+      <c r="I85" s="8">
+        <v>46136</v>
+      </c>
+      <c r="J85" s="8">
+        <v>46139</v>
+      </c>
+      <c r="K85" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="L85" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="M85" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="N85" s="9" t="s">
+        <v>279</v>
+      </c>
+      <c r="O85" s="9" t="s">
+        <v>294</v>
+      </c>
+      <c r="P85" s="9" t="s">
+        <v>288</v>
+      </c>
+      <c r="Q85" s="8">
+        <v>46136</v>
+      </c>
+      <c r="R85" s="8">
+        <v>46139</v>
+      </c>
+      <c r="S85" s="12" t="s">
         <v>295</v>
       </c>
-      <c r="F85" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="G85" s="9" t="s">
-        <v>281</v>
-      </c>
-      <c r="H85" s="9" t="s">
-        <v>281</v>
-      </c>
-      <c r="I85" s="8">
-        <v>46129</v>
-      </c>
-      <c r="J85" s="8">
-        <v>46132</v>
-      </c>
-      <c r="K85" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="L85" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="M85" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="N85" s="9" t="s">
-        <v>277</v>
-      </c>
-      <c r="O85" s="9" t="s">
-        <v>296</v>
-      </c>
-      <c r="P85" s="9" t="s">
-        <v>297</v>
-      </c>
-      <c r="Q85" s="8">
-        <v>46129</v>
-      </c>
-      <c r="R85" s="8">
-        <v>46132</v>
-      </c>
-      <c r="S85" s="10" t="s">
-        <v>31</v>
-      </c>
       <c r="T85" s="9">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="U85" s="10" t="s">
         <v>58</v>
@@ -6647,32 +6641,32 @@
     </row>
     <row r="86" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A86" s="4" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
       <c r="B86" s="5">
-        <v>46073.69994864584</v>
+        <v>46076.88137268518</v>
       </c>
       <c r="C86" s="6"/>
       <c r="D86" s="5">
-        <v>46153.16811694445</v>
+        <v>46195.60422616898</v>
       </c>
       <c r="E86" s="6" t="s">
-        <v>225</v>
+        <v>297</v>
       </c>
       <c r="F86" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G86" s="6" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="H86" s="6" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="I86" s="5">
-        <v>46153</v>
+        <v>46129</v>
       </c>
       <c r="J86" s="5">
-        <v>46153</v>
+        <v>46132</v>
       </c>
       <c r="K86" s="6" t="s">
         <v>26</v>
@@ -6684,22 +6678,22 @@
         <v>26</v>
       </c>
       <c r="N86" s="6" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="O86" s="6" t="s">
+        <v>298</v>
+      </c>
+      <c r="P86" s="6" t="s">
         <v>299</v>
       </c>
-      <c r="P86" s="6" t="s">
-        <v>300</v>
-      </c>
       <c r="Q86" s="5">
-        <v>46153</v>
+        <v>46129</v>
       </c>
       <c r="R86" s="5">
-        <v>46153</v>
-      </c>
-      <c r="S86" s="11" t="s">
-        <v>128</v>
+        <v>46132</v>
+      </c>
+      <c r="S86" s="10" t="s">
+        <v>31</v>
       </c>
       <c r="T86" s="6">
         <v>0</v>
@@ -6710,56 +6704,56 @@
     </row>
     <row r="87" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A87" s="7" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="B87" s="8">
-        <v>46073.699948912035</v>
+        <v>46073.69994864584</v>
       </c>
       <c r="C87" s="9"/>
       <c r="D87" s="8">
-        <v>46154.16785564815</v>
+        <v>46153.16811694445</v>
       </c>
       <c r="E87" s="9" t="s">
+        <v>229</v>
+      </c>
+      <c r="F87" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="G87" s="9" t="s">
+        <v>283</v>
+      </c>
+      <c r="H87" s="9" t="s">
+        <v>283</v>
+      </c>
+      <c r="I87" s="8">
+        <v>46153</v>
+      </c>
+      <c r="J87" s="8">
+        <v>46153</v>
+      </c>
+      <c r="K87" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="L87" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="M87" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="N87" s="9" t="s">
+        <v>279</v>
+      </c>
+      <c r="O87" s="9" t="s">
+        <v>301</v>
+      </c>
+      <c r="P87" s="9" t="s">
         <v>302</v>
       </c>
-      <c r="F87" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="G87" s="9" t="s">
-        <v>281</v>
-      </c>
-      <c r="H87" s="9" t="s">
-        <v>281</v>
-      </c>
-      <c r="I87" s="8">
-        <v>46154</v>
-      </c>
-      <c r="J87" s="8">
-        <v>46154</v>
-      </c>
-      <c r="K87" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="L87" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="M87" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="N87" s="9" t="s">
-        <v>277</v>
-      </c>
-      <c r="O87" s="9" t="s">
-        <v>222</v>
-      </c>
-      <c r="P87" s="9" t="s">
-        <v>303</v>
-      </c>
       <c r="Q87" s="8">
-        <v>46154</v>
+        <v>46153</v>
       </c>
       <c r="R87" s="8">
-        <v>46154</v>
+        <v>46153</v>
       </c>
       <c r="S87" s="11" t="s">
         <v>128</v>
@@ -6773,142 +6767,142 @@
     </row>
     <row r="88" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A88" s="4" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="B88" s="5">
-        <v>46073.69994572917</v>
+        <v>46073.699948912035</v>
       </c>
       <c r="C88" s="6"/>
       <c r="D88" s="5">
-        <v>46077.638347245374</v>
+        <v>46154.16785564815</v>
       </c>
       <c r="E88" s="6" t="s">
+        <v>304</v>
+      </c>
+      <c r="F88" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="G88" s="6" t="s">
+        <v>283</v>
+      </c>
+      <c r="H88" s="6" t="s">
+        <v>283</v>
+      </c>
+      <c r="I88" s="5">
+        <v>46154</v>
+      </c>
+      <c r="J88" s="5">
+        <v>46154</v>
+      </c>
+      <c r="K88" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="L88" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="M88" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="N88" s="6" t="s">
+        <v>279</v>
+      </c>
+      <c r="O88" s="6" t="s">
+        <v>226</v>
+      </c>
+      <c r="P88" s="6" t="s">
         <v>305</v>
       </c>
-      <c r="F88" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="G88" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="H88" s="6"/>
-      <c r="I88" s="6"/>
-      <c r="J88" s="6"/>
-      <c r="K88" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="L88" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="M88" s="6" t="s">
+      <c r="Q88" s="5">
+        <v>46154</v>
+      </c>
+      <c r="R88" s="5">
+        <v>46154</v>
+      </c>
+      <c r="S88" s="11" t="s">
+        <v>128</v>
+      </c>
+      <c r="T88" s="6">
         <v>0</v>
       </c>
-      <c r="N88" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="O88" s="6" t="s">
-        <v>306</v>
-      </c>
-      <c r="P88" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="Q88" s="6"/>
-      <c r="R88" s="6"/>
-      <c r="S88" s="6"/>
-      <c r="T88" s="6"/>
-      <c r="U88" s="6"/>
+      <c r="U88" s="10" t="s">
+        <v>58</v>
+      </c>
     </row>
     <row r="89" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A89" s="7" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="B89" s="8">
-        <v>46073.699946099536</v>
+        <v>46073.69994572917</v>
       </c>
       <c r="C89" s="9"/>
       <c r="D89" s="8">
-        <v>46155.16794435185</v>
+        <v>46077.638347245374</v>
       </c>
       <c r="E89" s="9" t="s">
+        <v>307</v>
+      </c>
+      <c r="F89" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="G89" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="H89" s="9"/>
+      <c r="I89" s="9"/>
+      <c r="J89" s="9"/>
+      <c r="K89" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="L89" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="M89" s="9" t="s">
+        <v>0</v>
+      </c>
+      <c r="N89" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="O89" s="9" t="s">
         <v>308</v>
       </c>
-      <c r="F89" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="G89" s="9" t="s">
-        <v>35</v>
-      </c>
-      <c r="H89" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="I89" s="8">
-        <v>46155</v>
-      </c>
-      <c r="J89" s="8">
-        <v>46155</v>
-      </c>
-      <c r="K89" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="L89" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="M89" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="N89" s="9" t="s">
-        <v>305</v>
-      </c>
-      <c r="O89" s="9" t="s">
-        <v>302</v>
-      </c>
       <c r="P89" s="9" t="s">
-        <v>309</v>
-      </c>
-      <c r="Q89" s="8">
-        <v>46155</v>
-      </c>
-      <c r="R89" s="8">
-        <v>46155</v>
-      </c>
-      <c r="S89" s="11" t="s">
-        <v>128</v>
-      </c>
-      <c r="T89" s="9">
-        <v>0</v>
-      </c>
-      <c r="U89" s="10" t="s">
-        <v>58</v>
-      </c>
+        <v>26</v>
+      </c>
+      <c r="Q89" s="9"/>
+      <c r="R89" s="9"/>
+      <c r="S89" s="9"/>
+      <c r="T89" s="9"/>
+      <c r="U89" s="9"/>
     </row>
     <row r="90" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A90" s="4" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="B90" s="5">
-        <v>46073.69994638889</v>
+        <v>46073.699946099536</v>
       </c>
       <c r="C90" s="6"/>
       <c r="D90" s="5">
-        <v>46195.604670092594</v>
+        <v>46155.16794435185</v>
       </c>
       <c r="E90" s="6" t="s">
-        <v>274</v>
+        <v>310</v>
       </c>
       <c r="F90" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G90" s="6" t="s">
-        <v>281</v>
+        <v>35</v>
       </c>
       <c r="H90" s="6" t="s">
-        <v>281</v>
+        <v>36</v>
       </c>
       <c r="I90" s="5">
-        <v>46156</v>
+        <v>46155</v>
       </c>
       <c r="J90" s="5">
-        <v>46160</v>
+        <v>46155</v>
       </c>
       <c r="K90" s="6" t="s">
         <v>26</v>
@@ -6920,19 +6914,19 @@
         <v>26</v>
       </c>
       <c r="N90" s="6" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="O90" s="6" t="s">
+        <v>304</v>
+      </c>
+      <c r="P90" s="6" t="s">
         <v>311</v>
       </c>
-      <c r="P90" s="6" t="s">
-        <v>312</v>
-      </c>
       <c r="Q90" s="5">
-        <v>46156</v>
+        <v>46155</v>
       </c>
       <c r="R90" s="5">
-        <v>46160</v>
+        <v>46155</v>
       </c>
       <c r="S90" s="11" t="s">
         <v>128</v>
@@ -6946,56 +6940,56 @@
     </row>
     <row r="91" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A91" s="7" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="B91" s="8">
-        <v>46073.69994668981</v>
+        <v>46073.69994638889</v>
       </c>
       <c r="C91" s="9"/>
       <c r="D91" s="8">
-        <v>46161.25032122685</v>
+        <v>46195.604670092594</v>
       </c>
       <c r="E91" s="9" t="s">
+        <v>276</v>
+      </c>
+      <c r="F91" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="G91" s="9" t="s">
+        <v>283</v>
+      </c>
+      <c r="H91" s="9" t="s">
+        <v>283</v>
+      </c>
+      <c r="I91" s="8">
+        <v>46156</v>
+      </c>
+      <c r="J91" s="8">
+        <v>46160</v>
+      </c>
+      <c r="K91" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="L91" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="M91" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="N91" s="9" t="s">
+        <v>307</v>
+      </c>
+      <c r="O91" s="9" t="s">
+        <v>313</v>
+      </c>
+      <c r="P91" s="9" t="s">
         <v>314</v>
       </c>
-      <c r="F91" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="G91" s="9" t="s">
-        <v>245</v>
-      </c>
-      <c r="H91" s="9" t="s">
-        <v>246</v>
-      </c>
-      <c r="I91" s="8">
-        <v>46161</v>
-      </c>
-      <c r="J91" s="8">
-        <v>46161</v>
-      </c>
-      <c r="K91" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="L91" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="M91" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="N91" s="9" t="s">
-        <v>305</v>
-      </c>
-      <c r="O91" s="9" t="s">
-        <v>274</v>
-      </c>
-      <c r="P91" s="9" t="s">
-        <v>315</v>
-      </c>
       <c r="Q91" s="8">
-        <v>46161</v>
+        <v>46156</v>
       </c>
       <c r="R91" s="8">
-        <v>46161</v>
+        <v>46160</v>
       </c>
       <c r="S91" s="11" t="s">
         <v>128</v>
@@ -7009,56 +7003,56 @@
     </row>
     <row r="92" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A92" s="4" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="B92" s="5">
-        <v>46073.69994695602</v>
+        <v>46073.69994668981</v>
       </c>
       <c r="C92" s="6"/>
       <c r="D92" s="5">
-        <v>46162.25040996527</v>
+        <v>46161.25032122685</v>
       </c>
       <c r="E92" s="6" t="s">
+        <v>316</v>
+      </c>
+      <c r="F92" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="G92" s="6" t="s">
+        <v>247</v>
+      </c>
+      <c r="H92" s="6" t="s">
+        <v>248</v>
+      </c>
+      <c r="I92" s="5">
+        <v>46161</v>
+      </c>
+      <c r="J92" s="5">
+        <v>46161</v>
+      </c>
+      <c r="K92" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="L92" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="M92" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="N92" s="6" t="s">
+        <v>307</v>
+      </c>
+      <c r="O92" s="6" t="s">
+        <v>276</v>
+      </c>
+      <c r="P92" s="6" t="s">
         <v>317</v>
       </c>
-      <c r="F92" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="G92" s="6" t="s">
-        <v>245</v>
-      </c>
-      <c r="H92" s="6" t="s">
-        <v>246</v>
-      </c>
-      <c r="I92" s="5">
-        <v>46162</v>
-      </c>
-      <c r="J92" s="5">
-        <v>46162</v>
-      </c>
-      <c r="K92" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="L92" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="M92" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="N92" s="6" t="s">
-        <v>305</v>
-      </c>
-      <c r="O92" s="6" t="s">
-        <v>314</v>
-      </c>
-      <c r="P92" s="6" t="s">
-        <v>318</v>
-      </c>
       <c r="Q92" s="5">
-        <v>46162</v>
+        <v>46161</v>
       </c>
       <c r="R92" s="5">
-        <v>46162</v>
+        <v>46161</v>
       </c>
       <c r="S92" s="11" t="s">
         <v>128</v>
@@ -7072,136 +7066,136 @@
     </row>
     <row r="93" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A93" s="7" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="B93" s="8">
-        <v>46073.699947245375</v>
+        <v>46073.69994695602</v>
       </c>
       <c r="C93" s="9"/>
       <c r="D93" s="8">
-        <v>46077.6387968287</v>
+        <v>46162.25040996527</v>
       </c>
       <c r="E93" s="9" t="s">
+        <v>319</v>
+      </c>
+      <c r="F93" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="G93" s="9" t="s">
+        <v>247</v>
+      </c>
+      <c r="H93" s="9" t="s">
+        <v>248</v>
+      </c>
+      <c r="I93" s="8">
+        <v>46162</v>
+      </c>
+      <c r="J93" s="8">
+        <v>46162</v>
+      </c>
+      <c r="K93" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="L93" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="M93" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="N93" s="9" t="s">
+        <v>307</v>
+      </c>
+      <c r="O93" s="9" t="s">
+        <v>316</v>
+      </c>
+      <c r="P93" s="9" t="s">
         <v>320</v>
       </c>
-      <c r="F93" s="9" t="s">
-        <v>25</v>
-      </c>
-      <c r="G93" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="H93" s="9"/>
-      <c r="I93" s="9"/>
-      <c r="J93" s="9"/>
-      <c r="K93" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="L93" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="M93" s="9" t="s">
+      <c r="Q93" s="8">
+        <v>46162</v>
+      </c>
+      <c r="R93" s="8">
+        <v>46162</v>
+      </c>
+      <c r="S93" s="11" t="s">
+        <v>128</v>
+      </c>
+      <c r="T93" s="9">
         <v>0</v>
       </c>
-      <c r="N93" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="O93" s="9" t="s">
-        <v>321</v>
-      </c>
-      <c r="P93" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="Q93" s="9"/>
-      <c r="R93" s="9"/>
-      <c r="S93" s="9"/>
-      <c r="T93" s="9"/>
-      <c r="U93" s="9"/>
+      <c r="U93" s="10" t="s">
+        <v>58</v>
+      </c>
     </row>
     <row r="94" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A94" s="4" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="B94" s="5">
-        <v>46073.699947500005</v>
+        <v>46073.699947245375</v>
       </c>
       <c r="C94" s="6"/>
       <c r="D94" s="5">
-        <v>46174.16833755787</v>
+        <v>46077.6387968287</v>
       </c>
       <c r="E94" s="6" t="s">
+        <v>322</v>
+      </c>
+      <c r="F94" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="G94" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="H94" s="6"/>
+      <c r="I94" s="6"/>
+      <c r="J94" s="6"/>
+      <c r="K94" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="L94" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="M94" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="N94" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="O94" s="6" t="s">
         <v>323</v>
       </c>
-      <c r="F94" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="G94" s="6" t="s">
-        <v>324</v>
-      </c>
-      <c r="H94" s="6" t="s">
-        <v>325</v>
-      </c>
-      <c r="I94" s="5">
-        <v>46164</v>
-      </c>
-      <c r="J94" s="5">
-        <v>46174</v>
-      </c>
-      <c r="K94" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="L94" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="M94" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="N94" s="6" t="s">
-        <v>320</v>
-      </c>
-      <c r="O94" s="6" t="s">
-        <v>317</v>
-      </c>
       <c r="P94" s="6" t="s">
-        <v>320</v>
-      </c>
-      <c r="Q94" s="5">
-        <v>46164</v>
-      </c>
-      <c r="R94" s="5">
-        <v>46174</v>
-      </c>
-      <c r="S94" s="11" t="s">
-        <v>128</v>
-      </c>
-      <c r="T94" s="6">
-        <v>0</v>
-      </c>
-      <c r="U94" s="10" t="s">
-        <v>58</v>
-      </c>
+        <v>26</v>
+      </c>
+      <c r="Q94" s="6"/>
+      <c r="R94" s="6"/>
+      <c r="S94" s="6"/>
+      <c r="T94" s="6"/>
+      <c r="U94" s="6"/>
     </row>
     <row r="95" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A95" s="7" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="B95" s="8">
-        <v>46073.699947789355</v>
+        <v>46073.699947500005</v>
       </c>
       <c r="C95" s="9"/>
       <c r="D95" s="8">
-        <v>46174.168340185184</v>
+        <v>46174.16833755787</v>
       </c>
       <c r="E95" s="9" t="s">
+        <v>325</v>
+      </c>
+      <c r="F95" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="G95" s="9" t="s">
+        <v>326</v>
+      </c>
+      <c r="H95" s="9" t="s">
         <v>327</v>
-      </c>
-      <c r="F95" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="G95" s="9" t="s">
-        <v>324</v>
-      </c>
-      <c r="H95" s="9" t="s">
-        <v>325</v>
       </c>
       <c r="I95" s="8">
         <v>46164</v>
@@ -7219,13 +7213,13 @@
         <v>26</v>
       </c>
       <c r="N95" s="9" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="O95" s="9" t="s">
-        <v>328</v>
+        <v>319</v>
       </c>
       <c r="P95" s="9" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="Q95" s="8">
         <v>46164</v>
@@ -7245,47 +7239,57 @@
     </row>
     <row r="96" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A96" s="4" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="B96" s="5">
-        <v>46092.48971385417</v>
+        <v>46073.699947789355</v>
       </c>
       <c r="C96" s="6"/>
       <c r="D96" s="5">
-        <v>46092.497058946756</v>
+        <v>46174.168340185184</v>
       </c>
       <c r="E96" s="6" t="s">
+        <v>329</v>
+      </c>
+      <c r="F96" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="G96" s="6" t="s">
+        <v>326</v>
+      </c>
+      <c r="H96" s="6" t="s">
+        <v>327</v>
+      </c>
+      <c r="I96" s="5">
+        <v>46164</v>
+      </c>
+      <c r="J96" s="5">
+        <v>46174</v>
+      </c>
+      <c r="K96" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="L96" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="M96" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="N96" s="6" t="s">
+        <v>322</v>
+      </c>
+      <c r="O96" s="6" t="s">
         <v>330</v>
       </c>
-      <c r="F96" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="G96" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="H96" s="6"/>
-      <c r="I96" s="6"/>
-      <c r="J96" s="6"/>
-      <c r="K96" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="L96" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="M96" s="6" t="s">
-        <v>0</v>
-      </c>
-      <c r="N96" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="O96" s="6" t="s">
-        <v>331</v>
-      </c>
       <c r="P96" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="Q96" s="6"/>
-      <c r="R96" s="6"/>
+        <v>322</v>
+      </c>
+      <c r="Q96" s="5">
+        <v>46164</v>
+      </c>
+      <c r="R96" s="5">
+        <v>46174</v>
+      </c>
       <c r="S96" s="11" t="s">
         <v>128</v>
       </c>
@@ -7298,57 +7302,47 @@
     </row>
     <row r="97" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A97" s="7" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="B97" s="8">
-        <v>46092.49161491898</v>
+        <v>46092.48971385417</v>
       </c>
       <c r="C97" s="9"/>
       <c r="D97" s="8">
-        <v>46171.168742951384</v>
+        <v>46092.497058946756</v>
       </c>
       <c r="E97" s="9" t="s">
+        <v>332</v>
+      </c>
+      <c r="F97" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="G97" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="H97" s="9"/>
+      <c r="I97" s="9"/>
+      <c r="J97" s="9"/>
+      <c r="K97" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="L97" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="M97" s="9" t="s">
+        <v>0</v>
+      </c>
+      <c r="N97" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="O97" s="9" t="s">
         <v>333</v>
       </c>
-      <c r="F97" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="G97" s="9" t="s">
-        <v>49</v>
-      </c>
-      <c r="H97" s="9" t="s">
-        <v>50</v>
-      </c>
-      <c r="I97" s="8">
-        <v>46164</v>
-      </c>
-      <c r="J97" s="8">
-        <v>46171</v>
-      </c>
-      <c r="K97" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="L97" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="M97" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="N97" s="9" t="s">
-        <v>330</v>
-      </c>
-      <c r="O97" s="9" t="s">
-        <v>317</v>
-      </c>
       <c r="P97" s="9" t="s">
-        <v>334</v>
-      </c>
-      <c r="Q97" s="8">
-        <v>46164</v>
-      </c>
-      <c r="R97" s="8">
-        <v>46171</v>
-      </c>
+        <v>26</v>
+      </c>
+      <c r="Q97" s="9"/>
+      <c r="R97" s="9"/>
       <c r="S97" s="11" t="s">
         <v>128</v>
       </c>
@@ -7361,17 +7355,17 @@
     </row>
     <row r="98" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A98" s="4" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="B98" s="5">
-        <v>46092.491661747685</v>
+        <v>46092.49161491898</v>
       </c>
       <c r="C98" s="6"/>
       <c r="D98" s="5">
-        <v>46181.16820616898</v>
+        <v>46171.168742951384</v>
       </c>
       <c r="E98" s="6" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="F98" s="6" t="s">
         <v>26</v>
@@ -7383,10 +7377,10 @@
         <v>50</v>
       </c>
       <c r="I98" s="5">
-        <v>46174</v>
+        <v>46164</v>
       </c>
       <c r="J98" s="5">
-        <v>46181</v>
+        <v>46171</v>
       </c>
       <c r="K98" s="6" t="s">
         <v>26</v>
@@ -7398,19 +7392,19 @@
         <v>26</v>
       </c>
       <c r="N98" s="6" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="O98" s="6" t="s">
-        <v>333</v>
+        <v>319</v>
       </c>
       <c r="P98" s="6" t="s">
-        <v>330</v>
+        <v>336</v>
       </c>
       <c r="Q98" s="5">
-        <v>46174</v>
+        <v>46164</v>
       </c>
       <c r="R98" s="5">
-        <v>46181</v>
+        <v>46171</v>
       </c>
       <c r="S98" s="11" t="s">
         <v>128</v>
@@ -7419,6 +7413,69 @@
         <v>0</v>
       </c>
       <c r="U98" s="10" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="99" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A99" s="7" t="s">
+        <v>337</v>
+      </c>
+      <c r="B99" s="8">
+        <v>46092.491661747685</v>
+      </c>
+      <c r="C99" s="9"/>
+      <c r="D99" s="8">
+        <v>46181.16820616898</v>
+      </c>
+      <c r="E99" s="9" t="s">
+        <v>338</v>
+      </c>
+      <c r="F99" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="G99" s="9" t="s">
+        <v>49</v>
+      </c>
+      <c r="H99" s="9" t="s">
+        <v>50</v>
+      </c>
+      <c r="I99" s="8">
+        <v>46174</v>
+      </c>
+      <c r="J99" s="8">
+        <v>46181</v>
+      </c>
+      <c r="K99" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="L99" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="M99" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="N99" s="9" t="s">
+        <v>332</v>
+      </c>
+      <c r="O99" s="9" t="s">
+        <v>335</v>
+      </c>
+      <c r="P99" s="9" t="s">
+        <v>332</v>
+      </c>
+      <c r="Q99" s="8">
+        <v>46174</v>
+      </c>
+      <c r="R99" s="8">
+        <v>46181</v>
+      </c>
+      <c r="S99" s="11" t="s">
+        <v>128</v>
+      </c>
+      <c r="T99" s="9">
+        <v>0</v>
+      </c>
+      <c r="U99" s="10" t="s">
         <v>58</v>
       </c>
     </row>

</xml_diff>

<commit_message>
KPI actualizado 2026-07-07 14:39 UTC
</commit_message>
<xml_diff>
--- a/data/50001490 - ZITRON PERU METRO LIMA PV04-PV05.xlsx
+++ b/data/50001490 - ZITRON PERU METRO LIMA PV04-PV05.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1218" uniqueCount="339">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1218" uniqueCount="341">
   <si>
     <t xml:space="preserve">50001490-ZITRON PERU METRO DE LIMA PV04-PV05 </t>
   </si>
@@ -944,6 +944,12 @@
   </si>
   <si>
     <t>Coordinacion Entrega con Cliente</t>
+  </si>
+  <si>
+    <t>Karin Pinto</t>
+  </si>
+  <si>
+    <t>kpinto@zitron.com</t>
   </si>
   <si>
     <t>Embalaje,Logistica:</t>
@@ -6886,7 +6892,7 @@
       </c>
       <c r="C90" s="6"/>
       <c r="D90" s="5">
-        <v>46155.16794435185</v>
+        <v>46210.60325569444</v>
       </c>
       <c r="E90" s="6" t="s">
         <v>310</v>
@@ -6895,10 +6901,10 @@
         <v>26</v>
       </c>
       <c r="G90" s="6" t="s">
-        <v>35</v>
+        <v>311</v>
       </c>
       <c r="H90" s="6" t="s">
-        <v>36</v>
+        <v>312</v>
       </c>
       <c r="I90" s="5">
         <v>46155</v>
@@ -6922,7 +6928,7 @@
         <v>304</v>
       </c>
       <c r="P90" s="6" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="Q90" s="5">
         <v>46155</v>
@@ -6942,7 +6948,7 @@
     </row>
     <row r="91" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A91" s="7" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="B91" s="8">
         <v>46073.69994638889</v>
@@ -6982,10 +6988,10 @@
         <v>307</v>
       </c>
       <c r="O91" s="9" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="P91" s="9" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="Q91" s="8">
         <v>46156</v>
@@ -7005,7 +7011,7 @@
     </row>
     <row r="92" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A92" s="4" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="B92" s="5">
         <v>46073.69994668981</v>
@@ -7015,7 +7021,7 @@
         <v>46161.25032122685</v>
       </c>
       <c r="E92" s="6" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="F92" s="6" t="s">
         <v>26</v>
@@ -7048,7 +7054,7 @@
         <v>276</v>
       </c>
       <c r="P92" s="6" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="Q92" s="5">
         <v>46161</v>
@@ -7068,7 +7074,7 @@
     </row>
     <row r="93" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A93" s="7" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="B93" s="8">
         <v>46073.69994695602</v>
@@ -7078,7 +7084,7 @@
         <v>46162.25040996527</v>
       </c>
       <c r="E93" s="9" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="F93" s="9" t="s">
         <v>26</v>
@@ -7108,10 +7114,10 @@
         <v>307</v>
       </c>
       <c r="O93" s="9" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="P93" s="9" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="Q93" s="8">
         <v>46162</v>
@@ -7131,7 +7137,7 @@
     </row>
     <row r="94" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A94" s="4" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="B94" s="5">
         <v>46073.699947245375</v>
@@ -7141,7 +7147,7 @@
         <v>46077.6387968287</v>
       </c>
       <c r="E94" s="6" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="F94" s="6" t="s">
         <v>25</v>
@@ -7165,7 +7171,7 @@
         <v>26</v>
       </c>
       <c r="O94" s="6" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="P94" s="6" t="s">
         <v>26</v>
@@ -7178,7 +7184,7 @@
     </row>
     <row r="95" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A95" s="7" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
       <c r="B95" s="8">
         <v>46073.699947500005</v>
@@ -7188,16 +7194,16 @@
         <v>46174.16833755787</v>
       </c>
       <c r="E95" s="9" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="F95" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G95" s="9" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="H95" s="9" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="I95" s="8">
         <v>46164</v>
@@ -7215,13 +7221,13 @@
         <v>26</v>
       </c>
       <c r="N95" s="9" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="O95" s="9" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="P95" s="9" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="Q95" s="8">
         <v>46164</v>
@@ -7241,7 +7247,7 @@
     </row>
     <row r="96" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A96" s="4" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="B96" s="5">
         <v>46073.699947789355</v>
@@ -7251,16 +7257,16 @@
         <v>46174.168340185184</v>
       </c>
       <c r="E96" s="6" t="s">
+        <v>331</v>
+      </c>
+      <c r="F96" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="G96" s="6" t="s">
+        <v>328</v>
+      </c>
+      <c r="H96" s="6" t="s">
         <v>329</v>
-      </c>
-      <c r="F96" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="G96" s="6" t="s">
-        <v>326</v>
-      </c>
-      <c r="H96" s="6" t="s">
-        <v>327</v>
       </c>
       <c r="I96" s="5">
         <v>46164</v>
@@ -7278,13 +7284,13 @@
         <v>26</v>
       </c>
       <c r="N96" s="6" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="O96" s="6" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="P96" s="6" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="Q96" s="5">
         <v>46164</v>
@@ -7304,7 +7310,7 @@
     </row>
     <row r="97" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A97" s="7" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="B97" s="8">
         <v>46092.48971385417</v>
@@ -7314,7 +7320,7 @@
         <v>46092.497058946756</v>
       </c>
       <c r="E97" s="9" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="F97" s="9" t="s">
         <v>25</v>
@@ -7338,7 +7344,7 @@
         <v>26</v>
       </c>
       <c r="O97" s="9" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="P97" s="9" t="s">
         <v>26</v>
@@ -7357,7 +7363,7 @@
     </row>
     <row r="98" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A98" s="4" t="s">
-        <v>334</v>
+        <v>336</v>
       </c>
       <c r="B98" s="5">
         <v>46092.49161491898</v>
@@ -7367,7 +7373,7 @@
         <v>46171.168742951384</v>
       </c>
       <c r="E98" s="6" t="s">
-        <v>335</v>
+        <v>337</v>
       </c>
       <c r="F98" s="6" t="s">
         <v>26</v>
@@ -7394,13 +7400,13 @@
         <v>26</v>
       </c>
       <c r="N98" s="6" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="O98" s="6" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="P98" s="6" t="s">
-        <v>336</v>
+        <v>338</v>
       </c>
       <c r="Q98" s="5">
         <v>46164</v>
@@ -7420,7 +7426,7 @@
     </row>
     <row r="99" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A99" s="7" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="B99" s="8">
         <v>46092.491661747685</v>
@@ -7430,7 +7436,7 @@
         <v>46181.16820616898</v>
       </c>
       <c r="E99" s="9" t="s">
-        <v>338</v>
+        <v>340</v>
       </c>
       <c r="F99" s="9" t="s">
         <v>26</v>
@@ -7457,13 +7463,13 @@
         <v>26</v>
       </c>
       <c r="N99" s="9" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="O99" s="9" t="s">
-        <v>335</v>
+        <v>337</v>
       </c>
       <c r="P99" s="9" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="Q99" s="8">
         <v>46174</v>

</xml_diff>

<commit_message>
KPI actualizado 2026-07-07 20:46 UTC
</commit_message>
<xml_diff>
--- a/data/50001490 - ZITRON PERU METRO LIMA PV04-PV05.xlsx
+++ b/data/50001490 - ZITRON PERU METRO LIMA PV04-PV05.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1218" uniqueCount="341">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1169" uniqueCount="326">
   <si>
     <t xml:space="preserve">50001490-ZITRON PERU METRO DE LIMA PV04-PV05 </t>
   </si>
@@ -643,6 +643,9 @@
     <t>nicolas.lopez@zitron.com</t>
   </si>
   <si>
+    <t>Revestimiento</t>
+  </si>
+  <si>
     <t>1213380177588299</t>
   </si>
   <si>
@@ -685,7 +688,7 @@
     <t>1213598288999630</t>
   </si>
   <si>
-    <t xml:space="preserve">Armado,Control de calidad Armado,Montaje motor,Montaje Alabe,Montaje Rodete,Ingenieria y diseñoo:,Montaje Sensor,Propuesta Fabricacion externa </t>
+    <t xml:space="preserve">Montaje motor,Montaje Alabe,Montaje Rodete,Ingenieria y diseñoo:,Montaje Sensor,Propuesta Fabricacion externa </t>
   </si>
   <si>
     <t>1213598288999631</t>
@@ -736,238 +739,190 @@
     <t>Control de calidad compras materiales a codigo // compras locale aprovisionamiento</t>
   </si>
   <si>
-    <t>Bodega:,Preparación Materiales</t>
-  </si>
-  <si>
-    <t>1213380177588305</t>
-  </si>
-  <si>
-    <t>Caldereria:</t>
-  </si>
-  <si>
-    <t>Preparación Materiales,Armado,Control de calidad Armado</t>
-  </si>
-  <si>
-    <t>1213380177588306</t>
-  </si>
-  <si>
-    <t>Preparación Materiales</t>
+    <t>1213380177588309</t>
+  </si>
+  <si>
+    <t>Recepcion motor,Recepcion Sensor,Recepcion Alabe,Recepcion Tableros,Recepcion Rodete</t>
+  </si>
+  <si>
+    <t>1213380177588310</t>
+  </si>
+  <si>
+    <t>Recepcion Rodete</t>
+  </si>
+  <si>
+    <t>Bodega:,Montaje Rodete</t>
+  </si>
+  <si>
+    <t>1213380177588311</t>
+  </si>
+  <si>
+    <t>Bodega:,Revisión tableros pruebas</t>
+  </si>
+  <si>
+    <t>1213380177588312</t>
+  </si>
+  <si>
+    <t>Recepcion Alabe</t>
+  </si>
+  <si>
+    <t>Bodega:,Montaje Alabe</t>
+  </si>
+  <si>
+    <t>1213380177588313</t>
+  </si>
+  <si>
+    <t>Recepcion motor</t>
+  </si>
+  <si>
+    <t>Bodega:,Montaje motor</t>
+  </si>
+  <si>
+    <t>1213400421980588</t>
+  </si>
+  <si>
+    <t>Recepcion Sensor</t>
+  </si>
+  <si>
+    <t>Bodega:,Montaje Sensor</t>
+  </si>
+  <si>
+    <t>1213400424143464</t>
+  </si>
+  <si>
+    <t>Recepcion Atenuador</t>
+  </si>
+  <si>
+    <t>Embalaje</t>
+  </si>
+  <si>
+    <t>1213400424143465</t>
+  </si>
+  <si>
+    <t>1213380177588314</t>
+  </si>
+  <si>
+    <t>Montaje:</t>
+  </si>
+  <si>
+    <t>Revestimiento,Montaje motor,Montaje Alabe,Montaje Rodete,Montaje Sensor,Pruebas FAT,RE-PINTADO</t>
+  </si>
+  <si>
+    <t>1213380177588315</t>
+  </si>
+  <si>
+    <t>benjamin.bustos@zitron.com</t>
+  </si>
+  <si>
+    <t>Montaje motor,Montaje Alabe,Montaje Rodete,Montaje:,Montaje Sensor</t>
+  </si>
+  <si>
+    <t>1213380177588316</t>
+  </si>
+  <si>
+    <t>Montaje motor</t>
+  </si>
+  <si>
+    <t>Revestimiento,Recepcion motor,Check Planos</t>
+  </si>
+  <si>
+    <t>Pruebas FAT,Montaje:</t>
+  </si>
+  <si>
+    <t>1213380177588317</t>
+  </si>
+  <si>
+    <t>Montaje Alabe</t>
+  </si>
+  <si>
+    <t>Revestimiento,Recepcion Alabe,Check Planos</t>
+  </si>
+  <si>
+    <t>1213380177588318</t>
+  </si>
+  <si>
+    <t>Montaje Rodete</t>
+  </si>
+  <si>
+    <t>Revestimiento,Recepcion Rodete,Check Planos</t>
+  </si>
+  <si>
+    <t>Media</t>
+  </si>
+  <si>
+    <t>1213400421980589</t>
+  </si>
+  <si>
+    <t>Montaje Sensor</t>
+  </si>
+  <si>
+    <t>Revestimiento,Recepcion Sensor,Check Planos</t>
+  </si>
+  <si>
+    <t>Pruebas FAT,Montaje:,Pruebas FAT</t>
+  </si>
+  <si>
+    <t>1213380177588319</t>
+  </si>
+  <si>
+    <t>Montaje motor,Montaje Alabe,Montaje Rodete,Montaje Sensor</t>
+  </si>
+  <si>
+    <t>Montaje:,Check Pruebas FAT</t>
+  </si>
+  <si>
+    <t>1213380177588320</t>
+  </si>
+  <si>
+    <t>RE-PINTADO</t>
+  </si>
+  <si>
+    <t>Montaje:,Coordinacion Entrega con Cliente</t>
+  </si>
+  <si>
+    <t>1213380177588321</t>
+  </si>
+  <si>
+    <t>Logistica:</t>
+  </si>
+  <si>
+    <t>Coordinacion Entrega con Cliente,Embalaje,PACKING LIST,Despacho</t>
+  </si>
+  <si>
+    <t>1213380177588322</t>
+  </si>
+  <si>
+    <t>Coordinacion Entrega con Cliente</t>
+  </si>
+  <si>
+    <t>Karin Pinto</t>
+  </si>
+  <si>
+    <t>kpinto@zitron.com</t>
+  </si>
+  <si>
+    <t>Embalaje,Logistica:</t>
+  </si>
+  <si>
+    <t>1213380177588323</t>
+  </si>
+  <si>
+    <t>Coordinacion Entrega con Cliente,Revisión tableros pruebas,Recepcion Atenuador,Recepcion  Damper</t>
+  </si>
+  <si>
+    <t>PACKING LIST,Logistica:</t>
+  </si>
+  <si>
+    <t>1213380177588324</t>
+  </si>
+  <si>
+    <t>PACKING LIST</t>
   </si>
   <si>
     <t>Nicolás Mol</t>
   </si>
   <si>
     <t>nicolas.mol@zitron.com</t>
-  </si>
-  <si>
-    <t>Armado,Caldereria:</t>
-  </si>
-  <si>
-    <t>1213380177588307</t>
-  </si>
-  <si>
-    <t>Armado</t>
-  </si>
-  <si>
-    <t>Preparación Materiales,Check Planos</t>
-  </si>
-  <si>
-    <t>Control de calidad Armado,Caldereria:</t>
-  </si>
-  <si>
-    <t>1213380177588308</t>
-  </si>
-  <si>
-    <t>Control de calidad Armado</t>
-  </si>
-  <si>
-    <t>Armado,Check Planos</t>
-  </si>
-  <si>
-    <t>Caldereria:,Revestimiento</t>
-  </si>
-  <si>
-    <t>1213380177588309</t>
-  </si>
-  <si>
-    <t>Recepcion motor,Recepcion Sensor,Recepcion Alabe,Recepcion Tableros,Recepcion Rodete</t>
-  </si>
-  <si>
-    <t>1213380177588310</t>
-  </si>
-  <si>
-    <t>Recepcion Rodete</t>
-  </si>
-  <si>
-    <t>Bodega:,Montaje Rodete</t>
-  </si>
-  <si>
-    <t>1213380177588311</t>
-  </si>
-  <si>
-    <t>Bodega:,Revisión tableros pruebas</t>
-  </si>
-  <si>
-    <t>1213380177588312</t>
-  </si>
-  <si>
-    <t>Recepcion Alabe</t>
-  </si>
-  <si>
-    <t>Bodega:,Montaje Alabe</t>
-  </si>
-  <si>
-    <t>1213380177588313</t>
-  </si>
-  <si>
-    <t>Recepcion motor</t>
-  </si>
-  <si>
-    <t>Bodega:,Montaje motor</t>
-  </si>
-  <si>
-    <t>1213400421980588</t>
-  </si>
-  <si>
-    <t>Recepcion Sensor</t>
-  </si>
-  <si>
-    <t>Bodega:,Montaje Sensor</t>
-  </si>
-  <si>
-    <t>1213400424143464</t>
-  </si>
-  <si>
-    <t>Recepcion Atenuador</t>
-  </si>
-  <si>
-    <t>Embalaje</t>
-  </si>
-  <si>
-    <t>1213400424143465</t>
-  </si>
-  <si>
-    <t>1213380177588314</t>
-  </si>
-  <si>
-    <t>Montaje:</t>
-  </si>
-  <si>
-    <t>Revestimiento,Montaje motor,Montaje Alabe,Montaje Rodete,Montaje Sensor,Pruebas FAT,RE-PINTADO</t>
-  </si>
-  <si>
-    <t>1213380177588315</t>
-  </si>
-  <si>
-    <t>Revestimiento</t>
-  </si>
-  <si>
-    <t>benjamin.bustos@zitron.com</t>
-  </si>
-  <si>
-    <t>Montaje motor,Montaje Alabe,Montaje Rodete,Montaje:,Montaje Sensor</t>
-  </si>
-  <si>
-    <t>1213380177588316</t>
-  </si>
-  <si>
-    <t>Montaje motor</t>
-  </si>
-  <si>
-    <t>Revestimiento,Recepcion motor,Check Planos</t>
-  </si>
-  <si>
-    <t>Pruebas FAT,Montaje:</t>
-  </si>
-  <si>
-    <t>1213380177588317</t>
-  </si>
-  <si>
-    <t>Montaje Alabe</t>
-  </si>
-  <si>
-    <t>Revestimiento,Recepcion Alabe,Check Planos</t>
-  </si>
-  <si>
-    <t>1213380177588318</t>
-  </si>
-  <si>
-    <t>Montaje Rodete</t>
-  </si>
-  <si>
-    <t>Revestimiento,Recepcion Rodete,Check Planos</t>
-  </si>
-  <si>
-    <t>Media</t>
-  </si>
-  <si>
-    <t>1213400421980589</t>
-  </si>
-  <si>
-    <t>Montaje Sensor</t>
-  </si>
-  <si>
-    <t>Revestimiento,Recepcion Sensor,Check Planos</t>
-  </si>
-  <si>
-    <t>Pruebas FAT,Montaje:,Pruebas FAT</t>
-  </si>
-  <si>
-    <t>1213380177588319</t>
-  </si>
-  <si>
-    <t>Montaje motor,Montaje Alabe,Montaje Rodete,Montaje Sensor</t>
-  </si>
-  <si>
-    <t>Montaje:,Check Pruebas FAT</t>
-  </si>
-  <si>
-    <t>1213380177588320</t>
-  </si>
-  <si>
-    <t>RE-PINTADO</t>
-  </si>
-  <si>
-    <t>Montaje:,Coordinacion Entrega con Cliente</t>
-  </si>
-  <si>
-    <t>1213380177588321</t>
-  </si>
-  <si>
-    <t>Logistica:</t>
-  </si>
-  <si>
-    <t>Coordinacion Entrega con Cliente,Embalaje,PACKING LIST,Despacho</t>
-  </si>
-  <si>
-    <t>1213380177588322</t>
-  </si>
-  <si>
-    <t>Coordinacion Entrega con Cliente</t>
-  </si>
-  <si>
-    <t>Karin Pinto</t>
-  </si>
-  <si>
-    <t>kpinto@zitron.com</t>
-  </si>
-  <si>
-    <t>Embalaje,Logistica:</t>
-  </si>
-  <si>
-    <t>1213380177588323</t>
-  </si>
-  <si>
-    <t>Coordinacion Entrega con Cliente,Revisión tableros pruebas,Recepcion Atenuador,Recepcion  Damper</t>
-  </si>
-  <si>
-    <t>PACKING LIST,Logistica:</t>
-  </si>
-  <si>
-    <t>1213380177588324</t>
-  </si>
-  <si>
-    <t>PACKING LIST</t>
   </si>
   <si>
     <t>Despacho,Logistica:</t>
@@ -1557,7 +1512,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:U99"/>
+  <dimension ref="A1:U95"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="10.4" customWidth="1"/>
@@ -5098,7 +5053,7 @@
       </c>
       <c r="C60" s="6"/>
       <c r="D60" s="5">
-        <v>46205.80976949074</v>
+        <v>46210.86168509259</v>
       </c>
       <c r="E60" s="6" t="s">
         <v>207</v>
@@ -5132,7 +5087,7 @@
         <v>26</v>
       </c>
       <c r="P60" s="6" t="s">
-        <v>26</v>
+        <v>210</v>
       </c>
       <c r="Q60" s="6"/>
       <c r="R60" s="6"/>
@@ -5142,7 +5097,7 @@
     </row>
     <row r="61" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A61" s="7" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="B61" s="8">
         <v>46073.69994815972</v>
@@ -5152,7 +5107,7 @@
         <v>46129.586425601854</v>
       </c>
       <c r="E61" s="9" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="F61" s="9" t="s">
         <v>25</v>
@@ -5176,7 +5131,7 @@
         <v>26</v>
       </c>
       <c r="O61" s="9" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="P61" s="9" t="s">
         <v>26</v>
@@ -5189,7 +5144,7 @@
     </row>
     <row r="62" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A62" s="4" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="B62" s="5">
         <v>46073.6999484375</v>
@@ -5201,16 +5156,16 @@
         <v>46099.54242268519</v>
       </c>
       <c r="E62" s="6" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="F62" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G62" s="6" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="H62" s="6" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="I62" s="5">
         <v>46003</v>
@@ -5228,13 +5183,13 @@
         <v>26</v>
       </c>
       <c r="N62" s="6" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="O62" s="6" t="s">
         <v>74</v>
       </c>
       <c r="P62" s="6" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="Q62" s="5">
         <v>46003</v>
@@ -5254,7 +5209,7 @@
     </row>
     <row r="63" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A63" s="7" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="B63" s="8">
         <v>46073.699946249995</v>
@@ -5266,16 +5221,16 @@
         <v>46129.58626813657</v>
       </c>
       <c r="E63" s="9" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="F63" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G63" s="9" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="H63" s="9" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="I63" s="8">
         <v>46058</v>
@@ -5293,13 +5248,13 @@
         <v>26</v>
       </c>
       <c r="N63" s="9" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="O63" s="9" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="P63" s="9" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="Q63" s="8">
         <v>46058</v>
@@ -5319,7 +5274,7 @@
     </row>
     <row r="64" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A64" s="4" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="B64" s="5">
         <v>46092.494241736116</v>
@@ -5328,7 +5283,7 @@
         <v>46129.58641790509</v>
       </c>
       <c r="D64" s="5">
-        <v>46139.54817715278</v>
+        <v>46210.861392569444</v>
       </c>
       <c r="E64" s="6" t="s">
         <v>115</v>
@@ -5337,10 +5292,10 @@
         <v>26</v>
       </c>
       <c r="G64" s="6" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="H64" s="6" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="I64" s="6"/>
       <c r="J64" s="5">
@@ -5356,13 +5311,13 @@
         <v>26</v>
       </c>
       <c r="N64" s="6" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="O64" s="6" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="P64" s="6" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="Q64" s="5">
         <v>46065</v>
@@ -5382,7 +5337,7 @@
     </row>
     <row r="65" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A65" s="7" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="B65" s="8">
         <v>46092.49428590278</v>
@@ -5392,16 +5347,16 @@
         <v>46154.16811805556</v>
       </c>
       <c r="E65" s="9" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="F65" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G65" s="9" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="H65" s="9" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="I65" s="8">
         <v>46154</v>
@@ -5419,13 +5374,13 @@
         <v>26</v>
       </c>
       <c r="N65" s="9" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="O65" s="9" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="P65" s="9" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="Q65" s="8">
         <v>46154</v>
@@ -5445,17 +5400,17 @@
     </row>
     <row r="66" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A66" s="4" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="B66" s="5">
         <v>46073.69994662037</v>
       </c>
       <c r="C66" s="6"/>
       <c r="D66" s="5">
-        <v>46206.53745743056</v>
+        <v>46210.858702094905</v>
       </c>
       <c r="E66" s="6" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="F66" s="6" t="s">
         <v>25</v>
@@ -5479,7 +5434,7 @@
         <v>26</v>
       </c>
       <c r="O66" s="6" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="P66" s="6" t="s">
         <v>26</v>
@@ -5492,26 +5447,28 @@
     </row>
     <row r="67" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A67" s="7" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="B67" s="8">
         <v>46073.69994689815</v>
       </c>
-      <c r="C67" s="9"/>
+      <c r="C67" s="8">
+        <v>46210.858693472226</v>
+      </c>
       <c r="D67" s="8">
-        <v>46199.82444644676</v>
+        <v>46210.85869597222</v>
       </c>
       <c r="E67" s="9" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="F67" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G67" s="9" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="H67" s="9" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="I67" s="8">
         <v>46063</v>
@@ -5529,13 +5486,13 @@
         <v>26</v>
       </c>
       <c r="N67" s="9" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="O67" s="9" t="s">
         <v>171</v>
       </c>
       <c r="P67" s="9" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="Q67" s="8">
         <v>46063</v>
@@ -5555,7 +5512,7 @@
     </row>
     <row r="68" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A68" s="4" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="B68" s="5">
         <v>46073.69994719907</v>
@@ -5564,10 +5521,10 @@
         <v>46206.53745016204</v>
       </c>
       <c r="D68" s="5">
-        <v>46206.53745243055</v>
+        <v>46210.86139240741</v>
       </c>
       <c r="E68" s="6" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="F68" s="6" t="s">
         <v>26</v>
@@ -5594,13 +5551,13 @@
         <v>26</v>
       </c>
       <c r="N68" s="6" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="O68" s="6" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="P68" s="6" t="s">
-        <v>241</v>
+        <v>233</v>
       </c>
       <c r="Q68" s="5">
         <v>46065</v>
@@ -5623,14 +5580,14 @@
         <v>242</v>
       </c>
       <c r="B69" s="8">
-        <v>46073.69994748842</v>
+        <v>46073.699948865746</v>
       </c>
       <c r="C69" s="9"/>
       <c r="D69" s="8">
-        <v>46077.62916171296</v>
+        <v>46195.604225717594</v>
       </c>
       <c r="E69" s="9" t="s">
-        <v>243</v>
+        <v>233</v>
       </c>
       <c r="F69" s="9" t="s">
         <v>25</v>
@@ -5654,7 +5611,7 @@
         <v>26</v>
       </c>
       <c r="O69" s="9" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="P69" s="9" t="s">
         <v>26</v>
@@ -5667,56 +5624,56 @@
     </row>
     <row r="70" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A70" s="4" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="B70" s="5">
-        <v>46073.69994777778</v>
+        <v>46073.69995097222</v>
       </c>
       <c r="C70" s="6"/>
       <c r="D70" s="5">
-        <v>46206.53745877315</v>
+        <v>46199.830143969906</v>
       </c>
       <c r="E70" s="6" t="s">
+        <v>245</v>
+      </c>
+      <c r="F70" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="G70" s="6" t="s">
+        <v>237</v>
+      </c>
+      <c r="H70" s="6" t="s">
+        <v>238</v>
+      </c>
+      <c r="I70" s="5">
+        <v>46097</v>
+      </c>
+      <c r="J70" s="5">
+        <v>46098</v>
+      </c>
+      <c r="K70" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="L70" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="M70" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="N70" s="6" t="s">
+        <v>233</v>
+      </c>
+      <c r="O70" s="6" t="s">
+        <v>148</v>
+      </c>
+      <c r="P70" s="6" t="s">
         <v>246</v>
       </c>
-      <c r="F70" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="G70" s="6" t="s">
-        <v>247</v>
-      </c>
-      <c r="H70" s="6" t="s">
-        <v>248</v>
-      </c>
-      <c r="I70" s="5">
-        <v>46069</v>
-      </c>
-      <c r="J70" s="5">
-        <v>46077</v>
-      </c>
-      <c r="K70" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="L70" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="M70" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="N70" s="6" t="s">
-        <v>243</v>
-      </c>
-      <c r="O70" s="6" t="s">
-        <v>240</v>
-      </c>
-      <c r="P70" s="6" t="s">
-        <v>249</v>
-      </c>
       <c r="Q70" s="5">
-        <v>46069</v>
+        <v>46097</v>
       </c>
       <c r="R70" s="5">
-        <v>46077</v>
+        <v>46098</v>
       </c>
       <c r="S70" s="10" t="s">
         <v>31</v>
@@ -5730,56 +5687,56 @@
     </row>
     <row r="71" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A71" s="7" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="B71" s="8">
-        <v>46073.699948113426</v>
+        <v>46073.69994640046</v>
       </c>
       <c r="C71" s="9"/>
       <c r="D71" s="8">
-        <v>46129.58642229167</v>
+        <v>46121.187778182866</v>
       </c>
       <c r="E71" s="9" t="s">
-        <v>251</v>
+        <v>56</v>
       </c>
       <c r="F71" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G71" s="9" t="s">
-        <v>247</v>
+        <v>237</v>
       </c>
       <c r="H71" s="9" t="s">
+        <v>238</v>
+      </c>
+      <c r="I71" s="8">
+        <v>46119</v>
+      </c>
+      <c r="J71" s="8">
+        <v>46120</v>
+      </c>
+      <c r="K71" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="L71" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="M71" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="N71" s="9" t="s">
+        <v>233</v>
+      </c>
+      <c r="O71" s="9" t="s">
+        <v>139</v>
+      </c>
+      <c r="P71" s="9" t="s">
         <v>248</v>
       </c>
-      <c r="I71" s="8">
-        <v>46078</v>
-      </c>
-      <c r="J71" s="8">
-        <v>46106</v>
-      </c>
-      <c r="K71" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="L71" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="M71" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="N71" s="9" t="s">
-        <v>243</v>
-      </c>
-      <c r="O71" s="9" t="s">
-        <v>252</v>
-      </c>
-      <c r="P71" s="9" t="s">
-        <v>253</v>
-      </c>
       <c r="Q71" s="8">
-        <v>46078</v>
+        <v>46119</v>
       </c>
       <c r="R71" s="8">
-        <v>46106</v>
+        <v>46120</v>
       </c>
       <c r="S71" s="10" t="s">
         <v>31</v>
@@ -5793,32 +5750,32 @@
     </row>
     <row r="72" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A72" s="4" t="s">
-        <v>254</v>
+        <v>249</v>
       </c>
       <c r="B72" s="5">
-        <v>46073.69994846065</v>
+        <v>46073.699946782406</v>
       </c>
       <c r="C72" s="6"/>
       <c r="D72" s="5">
-        <v>46209.56306775463</v>
+        <v>46199.82646660879</v>
       </c>
       <c r="E72" s="6" t="s">
-        <v>255</v>
+        <v>250</v>
       </c>
       <c r="F72" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G72" s="6" t="s">
-        <v>208</v>
+        <v>237</v>
       </c>
       <c r="H72" s="6" t="s">
-        <v>209</v>
+        <v>238</v>
       </c>
       <c r="I72" s="5">
-        <v>46107</v>
+        <v>46132</v>
       </c>
       <c r="J72" s="5">
-        <v>46108</v>
+        <v>46133</v>
       </c>
       <c r="K72" s="6" t="s">
         <v>26</v>
@@ -5830,19 +5787,19 @@
         <v>26</v>
       </c>
       <c r="N72" s="6" t="s">
-        <v>243</v>
+        <v>233</v>
       </c>
       <c r="O72" s="6" t="s">
-        <v>256</v>
+        <v>130</v>
       </c>
       <c r="P72" s="6" t="s">
-        <v>257</v>
+        <v>251</v>
       </c>
       <c r="Q72" s="5">
-        <v>46107</v>
+        <v>46132</v>
       </c>
       <c r="R72" s="5">
-        <v>46108</v>
+        <v>46133</v>
       </c>
       <c r="S72" s="10" t="s">
         <v>31</v>
@@ -5856,27 +5813,35 @@
     </row>
     <row r="73" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A73" s="7" t="s">
-        <v>258</v>
+        <v>252</v>
       </c>
       <c r="B73" s="8">
-        <v>46073.699948865746</v>
-      </c>
-      <c r="C73" s="9"/>
+        <v>46073.69994708333</v>
+      </c>
+      <c r="C73" s="8">
+        <v>46195.603957824074</v>
+      </c>
       <c r="D73" s="8">
-        <v>46195.604225717594</v>
+        <v>46195.603959687505</v>
       </c>
       <c r="E73" s="9" t="s">
-        <v>232</v>
+        <v>253</v>
       </c>
       <c r="F73" s="9" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G73" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="H73" s="9"/>
-      <c r="I73" s="9"/>
-      <c r="J73" s="9"/>
+        <v>237</v>
+      </c>
+      <c r="H73" s="9" t="s">
+        <v>238</v>
+      </c>
+      <c r="I73" s="8">
+        <v>46147</v>
+      </c>
+      <c r="J73" s="8">
+        <v>46148</v>
+      </c>
       <c r="K73" s="9" t="s">
         <v>26</v>
       </c>
@@ -5884,51 +5849,63 @@
         <v>26</v>
       </c>
       <c r="M73" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="N73" s="9" t="s">
+        <v>233</v>
+      </c>
+      <c r="O73" s="9" t="s">
+        <v>157</v>
+      </c>
+      <c r="P73" s="9" t="s">
+        <v>254</v>
+      </c>
+      <c r="Q73" s="8">
+        <v>46147</v>
+      </c>
+      <c r="R73" s="8">
+        <v>46148</v>
+      </c>
+      <c r="S73" s="11" t="s">
+        <v>128</v>
+      </c>
+      <c r="T73" s="9">
         <v>0</v>
       </c>
-      <c r="N73" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="O73" s="9" t="s">
-        <v>259</v>
-      </c>
-      <c r="P73" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="Q73" s="9"/>
-      <c r="R73" s="9"/>
-      <c r="S73" s="9"/>
-      <c r="T73" s="9"/>
-      <c r="U73" s="9"/>
+      <c r="U73" s="12" t="s">
+        <v>201</v>
+      </c>
     </row>
     <row r="74" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A74" s="4" t="s">
-        <v>260</v>
+        <v>255</v>
       </c>
       <c r="B74" s="5">
-        <v>46073.69995097222</v>
-      </c>
-      <c r="C74" s="6"/>
+        <v>46076.88127923611</v>
+      </c>
+      <c r="C74" s="5">
+        <v>46195.60421921297</v>
+      </c>
       <c r="D74" s="5">
-        <v>46199.830143969906</v>
+        <v>46195.60422127315</v>
       </c>
       <c r="E74" s="6" t="s">
-        <v>261</v>
+        <v>256</v>
       </c>
       <c r="F74" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G74" s="6" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="H74" s="6" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="I74" s="5">
-        <v>46097</v>
+        <v>46121</v>
       </c>
       <c r="J74" s="5">
-        <v>46098</v>
+        <v>46122</v>
       </c>
       <c r="K74" s="6" t="s">
         <v>26</v>
@@ -5940,19 +5917,19 @@
         <v>26</v>
       </c>
       <c r="N74" s="6" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="O74" s="6" t="s">
-        <v>148</v>
+        <v>180</v>
       </c>
       <c r="P74" s="6" t="s">
-        <v>262</v>
+        <v>257</v>
       </c>
       <c r="Q74" s="5">
-        <v>46097</v>
+        <v>46121</v>
       </c>
       <c r="R74" s="5">
-        <v>46098</v>
+        <v>46122</v>
       </c>
       <c r="S74" s="10" t="s">
         <v>31</v>
@@ -5960,38 +5937,40 @@
       <c r="T74" s="6">
         <v>0</v>
       </c>
-      <c r="U74" s="10" t="s">
-        <v>58</v>
+      <c r="U74" s="12" t="s">
+        <v>201</v>
       </c>
     </row>
     <row r="75" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A75" s="7" t="s">
-        <v>263</v>
+        <v>258</v>
       </c>
       <c r="B75" s="8">
-        <v>46073.69994640046</v>
-      </c>
-      <c r="C75" s="9"/>
+        <v>46077.57961084491</v>
+      </c>
+      <c r="C75" s="8">
+        <v>46195.60466336805</v>
+      </c>
       <c r="D75" s="8">
-        <v>46121.187778182866</v>
+        <v>46195.60466490741</v>
       </c>
       <c r="E75" s="9" t="s">
-        <v>56</v>
+        <v>259</v>
       </c>
       <c r="F75" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G75" s="9" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="H75" s="9" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="I75" s="8">
-        <v>46119</v>
+        <v>46104</v>
       </c>
       <c r="J75" s="8">
-        <v>46120</v>
+        <v>46105</v>
       </c>
       <c r="K75" s="9" t="s">
         <v>26</v>
@@ -6003,19 +5982,19 @@
         <v>26</v>
       </c>
       <c r="N75" s="9" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="O75" s="9" t="s">
-        <v>139</v>
+        <v>195</v>
       </c>
       <c r="P75" s="9" t="s">
-        <v>264</v>
+        <v>260</v>
       </c>
       <c r="Q75" s="8">
-        <v>46119</v>
+        <v>46104</v>
       </c>
       <c r="R75" s="8">
-        <v>46120</v>
+        <v>46105</v>
       </c>
       <c r="S75" s="10" t="s">
         <v>31</v>
@@ -6029,32 +6008,32 @@
     </row>
     <row r="76" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A76" s="4" t="s">
-        <v>265</v>
+        <v>261</v>
       </c>
       <c r="B76" s="5">
-        <v>46073.699946782406</v>
+        <v>46077.57965403935</v>
       </c>
       <c r="C76" s="6"/>
       <c r="D76" s="5">
-        <v>46199.82646660879</v>
+        <v>46182.692112696765</v>
       </c>
       <c r="E76" s="6" t="s">
-        <v>266</v>
+        <v>188</v>
       </c>
       <c r="F76" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G76" s="6" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="H76" s="6" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="I76" s="5">
-        <v>46132</v>
+        <v>46098</v>
       </c>
       <c r="J76" s="5">
-        <v>46133</v>
+        <v>46099</v>
       </c>
       <c r="K76" s="6" t="s">
         <v>26</v>
@@ -6066,19 +6045,19 @@
         <v>26</v>
       </c>
       <c r="N76" s="6" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="O76" s="6" t="s">
-        <v>130</v>
+        <v>187</v>
       </c>
       <c r="P76" s="6" t="s">
-        <v>267</v>
+        <v>260</v>
       </c>
       <c r="Q76" s="5">
-        <v>46132</v>
+        <v>46098</v>
       </c>
       <c r="R76" s="5">
-        <v>46133</v>
+        <v>46099</v>
       </c>
       <c r="S76" s="10" t="s">
         <v>31</v>
@@ -6092,35 +6071,27 @@
     </row>
     <row r="77" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A77" s="7" t="s">
-        <v>268</v>
+        <v>262</v>
       </c>
       <c r="B77" s="8">
-        <v>46073.69994708333</v>
-      </c>
-      <c r="C77" s="8">
-        <v>46195.603957824074</v>
-      </c>
+        <v>46073.69994733796</v>
+      </c>
+      <c r="C77" s="9"/>
       <c r="D77" s="8">
-        <v>46195.603959687505</v>
+        <v>46078.621237141204</v>
       </c>
       <c r="E77" s="9" t="s">
-        <v>269</v>
+        <v>263</v>
       </c>
       <c r="F77" s="9" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="G77" s="9" t="s">
-        <v>236</v>
-      </c>
-      <c r="H77" s="9" t="s">
-        <v>237</v>
-      </c>
-      <c r="I77" s="8">
-        <v>46147</v>
-      </c>
-      <c r="J77" s="8">
-        <v>46148</v>
-      </c>
+        <v>26</v>
+      </c>
+      <c r="H77" s="9"/>
+      <c r="I77" s="9"/>
+      <c r="J77" s="9"/>
       <c r="K77" s="9" t="s">
         <v>26</v>
       </c>
@@ -6128,63 +6099,51 @@
         <v>26</v>
       </c>
       <c r="M77" s="9" t="s">
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="N77" s="9" t="s">
-        <v>232</v>
+        <v>26</v>
       </c>
       <c r="O77" s="9" t="s">
-        <v>157</v>
+        <v>264</v>
       </c>
       <c r="P77" s="9" t="s">
-        <v>270</v>
-      </c>
-      <c r="Q77" s="8">
-        <v>46147</v>
-      </c>
-      <c r="R77" s="8">
-        <v>46148</v>
-      </c>
-      <c r="S77" s="11" t="s">
-        <v>128</v>
-      </c>
-      <c r="T77" s="9">
-        <v>0</v>
-      </c>
-      <c r="U77" s="12" t="s">
-        <v>201</v>
-      </c>
+        <v>26</v>
+      </c>
+      <c r="Q77" s="9"/>
+      <c r="R77" s="9"/>
+      <c r="S77" s="9"/>
+      <c r="T77" s="9"/>
+      <c r="U77" s="9"/>
     </row>
     <row r="78" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A78" s="4" t="s">
-        <v>271</v>
+        <v>265</v>
       </c>
       <c r="B78" s="5">
-        <v>46076.88127923611</v>
-      </c>
-      <c r="C78" s="5">
-        <v>46195.60421921297</v>
-      </c>
+        <v>46073.69994759259</v>
+      </c>
+      <c r="C78" s="6"/>
       <c r="D78" s="5">
-        <v>46195.60422127315</v>
+        <v>46210.861684930554</v>
       </c>
       <c r="E78" s="6" t="s">
-        <v>272</v>
+        <v>210</v>
       </c>
       <c r="F78" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G78" s="6" t="s">
-        <v>236</v>
+        <v>266</v>
       </c>
       <c r="H78" s="6" t="s">
-        <v>237</v>
+        <v>266</v>
       </c>
       <c r="I78" s="5">
-        <v>46121</v>
+        <v>46111</v>
       </c>
       <c r="J78" s="5">
-        <v>46122</v>
+        <v>46128</v>
       </c>
       <c r="K78" s="6" t="s">
         <v>26</v>
@@ -6196,19 +6155,19 @@
         <v>26</v>
       </c>
       <c r="N78" s="6" t="s">
-        <v>232</v>
+        <v>263</v>
       </c>
       <c r="O78" s="6" t="s">
-        <v>180</v>
+        <v>207</v>
       </c>
       <c r="P78" s="6" t="s">
-        <v>273</v>
+        <v>267</v>
       </c>
       <c r="Q78" s="5">
-        <v>46121</v>
+        <v>46111</v>
       </c>
       <c r="R78" s="5">
-        <v>46122</v>
+        <v>46119</v>
       </c>
       <c r="S78" s="10" t="s">
         <v>31</v>
@@ -6216,40 +6175,38 @@
       <c r="T78" s="6">
         <v>0</v>
       </c>
-      <c r="U78" s="12" t="s">
-        <v>201</v>
+      <c r="U78" s="10" t="s">
+        <v>58</v>
       </c>
     </row>
     <row r="79" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A79" s="7" t="s">
-        <v>274</v>
+        <v>268</v>
       </c>
       <c r="B79" s="8">
-        <v>46077.57961084491</v>
-      </c>
-      <c r="C79" s="8">
-        <v>46195.60466336805</v>
-      </c>
+        <v>46073.69994784722</v>
+      </c>
+      <c r="C79" s="9"/>
       <c r="D79" s="8">
-        <v>46195.60466490741</v>
+        <v>46198.59349042824</v>
       </c>
       <c r="E79" s="9" t="s">
-        <v>275</v>
+        <v>269</v>
       </c>
       <c r="F79" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G79" s="9" t="s">
-        <v>236</v>
+        <v>266</v>
       </c>
       <c r="H79" s="9" t="s">
-        <v>237</v>
+        <v>266</v>
       </c>
       <c r="I79" s="8">
-        <v>46104</v>
+        <v>46149</v>
       </c>
       <c r="J79" s="8">
-        <v>46105</v>
+        <v>46150</v>
       </c>
       <c r="K79" s="9" t="s">
         <v>26</v>
@@ -6261,22 +6218,22 @@
         <v>26</v>
       </c>
       <c r="N79" s="9" t="s">
-        <v>232</v>
+        <v>263</v>
       </c>
       <c r="O79" s="9" t="s">
-        <v>195</v>
+        <v>270</v>
       </c>
       <c r="P79" s="9" t="s">
-        <v>276</v>
+        <v>271</v>
       </c>
       <c r="Q79" s="8">
-        <v>46104</v>
+        <v>46149</v>
       </c>
       <c r="R79" s="8">
-        <v>46105</v>
-      </c>
-      <c r="S79" s="10" t="s">
-        <v>31</v>
+        <v>46150</v>
+      </c>
+      <c r="S79" s="11" t="s">
+        <v>128</v>
       </c>
       <c r="T79" s="9">
         <v>0</v>
@@ -6287,32 +6244,32 @@
     </row>
     <row r="80" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A80" s="4" t="s">
-        <v>277</v>
+        <v>272</v>
       </c>
       <c r="B80" s="5">
-        <v>46077.57965403935</v>
+        <v>46073.69994813658</v>
       </c>
       <c r="C80" s="6"/>
       <c r="D80" s="5">
-        <v>46182.692112696765</v>
+        <v>46198.592367060184</v>
       </c>
       <c r="E80" s="6" t="s">
-        <v>188</v>
+        <v>273</v>
       </c>
       <c r="F80" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G80" s="6" t="s">
-        <v>236</v>
+        <v>266</v>
       </c>
       <c r="H80" s="6" t="s">
-        <v>237</v>
+        <v>266</v>
       </c>
       <c r="I80" s="5">
-        <v>46098</v>
+        <v>46134</v>
       </c>
       <c r="J80" s="5">
-        <v>46099</v>
+        <v>46135</v>
       </c>
       <c r="K80" s="6" t="s">
         <v>26</v>
@@ -6324,19 +6281,19 @@
         <v>26</v>
       </c>
       <c r="N80" s="6" t="s">
-        <v>232</v>
+        <v>263</v>
       </c>
       <c r="O80" s="6" t="s">
-        <v>187</v>
+        <v>274</v>
       </c>
       <c r="P80" s="6" t="s">
-        <v>276</v>
+        <v>271</v>
       </c>
       <c r="Q80" s="5">
-        <v>46098</v>
+        <v>46134</v>
       </c>
       <c r="R80" s="5">
-        <v>46099</v>
+        <v>46135</v>
       </c>
       <c r="S80" s="10" t="s">
         <v>31</v>
@@ -6350,27 +6307,33 @@
     </row>
     <row r="81" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A81" s="7" t="s">
-        <v>278</v>
+        <v>275</v>
       </c>
       <c r="B81" s="8">
-        <v>46073.69994733796</v>
+        <v>46073.699948368056</v>
       </c>
       <c r="C81" s="9"/>
       <c r="D81" s="8">
-        <v>46078.621237141204</v>
+        <v>46198.59272494213</v>
       </c>
       <c r="E81" s="9" t="s">
-        <v>279</v>
+        <v>276</v>
       </c>
       <c r="F81" s="9" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G81" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="H81" s="9"/>
-      <c r="I81" s="9"/>
-      <c r="J81" s="9"/>
+        <v>266</v>
+      </c>
+      <c r="H81" s="9" t="s">
+        <v>266</v>
+      </c>
+      <c r="I81" s="8">
+        <v>46136</v>
+      </c>
+      <c r="J81" s="8">
+        <v>46139</v>
+      </c>
       <c r="K81" s="9" t="s">
         <v>26</v>
       </c>
@@ -6378,75 +6341,85 @@
         <v>26</v>
       </c>
       <c r="M81" s="9" t="s">
-        <v>0</v>
+        <v>26</v>
       </c>
       <c r="N81" s="9" t="s">
-        <v>26</v>
+        <v>263</v>
       </c>
       <c r="O81" s="9" t="s">
-        <v>280</v>
+        <v>277</v>
       </c>
       <c r="P81" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="Q81" s="9"/>
-      <c r="R81" s="9"/>
-      <c r="S81" s="9"/>
-      <c r="T81" s="9"/>
-      <c r="U81" s="9"/>
+        <v>271</v>
+      </c>
+      <c r="Q81" s="8">
+        <v>46136</v>
+      </c>
+      <c r="R81" s="8">
+        <v>46139</v>
+      </c>
+      <c r="S81" s="12" t="s">
+        <v>278</v>
+      </c>
+      <c r="T81" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="U81" s="10" t="s">
+        <v>58</v>
+      </c>
     </row>
     <row r="82" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A82" s="4" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="B82" s="5">
-        <v>46073.69994759259</v>
+        <v>46076.88137268518</v>
       </c>
       <c r="C82" s="6"/>
       <c r="D82" s="5">
-        <v>46128.16821587963</v>
+        <v>46195.60422616898</v>
       </c>
       <c r="E82" s="6" t="s">
+        <v>280</v>
+      </c>
+      <c r="F82" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="G82" s="6" t="s">
+        <v>266</v>
+      </c>
+      <c r="H82" s="6" t="s">
+        <v>266</v>
+      </c>
+      <c r="I82" s="5">
+        <v>46129</v>
+      </c>
+      <c r="J82" s="5">
+        <v>46132</v>
+      </c>
+      <c r="K82" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="L82" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="M82" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="N82" s="6" t="s">
+        <v>263</v>
+      </c>
+      <c r="O82" s="6" t="s">
+        <v>281</v>
+      </c>
+      <c r="P82" s="6" t="s">
         <v>282</v>
       </c>
-      <c r="F82" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="G82" s="6" t="s">
-        <v>283</v>
-      </c>
-      <c r="H82" s="6" t="s">
-        <v>283</v>
-      </c>
-      <c r="I82" s="5">
-        <v>46111</v>
-      </c>
-      <c r="J82" s="5">
-        <v>46128</v>
-      </c>
-      <c r="K82" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="L82" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="M82" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="N82" s="6" t="s">
-        <v>279</v>
-      </c>
-      <c r="O82" s="6" t="s">
-        <v>255</v>
-      </c>
-      <c r="P82" s="6" t="s">
-        <v>284</v>
-      </c>
       <c r="Q82" s="5">
-        <v>46111</v>
+        <v>46129</v>
       </c>
       <c r="R82" s="5">
-        <v>46119</v>
+        <v>46132</v>
       </c>
       <c r="S82" s="10" t="s">
         <v>31</v>
@@ -6460,32 +6433,32 @@
     </row>
     <row r="83" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A83" s="7" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="B83" s="8">
-        <v>46073.69994784722</v>
+        <v>46073.69994864584</v>
       </c>
       <c r="C83" s="9"/>
       <c r="D83" s="8">
-        <v>46198.59349042824</v>
+        <v>46153.16811694445</v>
       </c>
       <c r="E83" s="9" t="s">
-        <v>286</v>
+        <v>230</v>
       </c>
       <c r="F83" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G83" s="9" t="s">
-        <v>283</v>
+        <v>266</v>
       </c>
       <c r="H83" s="9" t="s">
-        <v>283</v>
+        <v>266</v>
       </c>
       <c r="I83" s="8">
-        <v>46149</v>
+        <v>46153</v>
       </c>
       <c r="J83" s="8">
-        <v>46150</v>
+        <v>46153</v>
       </c>
       <c r="K83" s="9" t="s">
         <v>26</v>
@@ -6497,19 +6470,19 @@
         <v>26</v>
       </c>
       <c r="N83" s="9" t="s">
-        <v>279</v>
+        <v>263</v>
       </c>
       <c r="O83" s="9" t="s">
-        <v>287</v>
+        <v>284</v>
       </c>
       <c r="P83" s="9" t="s">
-        <v>288</v>
+        <v>285</v>
       </c>
       <c r="Q83" s="8">
-        <v>46149</v>
+        <v>46153</v>
       </c>
       <c r="R83" s="8">
-        <v>46150</v>
+        <v>46153</v>
       </c>
       <c r="S83" s="11" t="s">
         <v>128</v>
@@ -6523,32 +6496,32 @@
     </row>
     <row r="84" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A84" s="4" t="s">
-        <v>289</v>
+        <v>286</v>
       </c>
       <c r="B84" s="5">
-        <v>46073.69994813658</v>
+        <v>46073.699948912035</v>
       </c>
       <c r="C84" s="6"/>
       <c r="D84" s="5">
-        <v>46198.592367060184</v>
+        <v>46154.16785564815</v>
       </c>
       <c r="E84" s="6" t="s">
-        <v>290</v>
+        <v>287</v>
       </c>
       <c r="F84" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G84" s="6" t="s">
-        <v>283</v>
+        <v>266</v>
       </c>
       <c r="H84" s="6" t="s">
-        <v>283</v>
+        <v>266</v>
       </c>
       <c r="I84" s="5">
-        <v>46134</v>
+        <v>46154</v>
       </c>
       <c r="J84" s="5">
-        <v>46135</v>
+        <v>46154</v>
       </c>
       <c r="K84" s="6" t="s">
         <v>26</v>
@@ -6560,22 +6533,22 @@
         <v>26</v>
       </c>
       <c r="N84" s="6" t="s">
-        <v>279</v>
+        <v>263</v>
       </c>
       <c r="O84" s="6" t="s">
-        <v>291</v>
+        <v>227</v>
       </c>
       <c r="P84" s="6" t="s">
         <v>288</v>
       </c>
       <c r="Q84" s="5">
-        <v>46134</v>
+        <v>46154</v>
       </c>
       <c r="R84" s="5">
-        <v>46135</v>
-      </c>
-      <c r="S84" s="10" t="s">
-        <v>31</v>
+        <v>46154</v>
+      </c>
+      <c r="S84" s="11" t="s">
+        <v>128</v>
       </c>
       <c r="T84" s="6">
         <v>0</v>
@@ -6586,33 +6559,27 @@
     </row>
     <row r="85" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A85" s="7" t="s">
-        <v>292</v>
+        <v>289</v>
       </c>
       <c r="B85" s="8">
-        <v>46073.699948368056</v>
+        <v>46073.69994572917</v>
       </c>
       <c r="C85" s="9"/>
       <c r="D85" s="8">
-        <v>46198.59272494213</v>
+        <v>46077.638347245374</v>
       </c>
       <c r="E85" s="9" t="s">
-        <v>293</v>
+        <v>290</v>
       </c>
       <c r="F85" s="9" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="G85" s="9" t="s">
-        <v>283</v>
-      </c>
-      <c r="H85" s="9" t="s">
-        <v>283</v>
-      </c>
-      <c r="I85" s="8">
-        <v>46136</v>
-      </c>
-      <c r="J85" s="8">
-        <v>46139</v>
-      </c>
+        <v>26</v>
+      </c>
+      <c r="H85" s="9"/>
+      <c r="I85" s="9"/>
+      <c r="J85" s="9"/>
       <c r="K85" s="9" t="s">
         <v>26</v>
       </c>
@@ -6620,61 +6587,51 @@
         <v>26</v>
       </c>
       <c r="M85" s="9" t="s">
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="N85" s="9" t="s">
-        <v>279</v>
+        <v>26</v>
       </c>
       <c r="O85" s="9" t="s">
-        <v>294</v>
+        <v>291</v>
       </c>
       <c r="P85" s="9" t="s">
-        <v>288</v>
-      </c>
-      <c r="Q85" s="8">
-        <v>46136</v>
-      </c>
-      <c r="R85" s="8">
-        <v>46139</v>
-      </c>
-      <c r="S85" s="12" t="s">
-        <v>295</v>
-      </c>
-      <c r="T85" s="9">
-        <v>0.5</v>
-      </c>
-      <c r="U85" s="10" t="s">
-        <v>58</v>
-      </c>
+        <v>26</v>
+      </c>
+      <c r="Q85" s="9"/>
+      <c r="R85" s="9"/>
+      <c r="S85" s="9"/>
+      <c r="T85" s="9"/>
+      <c r="U85" s="9"/>
     </row>
     <row r="86" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A86" s="4" t="s">
-        <v>296</v>
+        <v>292</v>
       </c>
       <c r="B86" s="5">
-        <v>46076.88137268518</v>
+        <v>46073.699946099536</v>
       </c>
       <c r="C86" s="6"/>
       <c r="D86" s="5">
-        <v>46195.60422616898</v>
+        <v>46210.60325569444</v>
       </c>
       <c r="E86" s="6" t="s">
-        <v>297</v>
+        <v>293</v>
       </c>
       <c r="F86" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G86" s="6" t="s">
-        <v>283</v>
+        <v>294</v>
       </c>
       <c r="H86" s="6" t="s">
-        <v>283</v>
+        <v>295</v>
       </c>
       <c r="I86" s="5">
-        <v>46129</v>
+        <v>46155</v>
       </c>
       <c r="J86" s="5">
-        <v>46132</v>
+        <v>46155</v>
       </c>
       <c r="K86" s="6" t="s">
         <v>26</v>
@@ -6686,22 +6643,22 @@
         <v>26</v>
       </c>
       <c r="N86" s="6" t="s">
-        <v>279</v>
+        <v>290</v>
       </c>
       <c r="O86" s="6" t="s">
-        <v>298</v>
+        <v>287</v>
       </c>
       <c r="P86" s="6" t="s">
-        <v>299</v>
+        <v>296</v>
       </c>
       <c r="Q86" s="5">
-        <v>46129</v>
+        <v>46155</v>
       </c>
       <c r="R86" s="5">
-        <v>46132</v>
-      </c>
-      <c r="S86" s="10" t="s">
-        <v>31</v>
+        <v>46155</v>
+      </c>
+      <c r="S86" s="11" t="s">
+        <v>128</v>
       </c>
       <c r="T86" s="6">
         <v>0</v>
@@ -6712,32 +6669,32 @@
     </row>
     <row r="87" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A87" s="7" t="s">
-        <v>300</v>
+        <v>297</v>
       </c>
       <c r="B87" s="8">
-        <v>46073.69994864584</v>
+        <v>46073.69994638889</v>
       </c>
       <c r="C87" s="9"/>
       <c r="D87" s="8">
-        <v>46153.16811694445</v>
+        <v>46195.604670092594</v>
       </c>
       <c r="E87" s="9" t="s">
-        <v>229</v>
+        <v>260</v>
       </c>
       <c r="F87" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G87" s="9" t="s">
-        <v>283</v>
+        <v>266</v>
       </c>
       <c r="H87" s="9" t="s">
-        <v>283</v>
+        <v>266</v>
       </c>
       <c r="I87" s="8">
-        <v>46153</v>
+        <v>46156</v>
       </c>
       <c r="J87" s="8">
-        <v>46153</v>
+        <v>46160</v>
       </c>
       <c r="K87" s="9" t="s">
         <v>26</v>
@@ -6749,19 +6706,19 @@
         <v>26</v>
       </c>
       <c r="N87" s="9" t="s">
-        <v>279</v>
+        <v>290</v>
       </c>
       <c r="O87" s="9" t="s">
-        <v>301</v>
+        <v>298</v>
       </c>
       <c r="P87" s="9" t="s">
-        <v>302</v>
+        <v>299</v>
       </c>
       <c r="Q87" s="8">
-        <v>46153</v>
+        <v>46156</v>
       </c>
       <c r="R87" s="8">
-        <v>46153</v>
+        <v>46160</v>
       </c>
       <c r="S87" s="11" t="s">
         <v>128</v>
@@ -6775,56 +6732,56 @@
     </row>
     <row r="88" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A88" s="4" t="s">
-        <v>303</v>
+        <v>300</v>
       </c>
       <c r="B88" s="5">
-        <v>46073.699948912035</v>
+        <v>46073.69994668981</v>
       </c>
       <c r="C88" s="6"/>
       <c r="D88" s="5">
-        <v>46154.16785564815</v>
+        <v>46161.25032122685</v>
       </c>
       <c r="E88" s="6" t="s">
+        <v>301</v>
+      </c>
+      <c r="F88" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="G88" s="6" t="s">
+        <v>302</v>
+      </c>
+      <c r="H88" s="6" t="s">
+        <v>303</v>
+      </c>
+      <c r="I88" s="5">
+        <v>46161</v>
+      </c>
+      <c r="J88" s="5">
+        <v>46161</v>
+      </c>
+      <c r="K88" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="L88" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="M88" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="N88" s="6" t="s">
+        <v>290</v>
+      </c>
+      <c r="O88" s="6" t="s">
+        <v>260</v>
+      </c>
+      <c r="P88" s="6" t="s">
         <v>304</v>
       </c>
-      <c r="F88" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="G88" s="6" t="s">
-        <v>283</v>
-      </c>
-      <c r="H88" s="6" t="s">
-        <v>283</v>
-      </c>
-      <c r="I88" s="5">
-        <v>46154</v>
-      </c>
-      <c r="J88" s="5">
-        <v>46154</v>
-      </c>
-      <c r="K88" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="L88" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="M88" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="N88" s="6" t="s">
-        <v>279</v>
-      </c>
-      <c r="O88" s="6" t="s">
-        <v>226</v>
-      </c>
-      <c r="P88" s="6" t="s">
-        <v>305</v>
-      </c>
       <c r="Q88" s="5">
-        <v>46154</v>
+        <v>46161</v>
       </c>
       <c r="R88" s="5">
-        <v>46154</v>
+        <v>46161</v>
       </c>
       <c r="S88" s="11" t="s">
         <v>128</v>
@@ -6838,142 +6795,142 @@
     </row>
     <row r="89" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A89" s="7" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="B89" s="8">
-        <v>46073.69994572917</v>
+        <v>46073.69994695602</v>
       </c>
       <c r="C89" s="9"/>
       <c r="D89" s="8">
-        <v>46077.638347245374</v>
+        <v>46162.25040996527</v>
       </c>
       <c r="E89" s="9" t="s">
+        <v>306</v>
+      </c>
+      <c r="F89" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="G89" s="9" t="s">
+        <v>302</v>
+      </c>
+      <c r="H89" s="9" t="s">
+        <v>303</v>
+      </c>
+      <c r="I89" s="8">
+        <v>46162</v>
+      </c>
+      <c r="J89" s="8">
+        <v>46162</v>
+      </c>
+      <c r="K89" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="L89" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="M89" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="N89" s="9" t="s">
+        <v>290</v>
+      </c>
+      <c r="O89" s="9" t="s">
+        <v>301</v>
+      </c>
+      <c r="P89" s="9" t="s">
         <v>307</v>
       </c>
-      <c r="F89" s="9" t="s">
-        <v>25</v>
-      </c>
-      <c r="G89" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="H89" s="9"/>
-      <c r="I89" s="9"/>
-      <c r="J89" s="9"/>
-      <c r="K89" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="L89" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="M89" s="9" t="s">
+      <c r="Q89" s="8">
+        <v>46162</v>
+      </c>
+      <c r="R89" s="8">
+        <v>46162</v>
+      </c>
+      <c r="S89" s="11" t="s">
+        <v>128</v>
+      </c>
+      <c r="T89" s="9">
         <v>0</v>
       </c>
-      <c r="N89" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="O89" s="9" t="s">
-        <v>308</v>
-      </c>
-      <c r="P89" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="Q89" s="9"/>
-      <c r="R89" s="9"/>
-      <c r="S89" s="9"/>
-      <c r="T89" s="9"/>
-      <c r="U89" s="9"/>
+      <c r="U89" s="10" t="s">
+        <v>58</v>
+      </c>
     </row>
     <row r="90" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A90" s="4" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="B90" s="5">
-        <v>46073.699946099536</v>
+        <v>46073.699947245375</v>
       </c>
       <c r="C90" s="6"/>
       <c r="D90" s="5">
-        <v>46210.60325569444</v>
+        <v>46077.6387968287</v>
       </c>
       <c r="E90" s="6" t="s">
+        <v>309</v>
+      </c>
+      <c r="F90" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="G90" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="H90" s="6"/>
+      <c r="I90" s="6"/>
+      <c r="J90" s="6"/>
+      <c r="K90" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="L90" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="M90" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="N90" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="O90" s="6" t="s">
         <v>310</v>
       </c>
-      <c r="F90" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="G90" s="6" t="s">
-        <v>311</v>
-      </c>
-      <c r="H90" s="6" t="s">
-        <v>312</v>
-      </c>
-      <c r="I90" s="5">
-        <v>46155</v>
-      </c>
-      <c r="J90" s="5">
-        <v>46155</v>
-      </c>
-      <c r="K90" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="L90" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="M90" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="N90" s="6" t="s">
-        <v>307</v>
-      </c>
-      <c r="O90" s="6" t="s">
-        <v>304</v>
-      </c>
       <c r="P90" s="6" t="s">
-        <v>313</v>
-      </c>
-      <c r="Q90" s="5">
-        <v>46155</v>
-      </c>
-      <c r="R90" s="5">
-        <v>46155</v>
-      </c>
-      <c r="S90" s="11" t="s">
-        <v>128</v>
-      </c>
-      <c r="T90" s="6">
-        <v>0</v>
-      </c>
-      <c r="U90" s="10" t="s">
-        <v>58</v>
-      </c>
+        <v>26</v>
+      </c>
+      <c r="Q90" s="6"/>
+      <c r="R90" s="6"/>
+      <c r="S90" s="6"/>
+      <c r="T90" s="6"/>
+      <c r="U90" s="6"/>
     </row>
     <row r="91" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A91" s="7" t="s">
-        <v>314</v>
+        <v>311</v>
       </c>
       <c r="B91" s="8">
-        <v>46073.69994638889</v>
+        <v>46073.699947500005</v>
       </c>
       <c r="C91" s="9"/>
       <c r="D91" s="8">
-        <v>46195.604670092594</v>
+        <v>46174.16833755787</v>
       </c>
       <c r="E91" s="9" t="s">
-        <v>276</v>
+        <v>312</v>
       </c>
       <c r="F91" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G91" s="9" t="s">
-        <v>283</v>
+        <v>313</v>
       </c>
       <c r="H91" s="9" t="s">
-        <v>283</v>
+        <v>314</v>
       </c>
       <c r="I91" s="8">
-        <v>46156</v>
+        <v>46164</v>
       </c>
       <c r="J91" s="8">
-        <v>46160</v>
+        <v>46174</v>
       </c>
       <c r="K91" s="9" t="s">
         <v>26</v>
@@ -6985,19 +6942,19 @@
         <v>26</v>
       </c>
       <c r="N91" s="9" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="O91" s="9" t="s">
-        <v>315</v>
+        <v>306</v>
       </c>
       <c r="P91" s="9" t="s">
-        <v>316</v>
+        <v>309</v>
       </c>
       <c r="Q91" s="8">
-        <v>46156</v>
+        <v>46164</v>
       </c>
       <c r="R91" s="8">
-        <v>46160</v>
+        <v>46174</v>
       </c>
       <c r="S91" s="11" t="s">
         <v>128</v>
@@ -7011,32 +6968,32 @@
     </row>
     <row r="92" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A92" s="4" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
       <c r="B92" s="5">
-        <v>46073.69994668981</v>
+        <v>46073.699947789355</v>
       </c>
       <c r="C92" s="6"/>
       <c r="D92" s="5">
-        <v>46161.25032122685</v>
+        <v>46174.168340185184</v>
       </c>
       <c r="E92" s="6" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
       <c r="F92" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G92" s="6" t="s">
-        <v>247</v>
+        <v>313</v>
       </c>
       <c r="H92" s="6" t="s">
-        <v>248</v>
+        <v>314</v>
       </c>
       <c r="I92" s="5">
-        <v>46161</v>
+        <v>46164</v>
       </c>
       <c r="J92" s="5">
-        <v>46161</v>
+        <v>46174</v>
       </c>
       <c r="K92" s="6" t="s">
         <v>26</v>
@@ -7048,19 +7005,19 @@
         <v>26</v>
       </c>
       <c r="N92" s="6" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="O92" s="6" t="s">
-        <v>276</v>
+        <v>317</v>
       </c>
       <c r="P92" s="6" t="s">
-        <v>319</v>
+        <v>309</v>
       </c>
       <c r="Q92" s="5">
-        <v>46161</v>
+        <v>46164</v>
       </c>
       <c r="R92" s="5">
-        <v>46161</v>
+        <v>46174</v>
       </c>
       <c r="S92" s="11" t="s">
         <v>128</v>
@@ -7074,33 +7031,27 @@
     </row>
     <row r="93" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A93" s="7" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="B93" s="8">
-        <v>46073.69994695602</v>
+        <v>46092.48971385417</v>
       </c>
       <c r="C93" s="9"/>
       <c r="D93" s="8">
-        <v>46162.25040996527</v>
+        <v>46092.497058946756</v>
       </c>
       <c r="E93" s="9" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
       <c r="F93" s="9" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="G93" s="9" t="s">
-        <v>247</v>
-      </c>
-      <c r="H93" s="9" t="s">
-        <v>248</v>
-      </c>
-      <c r="I93" s="8">
-        <v>46162</v>
-      </c>
-      <c r="J93" s="8">
-        <v>46162</v>
-      </c>
+        <v>26</v>
+      </c>
+      <c r="H93" s="9"/>
+      <c r="I93" s="9"/>
+      <c r="J93" s="9"/>
       <c r="K93" s="9" t="s">
         <v>26</v>
       </c>
@@ -7108,23 +7059,19 @@
         <v>26</v>
       </c>
       <c r="M93" s="9" t="s">
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="N93" s="9" t="s">
-        <v>307</v>
+        <v>26</v>
       </c>
       <c r="O93" s="9" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="P93" s="9" t="s">
-        <v>322</v>
-      </c>
-      <c r="Q93" s="8">
-        <v>46162</v>
-      </c>
-      <c r="R93" s="8">
-        <v>46162</v>
-      </c>
+        <v>26</v>
+      </c>
+      <c r="Q93" s="9"/>
+      <c r="R93" s="9"/>
       <c r="S93" s="11" t="s">
         <v>128</v>
       </c>
@@ -7137,27 +7084,33 @@
     </row>
     <row r="94" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A94" s="4" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
       <c r="B94" s="5">
-        <v>46073.699947245375</v>
+        <v>46092.49161491898</v>
       </c>
       <c r="C94" s="6"/>
       <c r="D94" s="5">
-        <v>46077.6387968287</v>
+        <v>46171.168742951384</v>
       </c>
       <c r="E94" s="6" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="F94" s="6" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G94" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="H94" s="6"/>
-      <c r="I94" s="6"/>
-      <c r="J94" s="6"/>
+        <v>49</v>
+      </c>
+      <c r="H94" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="I94" s="5">
+        <v>46164</v>
+      </c>
+      <c r="J94" s="5">
+        <v>46171</v>
+      </c>
       <c r="K94" s="6" t="s">
         <v>26</v>
       </c>
@@ -7165,75 +7118,85 @@
         <v>26</v>
       </c>
       <c r="M94" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="N94" s="6" t="s">
+        <v>319</v>
+      </c>
+      <c r="O94" s="6" t="s">
+        <v>306</v>
+      </c>
+      <c r="P94" s="6" t="s">
+        <v>323</v>
+      </c>
+      <c r="Q94" s="5">
+        <v>46164</v>
+      </c>
+      <c r="R94" s="5">
+        <v>46171</v>
+      </c>
+      <c r="S94" s="11" t="s">
+        <v>128</v>
+      </c>
+      <c r="T94" s="6">
         <v>0</v>
       </c>
-      <c r="N94" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="O94" s="6" t="s">
-        <v>325</v>
-      </c>
-      <c r="P94" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="Q94" s="6"/>
-      <c r="R94" s="6"/>
-      <c r="S94" s="6"/>
-      <c r="T94" s="6"/>
-      <c r="U94" s="6"/>
+      <c r="U94" s="10" t="s">
+        <v>58</v>
+      </c>
     </row>
     <row r="95" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A95" s="7" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="B95" s="8">
-        <v>46073.699947500005</v>
+        <v>46092.491661747685</v>
       </c>
       <c r="C95" s="9"/>
       <c r="D95" s="8">
-        <v>46174.16833755787</v>
+        <v>46181.16820616898</v>
       </c>
       <c r="E95" s="9" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="F95" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G95" s="9" t="s">
-        <v>328</v>
+        <v>49</v>
       </c>
       <c r="H95" s="9" t="s">
-        <v>329</v>
+        <v>50</v>
       </c>
       <c r="I95" s="8">
-        <v>46164</v>
+        <v>46174</v>
       </c>
       <c r="J95" s="8">
+        <v>46181</v>
+      </c>
+      <c r="K95" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="L95" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="M95" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="N95" s="9" t="s">
+        <v>319</v>
+      </c>
+      <c r="O95" s="9" t="s">
+        <v>322</v>
+      </c>
+      <c r="P95" s="9" t="s">
+        <v>319</v>
+      </c>
+      <c r="Q95" s="8">
         <v>46174</v>
       </c>
-      <c r="K95" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="L95" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="M95" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="N95" s="9" t="s">
-        <v>324</v>
-      </c>
-      <c r="O95" s="9" t="s">
-        <v>321</v>
-      </c>
-      <c r="P95" s="9" t="s">
-        <v>324</v>
-      </c>
-      <c r="Q95" s="8">
-        <v>46164</v>
-      </c>
       <c r="R95" s="8">
-        <v>46174</v>
+        <v>46181</v>
       </c>
       <c r="S95" s="11" t="s">
         <v>128</v>
@@ -7242,248 +7205,6 @@
         <v>0</v>
       </c>
       <c r="U95" s="10" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="96" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A96" s="4" t="s">
-        <v>330</v>
-      </c>
-      <c r="B96" s="5">
-        <v>46073.699947789355</v>
-      </c>
-      <c r="C96" s="6"/>
-      <c r="D96" s="5">
-        <v>46174.168340185184</v>
-      </c>
-      <c r="E96" s="6" t="s">
-        <v>331</v>
-      </c>
-      <c r="F96" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="G96" s="6" t="s">
-        <v>328</v>
-      </c>
-      <c r="H96" s="6" t="s">
-        <v>329</v>
-      </c>
-      <c r="I96" s="5">
-        <v>46164</v>
-      </c>
-      <c r="J96" s="5">
-        <v>46174</v>
-      </c>
-      <c r="K96" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="L96" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="M96" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="N96" s="6" t="s">
-        <v>324</v>
-      </c>
-      <c r="O96" s="6" t="s">
-        <v>332</v>
-      </c>
-      <c r="P96" s="6" t="s">
-        <v>324</v>
-      </c>
-      <c r="Q96" s="5">
-        <v>46164</v>
-      </c>
-      <c r="R96" s="5">
-        <v>46174</v>
-      </c>
-      <c r="S96" s="11" t="s">
-        <v>128</v>
-      </c>
-      <c r="T96" s="6">
-        <v>0</v>
-      </c>
-      <c r="U96" s="10" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="97" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A97" s="7" t="s">
-        <v>333</v>
-      </c>
-      <c r="B97" s="8">
-        <v>46092.48971385417</v>
-      </c>
-      <c r="C97" s="9"/>
-      <c r="D97" s="8">
-        <v>46092.497058946756</v>
-      </c>
-      <c r="E97" s="9" t="s">
-        <v>334</v>
-      </c>
-      <c r="F97" s="9" t="s">
-        <v>25</v>
-      </c>
-      <c r="G97" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="H97" s="9"/>
-      <c r="I97" s="9"/>
-      <c r="J97" s="9"/>
-      <c r="K97" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="L97" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="M97" s="9" t="s">
-        <v>0</v>
-      </c>
-      <c r="N97" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="O97" s="9" t="s">
-        <v>335</v>
-      </c>
-      <c r="P97" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="Q97" s="9"/>
-      <c r="R97" s="9"/>
-      <c r="S97" s="11" t="s">
-        <v>128</v>
-      </c>
-      <c r="T97" s="9">
-        <v>0</v>
-      </c>
-      <c r="U97" s="10" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="98" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A98" s="4" t="s">
-        <v>336</v>
-      </c>
-      <c r="B98" s="5">
-        <v>46092.49161491898</v>
-      </c>
-      <c r="C98" s="6"/>
-      <c r="D98" s="5">
-        <v>46171.168742951384</v>
-      </c>
-      <c r="E98" s="6" t="s">
-        <v>337</v>
-      </c>
-      <c r="F98" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="G98" s="6" t="s">
-        <v>49</v>
-      </c>
-      <c r="H98" s="6" t="s">
-        <v>50</v>
-      </c>
-      <c r="I98" s="5">
-        <v>46164</v>
-      </c>
-      <c r="J98" s="5">
-        <v>46171</v>
-      </c>
-      <c r="K98" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="L98" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="M98" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="N98" s="6" t="s">
-        <v>334</v>
-      </c>
-      <c r="O98" s="6" t="s">
-        <v>321</v>
-      </c>
-      <c r="P98" s="6" t="s">
-        <v>338</v>
-      </c>
-      <c r="Q98" s="5">
-        <v>46164</v>
-      </c>
-      <c r="R98" s="5">
-        <v>46171</v>
-      </c>
-      <c r="S98" s="11" t="s">
-        <v>128</v>
-      </c>
-      <c r="T98" s="6">
-        <v>0</v>
-      </c>
-      <c r="U98" s="10" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="99" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A99" s="7" t="s">
-        <v>339</v>
-      </c>
-      <c r="B99" s="8">
-        <v>46092.491661747685</v>
-      </c>
-      <c r="C99" s="9"/>
-      <c r="D99" s="8">
-        <v>46181.16820616898</v>
-      </c>
-      <c r="E99" s="9" t="s">
-        <v>340</v>
-      </c>
-      <c r="F99" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="G99" s="9" t="s">
-        <v>49</v>
-      </c>
-      <c r="H99" s="9" t="s">
-        <v>50</v>
-      </c>
-      <c r="I99" s="8">
-        <v>46174</v>
-      </c>
-      <c r="J99" s="8">
-        <v>46181</v>
-      </c>
-      <c r="K99" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="L99" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="M99" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="N99" s="9" t="s">
-        <v>334</v>
-      </c>
-      <c r="O99" s="9" t="s">
-        <v>337</v>
-      </c>
-      <c r="P99" s="9" t="s">
-        <v>334</v>
-      </c>
-      <c r="Q99" s="8">
-        <v>46174</v>
-      </c>
-      <c r="R99" s="8">
-        <v>46181</v>
-      </c>
-      <c r="S99" s="11" t="s">
-        <v>128</v>
-      </c>
-      <c r="T99" s="9">
-        <v>0</v>
-      </c>
-      <c r="U99" s="10" t="s">
         <v>58</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualiza portafolio 2026-07-10 15:02 UTC
</commit_message>
<xml_diff>
--- a/data/50001490 - ZITRON PERU METRO LIMA PV04-PV05.xlsx
+++ b/data/50001490 - ZITRON PERU METRO LIMA PV04-PV05.xlsx
@@ -5584,7 +5584,7 @@
       </c>
       <c r="C69" s="9"/>
       <c r="D69" s="8">
-        <v>46195.604225717594</v>
+        <v>46213.56641354167</v>
       </c>
       <c r="E69" s="9" t="s">
         <v>233</v>
@@ -5631,7 +5631,7 @@
       </c>
       <c r="C70" s="6"/>
       <c r="D70" s="5">
-        <v>46199.830143969906</v>
+        <v>46213.56641027778</v>
       </c>
       <c r="E70" s="6" t="s">
         <v>245</v>
@@ -6314,7 +6314,7 @@
       </c>
       <c r="C81" s="9"/>
       <c r="D81" s="8">
-        <v>46198.59272494213</v>
+        <v>46213.56641375</v>
       </c>
       <c r="E81" s="9" t="s">
         <v>276</v>

</xml_diff>

<commit_message>
Actualiza portafolio 2026-07-10 18:39 UTC
</commit_message>
<xml_diff>
--- a/data/50001490 - ZITRON PERU METRO LIMA PV04-PV05.xlsx
+++ b/data/50001490 - ZITRON PERU METRO LIMA PV04-PV05.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1169" uniqueCount="326">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1169" uniqueCount="327">
   <si>
     <t xml:space="preserve">50001490-ZITRON PERU METRO DE LIMA PV04-PV05 </t>
   </si>
@@ -134,6 +134,9 @@
   </si>
   <si>
     <t>Definicion Tecnica de componentes principales</t>
+  </si>
+  <si>
+    <t>ZVR-1-22-90/6 (W22 Carcasa de Hierro Gris) MOTOR (2) 90 KW – 06 POLOS – 380 V -60 HZ- 1000 msnm. Resistente al fuego 250°C / 2 horas Sentido de giro bidireccional Frame: 250 Forma constructiva: B3T Protección: IP55 Refrigeración: TEFC Calentamiento: CLASE B Servicio: S1 Factor de Servicio: 1,15 Rendimiento: IE1 Aislamiento: clase H Arranque: VDF Caja de bornes en el exterior del ventilador Sondas: Sondas de temperatura PTC en los devanados Sondas de temperatura PTC 100 en cojinetes Sonda Stall (anti-bombeo) (Directo e inverso) Sonda de caudal (Directo e inverso) Sonda de vibraciones Sonda de rodamientos PT100 PT100 de temperatura de aire ZVRv-1-22-90/6 (W22 Carcasa de Hierro Gris) MOTOR (2) 90 KW – 06 POLOS – 380 V -60 HZ- 1000 msnm. Resistente al fuego 250°C / 2 horas Sentido de giro bidireccional Frame: 250 Forma constructiva: B3T Protección: IP55.</t>
   </si>
   <si>
     <t>Ingenieria electrica,Ingenieria Basica Motor,Ingenieria Basica Alabes,Ingenieria basica Rodete,Ingenieria Detalle,Ingenieria Basica Damper , Ingenieria basica atenuador</t>
@@ -1865,7 +1868,7 @@
         <v>46092.71883331018</v>
       </c>
       <c r="D8" s="5">
-        <v>46093.75450768518</v>
+        <v>46213.75870287037</v>
       </c>
       <c r="E8" s="6" t="s">
         <v>40</v>
@@ -1889,7 +1892,7 @@
         <v>26</v>
       </c>
       <c r="L8" s="6" t="s">
-        <v>26</v>
+        <v>41</v>
       </c>
       <c r="M8" s="6" t="s">
         <v>26</v>
@@ -1901,7 +1904,7 @@
         <v>26</v>
       </c>
       <c r="P8" s="6" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="Q8" s="5">
         <v>45993</v>
@@ -1921,7 +1924,7 @@
     </row>
     <row r="9" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A9" s="7" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B9" s="8">
         <v>46073.69994784722</v>
@@ -1933,7 +1936,7 @@
         <v>46092.71886530092</v>
       </c>
       <c r="E9" s="9" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="F9" s="9" t="s">
         <v>26</v>
@@ -1986,7 +1989,7 @@
     </row>
     <row r="10" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B10" s="5">
         <v>46073.699948124995</v>
@@ -1996,7 +1999,7 @@
         <v>46127.89302402778</v>
       </c>
       <c r="E10" s="6" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="F10" s="6" t="s">
         <v>25</v>
@@ -2020,7 +2023,7 @@
         <v>26</v>
       </c>
       <c r="O10" s="6" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="P10" s="6" t="s">
         <v>26</v>
@@ -2033,7 +2036,7 @@
     </row>
     <row r="11" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A11" s="7" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B11" s="8">
         <v>46073.699948379624</v>
@@ -2045,16 +2048,16 @@
         <v>46093.86157599537</v>
       </c>
       <c r="E11" s="9" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="F11" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G11" s="9" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="H11" s="9" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="I11" s="8">
         <v>45994</v>
@@ -2072,13 +2075,13 @@
         <v>26</v>
       </c>
       <c r="N11" s="9" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="O11" s="9" t="s">
         <v>40</v>
       </c>
       <c r="P11" s="9" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="Q11" s="8">
         <v>45994</v>
@@ -2098,7 +2101,7 @@
     </row>
     <row r="12" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A12" s="4" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B12" s="5">
         <v>46073.69994864584</v>
@@ -2108,16 +2111,16 @@
         <v>46134.69385214121</v>
       </c>
       <c r="E12" s="6" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="F12" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G12" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="H12" s="6" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="I12" s="5">
         <v>46121</v>
@@ -2135,13 +2138,13 @@
         <v>26</v>
       </c>
       <c r="N12" s="6" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="O12" s="6" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="P12" s="6" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="Q12" s="5">
         <v>46121</v>
@@ -2156,12 +2159,12 @@
         <v>0</v>
       </c>
       <c r="U12" s="10" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="13" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A13" s="7" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B13" s="8">
         <v>46073.69994892361</v>
@@ -2173,7 +2176,7 @@
         <v>46093.7548365625</v>
       </c>
       <c r="E13" s="9" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="F13" s="9" t="s">
         <v>25</v>
@@ -2197,7 +2200,7 @@
         <v>26</v>
       </c>
       <c r="O13" s="9" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="P13" s="9" t="s">
         <v>26</v>
@@ -2214,7 +2217,7 @@
     </row>
     <row r="14" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A14" s="4" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B14" s="5">
         <v>46073.69994622685</v>
@@ -2226,16 +2229,16 @@
         <v>46093.754690856484</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="F14" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G14" s="6" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="H14" s="6" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="I14" s="5">
         <v>45994</v>
@@ -2253,13 +2256,13 @@
         <v>26</v>
       </c>
       <c r="N14" s="6" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="O14" s="6" t="s">
         <v>40</v>
       </c>
       <c r="P14" s="6" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="Q14" s="5">
         <v>45994</v>
@@ -2279,7 +2282,7 @@
     </row>
     <row r="15" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A15" s="7" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B15" s="8">
         <v>46073.6999465625</v>
@@ -2291,16 +2294,16 @@
         <v>46093.75469819445</v>
       </c>
       <c r="E15" s="9" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="F15" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G15" s="9" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="H15" s="9" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="I15" s="8">
         <v>45994</v>
@@ -2318,13 +2321,13 @@
         <v>26</v>
       </c>
       <c r="N15" s="9" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="O15" s="9" t="s">
         <v>40</v>
       </c>
       <c r="P15" s="9" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="Q15" s="8">
         <v>45994</v>
@@ -2344,7 +2347,7 @@
     </row>
     <row r="16" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A16" s="4" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B16" s="5">
         <v>46073.69994685185</v>
@@ -2356,16 +2359,16 @@
         <v>46093.75471203704</v>
       </c>
       <c r="E16" s="6" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="F16" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G16" s="6" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="H16" s="6" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="I16" s="5">
         <v>45994</v>
@@ -2383,13 +2386,13 @@
         <v>26</v>
       </c>
       <c r="N16" s="6" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="O16" s="6" t="s">
         <v>40</v>
       </c>
       <c r="P16" s="6" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="Q16" s="5">
         <v>45994</v>
@@ -2409,7 +2412,7 @@
     </row>
     <row r="17" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A17" s="7" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B17" s="8">
         <v>46073.69994711806</v>
@@ -2421,16 +2424,16 @@
         <v>46093.75472228009</v>
       </c>
       <c r="E17" s="9" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="F17" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G17" s="9" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="H17" s="9" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="I17" s="8">
         <v>45994</v>
@@ -2448,13 +2451,13 @@
         <v>26</v>
       </c>
       <c r="N17" s="9" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="O17" s="9" t="s">
         <v>40</v>
       </c>
       <c r="P17" s="9" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="Q17" s="8">
         <v>45994</v>
@@ -2474,7 +2477,7 @@
     </row>
     <row r="18" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A18" s="4" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B18" s="5">
         <v>46077.577641701384</v>
@@ -2486,16 +2489,16 @@
         <v>46093.7547315625</v>
       </c>
       <c r="E18" s="6" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="F18" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G18" s="6" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="H18" s="6" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="I18" s="5">
         <v>45994</v>
@@ -2513,13 +2516,13 @@
         <v>26</v>
       </c>
       <c r="N18" s="6" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="O18" s="6" t="s">
         <v>40</v>
       </c>
       <c r="P18" s="6" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="Q18" s="5">
         <v>45994</v>
@@ -2539,7 +2542,7 @@
     </row>
     <row r="19" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A19" s="7" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B19" s="8">
         <v>46077.57773309028</v>
@@ -2551,16 +2554,16 @@
         <v>46093.75474146991</v>
       </c>
       <c r="E19" s="9" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="F19" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G19" s="9" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="H19" s="9" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="I19" s="8">
         <v>45994</v>
@@ -2578,13 +2581,13 @@
         <v>26</v>
       </c>
       <c r="N19" s="9" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="O19" s="9" t="s">
         <v>40</v>
       </c>
       <c r="P19" s="9" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="Q19" s="8">
         <v>45994</v>
@@ -2604,7 +2607,7 @@
     </row>
     <row r="20" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A20" s="4" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B20" s="5">
         <v>46073.69994737269</v>
@@ -2616,16 +2619,16 @@
         <v>46093.75482354166</v>
       </c>
       <c r="E20" s="6" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="F20" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G20" s="6" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="H20" s="6" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="I20" s="5">
         <v>45994</v>
@@ -2643,13 +2646,13 @@
         <v>26</v>
       </c>
       <c r="N20" s="6" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="O20" s="6" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="P20" s="6" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="Q20" s="5">
         <v>45994</v>
@@ -2669,7 +2672,7 @@
     </row>
     <row r="21" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A21" s="7" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B21" s="8">
         <v>46073.69994763889</v>
@@ -2681,7 +2684,7 @@
         <v>46139.54278021991</v>
       </c>
       <c r="E21" s="9" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="F21" s="9" t="s">
         <v>25</v>
@@ -2705,7 +2708,7 @@
         <v>26</v>
       </c>
       <c r="O21" s="9" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="P21" s="9" t="s">
         <v>26</v>
@@ -2722,7 +2725,7 @@
     </row>
     <row r="22" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A22" s="4" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B22" s="5">
         <v>46073.6999481713</v>
@@ -2734,16 +2737,16 @@
         <v>46093.754786307865</v>
       </c>
       <c r="E22" s="6" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="F22" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G22" s="6" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="H22" s="6" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="I22" s="5">
         <v>45996</v>
@@ -2761,13 +2764,13 @@
         <v>26</v>
       </c>
       <c r="N22" s="6" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="O22" s="6" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="P22" s="6" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="Q22" s="5">
         <v>45996</v>
@@ -2787,7 +2790,7 @@
     </row>
     <row r="23" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A23" s="7" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B23" s="8">
         <v>46073.69994789352</v>
@@ -2799,16 +2802,16 @@
         <v>46093.75479849537</v>
       </c>
       <c r="E23" s="9" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="F23" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G23" s="9" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="H23" s="9" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="I23" s="8">
         <v>46003</v>
@@ -2826,13 +2829,13 @@
         <v>26</v>
       </c>
       <c r="N23" s="9" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="O23" s="9" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="P23" s="9" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="Q23" s="8">
         <v>46003</v>
@@ -2852,7 +2855,7 @@
     </row>
     <row r="24" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A24" s="4" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B24" s="5">
         <v>46073.69994854167</v>
@@ -2864,16 +2867,16 @@
         <v>46093.87454729166</v>
       </c>
       <c r="E24" s="6" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="F24" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G24" s="6" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="H24" s="6" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="I24" s="5">
         <v>45999</v>
@@ -2891,13 +2894,13 @@
         <v>26</v>
       </c>
       <c r="N24" s="6" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="O24" s="6" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="P24" s="6" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="Q24" s="5">
         <v>45999</v>
@@ -2917,7 +2920,7 @@
     </row>
     <row r="25" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A25" s="7" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B25" s="8">
         <v>46073.69994881944</v>
@@ -2929,16 +2932,16 @@
         <v>46093.754844745374</v>
       </c>
       <c r="E25" s="9" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="F25" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G25" s="9" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="H25" s="9" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="I25" s="8">
         <v>46003</v>
@@ -2956,13 +2959,13 @@
         <v>26</v>
       </c>
       <c r="N25" s="9" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="O25" s="9" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="P25" s="9" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="Q25" s="8">
         <v>46003</v>
@@ -2982,7 +2985,7 @@
     </row>
     <row r="26" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A26" s="4" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B26" s="5">
         <v>46073.699946319444</v>
@@ -2994,16 +2997,16 @@
         <v>46093.75485591435</v>
       </c>
       <c r="E26" s="6" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="F26" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G26" s="6" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="H26" s="6" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="I26" s="5">
         <v>46003</v>
@@ -3021,13 +3024,13 @@
         <v>26</v>
       </c>
       <c r="N26" s="6" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="O26" s="6" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="P26" s="6" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="Q26" s="5">
         <v>46003</v>
@@ -3047,7 +3050,7 @@
     </row>
     <row r="27" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A27" s="7" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B27" s="8">
         <v>46076.88102377315</v>
@@ -3059,16 +3062,16 @@
         <v>46093.754866759264</v>
       </c>
       <c r="E27" s="9" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="F27" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G27" s="9" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="H27" s="9" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="I27" s="8">
         <v>46003</v>
@@ -3086,13 +3089,13 @@
         <v>26</v>
       </c>
       <c r="N27" s="9" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="O27" s="9" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="P27" s="9" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="Q27" s="8">
         <v>46003</v>
@@ -3112,7 +3115,7 @@
     </row>
     <row r="28" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A28" s="4" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B28" s="5">
         <v>46077.579292766204</v>
@@ -3124,16 +3127,16 @@
         <v>46093.75487452546</v>
       </c>
       <c r="E28" s="6" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="F28" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G28" s="6" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="H28" s="6" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="I28" s="5">
         <v>46003</v>
@@ -3151,13 +3154,13 @@
         <v>26</v>
       </c>
       <c r="N28" s="6" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="O28" s="6" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="P28" s="6" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="Q28" s="5">
         <v>46003</v>
@@ -3177,7 +3180,7 @@
     </row>
     <row r="29" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A29" s="7" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B29" s="8">
         <v>46077.579365196754</v>
@@ -3189,16 +3192,16 @@
         <v>46093.75488136574</v>
       </c>
       <c r="E29" s="9" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="F29" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G29" s="9" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="H29" s="9" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="I29" s="8">
         <v>46003</v>
@@ -3216,13 +3219,13 @@
         <v>26</v>
       </c>
       <c r="N29" s="9" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="O29" s="9" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="P29" s="9" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="Q29" s="8">
         <v>46003</v>
@@ -3242,7 +3245,7 @@
     </row>
     <row r="30" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A30" s="4" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="B30" s="5">
         <v>46139.54271195602</v>
@@ -3254,16 +3257,16 @@
         <v>46139.548176979166</v>
       </c>
       <c r="E30" s="6" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="F30" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G30" s="6" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="H30" s="6" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="I30" s="5">
         <v>46136</v>
@@ -3281,13 +3284,13 @@
         <v>26</v>
       </c>
       <c r="N30" s="6" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="O30" s="6" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="P30" s="6" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="Q30" s="5">
         <v>46136</v>
@@ -3307,7 +3310,7 @@
     </row>
     <row r="31" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A31" s="7" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="B31" s="8">
         <v>46073.699946747685</v>
@@ -3317,7 +3320,7 @@
         <v>46191.83935533564</v>
       </c>
       <c r="E31" s="9" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="F31" s="9" t="s">
         <v>25</v>
@@ -3341,7 +3344,7 @@
         <v>26</v>
       </c>
       <c r="O31" s="9" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="P31" s="9" t="s">
         <v>26</v>
@@ -3354,7 +3357,7 @@
     </row>
     <row r="32" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A32" s="4" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="B32" s="5">
         <v>46073.69994704861</v>
@@ -3366,16 +3369,16 @@
         <v>46191.83935060185</v>
       </c>
       <c r="E32" s="6" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="F32" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G32" s="6" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="H32" s="6" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="I32" s="5">
         <v>46014</v>
@@ -3393,13 +3396,13 @@
         <v>26</v>
       </c>
       <c r="N32" s="6" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="O32" s="6" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="P32" s="6" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="Q32" s="5">
         <v>46014</v>
@@ -3414,12 +3417,12 @@
         <v>0</v>
       </c>
       <c r="U32" s="10" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="33" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A33" s="7" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="B33" s="8">
         <v>46073.69994738426</v>
@@ -3431,16 +3434,16 @@
         <v>46182.68413366898</v>
       </c>
       <c r="E33" s="9" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="F33" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G33" s="9" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="H33" s="9" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="I33" s="8">
         <v>46014</v>
@@ -3458,29 +3461,29 @@
         <v>26</v>
       </c>
       <c r="N33" s="9" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="O33" s="9" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="P33" s="9" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="Q33" s="9"/>
       <c r="R33" s="9"/>
       <c r="S33" s="11" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="T33" s="9">
         <v>0</v>
       </c>
       <c r="U33" s="10" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="34" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A34" s="4" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="B34" s="5">
         <v>46073.69994769676</v>
@@ -3492,16 +3495,16 @@
         <v>46191.83755358796</v>
       </c>
       <c r="E34" s="6" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="F34" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G34" s="6" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="H34" s="6" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="I34" s="5">
         <v>46017</v>
@@ -3519,29 +3522,29 @@
         <v>26</v>
       </c>
       <c r="N34" s="6" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="O34" s="6" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="P34" s="6" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="Q34" s="6"/>
       <c r="R34" s="6"/>
       <c r="S34" s="11" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="T34" s="6">
         <v>0</v>
       </c>
       <c r="U34" s="10" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="35" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A35" s="7" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="B35" s="8">
         <v>46073.69994803241</v>
@@ -3551,16 +3554,16 @@
         <v>46174.65273861111</v>
       </c>
       <c r="E35" s="9" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="F35" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G35" s="9" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="H35" s="9" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="I35" s="8">
         <v>46008</v>
@@ -3578,13 +3581,13 @@
         <v>26</v>
       </c>
       <c r="N35" s="9" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="O35" s="9" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="P35" s="9" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="Q35" s="8">
         <v>46008</v>
@@ -3599,12 +3602,12 @@
         <v>0.5</v>
       </c>
       <c r="U35" s="10" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="36" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A36" s="4" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="B36" s="5">
         <v>46073.699948333335</v>
@@ -3616,16 +3619,16 @@
         <v>46174.652731724535</v>
       </c>
       <c r="E36" s="6" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="F36" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G36" s="6" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="H36" s="6" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="I36" s="5">
         <v>46008</v>
@@ -3643,29 +3646,29 @@
         <v>26</v>
       </c>
       <c r="N36" s="6" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="O36" s="6" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="P36" s="6" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="Q36" s="6"/>
       <c r="R36" s="6"/>
       <c r="S36" s="11" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="T36" s="6">
         <v>0</v>
       </c>
       <c r="U36" s="10" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="37" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A37" s="7" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="B37" s="8">
         <v>46073.699948622685</v>
@@ -3675,16 +3678,16 @@
         <v>46174.65273809028</v>
       </c>
       <c r="E37" s="9" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="F37" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G37" s="9" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="H37" s="9" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="I37" s="8">
         <v>46020</v>
@@ -3702,29 +3705,29 @@
         <v>26</v>
       </c>
       <c r="N37" s="9" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="O37" s="9" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="P37" s="9" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="Q37" s="9"/>
       <c r="R37" s="9"/>
       <c r="S37" s="11" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="T37" s="9">
         <v>0</v>
       </c>
       <c r="U37" s="10" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="38" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A38" s="4" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="B38" s="5">
         <v>46073.69994892361</v>
@@ -3736,16 +3739,16 @@
         <v>46191.83671528935</v>
       </c>
       <c r="E38" s="6" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="F38" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G38" s="6" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="H38" s="6" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="I38" s="5">
         <v>46014</v>
@@ -3763,13 +3766,13 @@
         <v>26</v>
       </c>
       <c r="N38" s="6" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="O38" s="6" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="P38" s="6" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="Q38" s="5">
         <v>46014</v>
@@ -3784,12 +3787,12 @@
         <v>0</v>
       </c>
       <c r="U38" s="10" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="39" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A39" s="7" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="B39" s="8">
         <v>46073.699949201386</v>
@@ -3801,16 +3804,16 @@
         <v>46174.64929997685</v>
       </c>
       <c r="E39" s="9" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="F39" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G39" s="9" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="H39" s="9" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="I39" s="8">
         <v>46014</v>
@@ -3828,29 +3831,29 @@
         <v>26</v>
       </c>
       <c r="N39" s="9" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="O39" s="9" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="P39" s="9" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="Q39" s="9"/>
       <c r="R39" s="9"/>
       <c r="S39" s="11" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="T39" s="9">
         <v>0</v>
       </c>
       <c r="U39" s="10" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="40" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A40" s="4" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="B40" s="5">
         <v>46073.69994585648</v>
@@ -3862,16 +3865,16 @@
         <v>46182.67566810185</v>
       </c>
       <c r="E40" s="6" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="F40" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G40" s="6" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="H40" s="6" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="I40" s="5">
         <v>46017</v>
@@ -3889,29 +3892,29 @@
         <v>26</v>
       </c>
       <c r="N40" s="6" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="O40" s="6" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="P40" s="6" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="Q40" s="6"/>
       <c r="R40" s="6"/>
       <c r="S40" s="11" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="T40" s="6">
         <v>0</v>
       </c>
       <c r="U40" s="10" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="41" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A41" s="7" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="B41" s="8">
         <v>46073.69994628472</v>
@@ -3923,16 +3926,16 @@
         <v>46127.78344613426</v>
       </c>
       <c r="E41" s="9" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="F41" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G41" s="9" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="H41" s="9" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="I41" s="8">
         <v>46000</v>
@@ -3950,13 +3953,13 @@
         <v>26</v>
       </c>
       <c r="N41" s="9" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="O41" s="9" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="P41" s="9" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="Q41" s="8">
         <v>46000</v>
@@ -3965,7 +3968,7 @@
         <v>46147</v>
       </c>
       <c r="S41" s="11" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="T41" s="9">
         <v>1</v>
@@ -3976,7 +3979,7 @@
     </row>
     <row r="42" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A42" s="4" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="B42" s="5">
         <v>46073.69994653935</v>
@@ -3988,16 +3991,16 @@
         <v>46120.69255305556</v>
       </c>
       <c r="E42" s="6" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="F42" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G42" s="6" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="H42" s="6" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="I42" s="5">
         <v>46000</v>
@@ -4015,29 +4018,29 @@
         <v>26</v>
       </c>
       <c r="N42" s="6" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="O42" s="6" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="P42" s="6" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="Q42" s="6"/>
       <c r="R42" s="6"/>
       <c r="S42" s="11" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="T42" s="6">
         <v>0</v>
       </c>
       <c r="U42" s="10" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="43" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A43" s="7" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="B43" s="8">
         <v>46073.69994680556</v>
@@ -4049,16 +4052,16 @@
         <v>46127.783407256946</v>
       </c>
       <c r="E43" s="9" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="F43" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G43" s="9" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="H43" s="9" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="I43" s="8">
         <v>46020</v>
@@ -4076,29 +4079,29 @@
         <v>26</v>
       </c>
       <c r="N43" s="9" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="O43" s="9" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="P43" s="9" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="Q43" s="9"/>
       <c r="R43" s="9"/>
       <c r="S43" s="11" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="T43" s="9">
         <v>0</v>
       </c>
       <c r="U43" s="10" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="44" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A44" s="4" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="B44" s="5">
         <v>46073.69994707176</v>
@@ -4110,16 +4113,16 @@
         <v>46127.78341805555</v>
       </c>
       <c r="E44" s="6" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="F44" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G44" s="6" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="H44" s="6" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="I44" s="5">
         <v>46020</v>
@@ -4137,29 +4140,29 @@
         <v>26</v>
       </c>
       <c r="N44" s="6" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="O44" s="6" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="P44" s="6" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="Q44" s="6"/>
       <c r="R44" s="6"/>
       <c r="S44" s="11" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="T44" s="6">
         <v>0</v>
       </c>
       <c r="U44" s="10" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="45" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A45" s="7" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="B45" s="8">
         <v>46073.69994733796</v>
@@ -4171,16 +4174,16 @@
         <v>46139.54791172454</v>
       </c>
       <c r="E45" s="9" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="F45" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G45" s="9" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="H45" s="9" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="I45" s="8">
         <v>46014</v>
@@ -4198,13 +4201,13 @@
         <v>26</v>
       </c>
       <c r="N45" s="9" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="O45" s="9" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="P45" s="9" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="Q45" s="8">
         <v>46014</v>
@@ -4224,7 +4227,7 @@
     </row>
     <row r="46" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A46" s="4" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="B46" s="5">
         <v>46073.69994759259</v>
@@ -4236,16 +4239,16 @@
         <v>46104.82754626157</v>
       </c>
       <c r="E46" s="6" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="F46" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G46" s="6" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="H46" s="6" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="I46" s="5">
         <v>46014</v>
@@ -4263,29 +4266,29 @@
         <v>26</v>
       </c>
       <c r="N46" s="6" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="O46" s="6" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="P46" s="6" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="Q46" s="6"/>
       <c r="R46" s="6"/>
       <c r="S46" s="11" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="T46" s="6">
         <v>0</v>
       </c>
       <c r="U46" s="10" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="47" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A47" s="7" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="B47" s="8">
         <v>46073.699947870366</v>
@@ -4297,16 +4300,16 @@
         <v>46132.57863447917</v>
       </c>
       <c r="E47" s="9" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="F47" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G47" s="9" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="H47" s="9" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="I47" s="8">
         <v>46035</v>
@@ -4324,29 +4327,29 @@
         <v>26</v>
       </c>
       <c r="N47" s="9" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="O47" s="9" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="P47" s="9" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="Q47" s="9"/>
       <c r="R47" s="9"/>
       <c r="S47" s="11" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="T47" s="9">
         <v>0</v>
       </c>
       <c r="U47" s="10" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="48" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A48" s="4" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="B48" s="5">
         <v>46076.881105196764</v>
@@ -4358,16 +4361,16 @@
         <v>46139.54788491898</v>
       </c>
       <c r="E48" s="6" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="F48" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G48" s="6" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="H48" s="6" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="I48" s="5">
         <v>46014</v>
@@ -4385,13 +4388,13 @@
         <v>26</v>
       </c>
       <c r="N48" s="6" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="O48" s="6" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="P48" s="6" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="Q48" s="5">
         <v>46014</v>
@@ -4411,7 +4414,7 @@
     </row>
     <row r="49" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A49" s="7" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="B49" s="8">
         <v>46076.88918239583</v>
@@ -4423,16 +4426,16 @@
         <v>46112.491848171296</v>
       </c>
       <c r="E49" s="9" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="F49" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G49" s="9" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="H49" s="9" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="I49" s="8">
         <v>46014</v>
@@ -4450,13 +4453,13 @@
         <v>26</v>
       </c>
       <c r="N49" s="9" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="O49" s="9" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="P49" s="9" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="Q49" s="9"/>
       <c r="R49" s="9"/>
@@ -4466,7 +4469,7 @@
     </row>
     <row r="50" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A50" s="4" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="B50" s="5">
         <v>46076.88930991898</v>
@@ -4478,16 +4481,16 @@
         <v>46112.50608989583</v>
       </c>
       <c r="E50" s="6" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="F50" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G50" s="6" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="H50" s="6" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="I50" s="5">
         <v>46043</v>
@@ -4505,13 +4508,13 @@
         <v>26</v>
       </c>
       <c r="N50" s="6" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="O50" s="6" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="P50" s="6" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="Q50" s="6"/>
       <c r="R50" s="6"/>
@@ -4521,7 +4524,7 @@
     </row>
     <row r="51" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A51" s="7" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="B51" s="8">
         <v>46077.579487986106</v>
@@ -4533,16 +4536,16 @@
         <v>46191.83738863426</v>
       </c>
       <c r="E51" s="9" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="F51" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G51" s="9" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="H51" s="9" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="I51" s="8">
         <v>46014</v>
@@ -4560,10 +4563,10 @@
         <v>26</v>
       </c>
       <c r="N51" s="9" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="O51" s="9" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="P51" s="9" t="s">
         <v>26</v>
@@ -4581,12 +4584,12 @@
         <v>0</v>
       </c>
       <c r="U51" s="10" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="52" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A52" s="4" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="B52" s="5">
         <v>46077.5872287963</v>
@@ -4598,16 +4601,16 @@
         <v>46182.68337341435</v>
       </c>
       <c r="E52" s="6" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="F52" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G52" s="6" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="H52" s="6" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="I52" s="5">
         <v>46014</v>
@@ -4625,13 +4628,13 @@
         <v>26</v>
       </c>
       <c r="N52" s="6" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="O52" s="6" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="P52" s="6" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="Q52" s="6"/>
       <c r="R52" s="6"/>
@@ -4641,7 +4644,7 @@
     </row>
     <row r="53" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A53" s="7" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="B53" s="8">
         <v>46077.58741234954</v>
@@ -4653,16 +4656,16 @@
         <v>46182.69210671296</v>
       </c>
       <c r="E53" s="9" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="F53" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G53" s="9" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="H53" s="9" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="I53" s="8">
         <v>46017</v>
@@ -4680,13 +4683,13 @@
         <v>26</v>
       </c>
       <c r="N53" s="9" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="O53" s="9" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="P53" s="9" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="Q53" s="9"/>
       <c r="R53" s="9"/>
@@ -4696,7 +4699,7 @@
     </row>
     <row r="54" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A54" s="4" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="B54" s="5">
         <v>46077.57954119213</v>
@@ -4708,16 +4711,16 @@
         <v>46174.6518578588</v>
       </c>
       <c r="E54" s="6" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="F54" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G54" s="6" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="H54" s="6" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="I54" s="5">
         <v>46014</v>
@@ -4735,10 +4738,10 @@
         <v>26</v>
       </c>
       <c r="N54" s="6" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="O54" s="6" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="P54" s="6" t="s">
         <v>26</v>
@@ -4756,12 +4759,12 @@
         <v>0</v>
       </c>
       <c r="U54" s="10" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="55" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A55" s="7" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="B55" s="8">
         <v>46077.587555833336</v>
@@ -4773,16 +4776,16 @@
         <v>46169.8399244676</v>
       </c>
       <c r="E55" s="9" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="F55" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G55" s="9" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="H55" s="9" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="I55" s="8">
         <v>46014</v>
@@ -4800,13 +4803,13 @@
         <v>26</v>
       </c>
       <c r="N55" s="9" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="O55" s="9" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P55" s="9" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="Q55" s="9"/>
       <c r="R55" s="9"/>
@@ -4816,7 +4819,7 @@
     </row>
     <row r="56" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A56" s="4" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="B56" s="5">
         <v>46077.5876627199</v>
@@ -4828,16 +4831,16 @@
         <v>46174.651731377315</v>
       </c>
       <c r="E56" s="6" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="F56" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G56" s="6" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="H56" s="6" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="I56" s="5">
         <v>46017</v>
@@ -4855,13 +4858,13 @@
         <v>26</v>
       </c>
       <c r="N56" s="6" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="O56" s="6" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="P56" s="6" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="Q56" s="6"/>
       <c r="R56" s="6"/>
@@ -4871,7 +4874,7 @@
     </row>
     <row r="57" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A57" s="7" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="B57" s="8">
         <v>46139.543413900465</v>
@@ -4883,16 +4886,16 @@
         <v>46205.80892784722</v>
       </c>
       <c r="E57" s="9" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="F57" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G57" s="9" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="H57" s="9" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="I57" s="8">
         <v>46139</v>
@@ -4910,10 +4913,10 @@
         <v>26</v>
       </c>
       <c r="N57" s="9" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="O57" s="9" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="P57" s="9" t="s">
         <v>26</v>
@@ -4925,18 +4928,18 @@
         <v>46177</v>
       </c>
       <c r="S57" s="11" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="T57" s="9">
         <v>0</v>
       </c>
       <c r="U57" s="12" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
     </row>
     <row r="58" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A58" s="4" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="B58" s="5">
         <v>46139.543700821756</v>
@@ -4948,16 +4951,16 @@
         <v>46191.83987099537</v>
       </c>
       <c r="E58" s="6" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F58" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G58" s="6" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="H58" s="6" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="I58" s="5">
         <v>46139</v>
@@ -4975,13 +4978,13 @@
         <v>26</v>
       </c>
       <c r="N58" s="6" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="O58" s="6" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="P58" s="6" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="Q58" s="6"/>
       <c r="R58" s="6"/>
@@ -4991,7 +4994,7 @@
     </row>
     <row r="59" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A59" s="7" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="B59" s="8">
         <v>46139.54378479166</v>
@@ -5003,16 +5006,16 @@
         <v>46191.83995613426</v>
       </c>
       <c r="E59" s="9" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="F59" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G59" s="9" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="H59" s="9" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="I59" s="8">
         <v>46149</v>
@@ -5030,10 +5033,10 @@
         <v>26</v>
       </c>
       <c r="N59" s="9" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="O59" s="9" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="P59" s="9" t="s">
         <v>26</v>
@@ -5046,7 +5049,7 @@
     </row>
     <row r="60" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A60" s="4" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="B60" s="5">
         <v>46205.80892462963</v>
@@ -5056,16 +5059,16 @@
         <v>46212.84863678241</v>
       </c>
       <c r="E60" s="6" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="F60" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G60" s="6" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="H60" s="6" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="I60" s="6"/>
       <c r="J60" s="5">
@@ -5081,13 +5084,13 @@
         <v>26</v>
       </c>
       <c r="N60" s="6" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="O60" s="6" t="s">
         <v>26</v>
       </c>
       <c r="P60" s="6" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="Q60" s="6"/>
       <c r="R60" s="6"/>
@@ -5097,7 +5100,7 @@
     </row>
     <row r="61" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A61" s="7" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="B61" s="8">
         <v>46073.69994815972</v>
@@ -5107,7 +5110,7 @@
         <v>46129.586425601854</v>
       </c>
       <c r="E61" s="9" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="F61" s="9" t="s">
         <v>25</v>
@@ -5131,7 +5134,7 @@
         <v>26</v>
       </c>
       <c r="O61" s="9" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="P61" s="9" t="s">
         <v>26</v>
@@ -5144,7 +5147,7 @@
     </row>
     <row r="62" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A62" s="4" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="B62" s="5">
         <v>46073.6999484375</v>
@@ -5156,16 +5159,16 @@
         <v>46099.54242268519</v>
       </c>
       <c r="E62" s="6" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="F62" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G62" s="6" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="H62" s="6" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="I62" s="5">
         <v>46003</v>
@@ -5183,13 +5186,13 @@
         <v>26</v>
       </c>
       <c r="N62" s="6" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="O62" s="6" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="P62" s="6" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="Q62" s="5">
         <v>46003</v>
@@ -5209,7 +5212,7 @@
     </row>
     <row r="63" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A63" s="7" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="B63" s="8">
         <v>46073.699946249995</v>
@@ -5221,16 +5224,16 @@
         <v>46129.58626813657</v>
       </c>
       <c r="E63" s="9" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="F63" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G63" s="9" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="H63" s="9" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="I63" s="8">
         <v>46058</v>
@@ -5248,13 +5251,13 @@
         <v>26</v>
       </c>
       <c r="N63" s="9" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="O63" s="9" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="P63" s="9" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="Q63" s="8">
         <v>46058</v>
@@ -5274,7 +5277,7 @@
     </row>
     <row r="64" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A64" s="4" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="B64" s="5">
         <v>46092.494241736116</v>
@@ -5286,16 +5289,16 @@
         <v>46210.861392569444</v>
       </c>
       <c r="E64" s="6" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="F64" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G64" s="6" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="H64" s="6" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="I64" s="6"/>
       <c r="J64" s="5">
@@ -5311,13 +5314,13 @@
         <v>26</v>
       </c>
       <c r="N64" s="6" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="O64" s="6" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="P64" s="6" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="Q64" s="5">
         <v>46065</v>
@@ -5337,7 +5340,7 @@
     </row>
     <row r="65" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A65" s="7" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="B65" s="8">
         <v>46092.49428590278</v>
@@ -5347,16 +5350,16 @@
         <v>46154.16811805556</v>
       </c>
       <c r="E65" s="9" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="F65" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G65" s="9" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="H65" s="9" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="I65" s="8">
         <v>46154</v>
@@ -5374,13 +5377,13 @@
         <v>26</v>
       </c>
       <c r="N65" s="9" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="O65" s="9" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="P65" s="9" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="Q65" s="8">
         <v>46154</v>
@@ -5389,18 +5392,18 @@
         <v>46154</v>
       </c>
       <c r="S65" s="11" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="T65" s="9">
         <v>0</v>
       </c>
       <c r="U65" s="10" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="66" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A66" s="4" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="B66" s="5">
         <v>46073.69994662037</v>
@@ -5410,7 +5413,7 @@
         <v>46210.858702094905</v>
       </c>
       <c r="E66" s="6" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="F66" s="6" t="s">
         <v>25</v>
@@ -5434,7 +5437,7 @@
         <v>26</v>
       </c>
       <c r="O66" s="6" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="P66" s="6" t="s">
         <v>26</v>
@@ -5447,7 +5450,7 @@
     </row>
     <row r="67" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A67" s="7" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="B67" s="8">
         <v>46073.69994689815</v>
@@ -5459,16 +5462,16 @@
         <v>46210.85869597222</v>
       </c>
       <c r="E67" s="9" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="F67" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G67" s="9" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="H67" s="9" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="I67" s="8">
         <v>46063</v>
@@ -5486,13 +5489,13 @@
         <v>26</v>
       </c>
       <c r="N67" s="9" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="O67" s="9" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="P67" s="9" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="Q67" s="8">
         <v>46063</v>
@@ -5507,12 +5510,12 @@
         <v>0</v>
       </c>
       <c r="U67" s="12" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
     </row>
     <row r="68" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A68" s="4" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="B68" s="5">
         <v>46073.69994719907</v>
@@ -5524,16 +5527,16 @@
         <v>46210.86139240741</v>
       </c>
       <c r="E68" s="6" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="F68" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G68" s="6" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="H68" s="6" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="I68" s="5">
         <v>46065</v>
@@ -5551,13 +5554,13 @@
         <v>26</v>
       </c>
       <c r="N68" s="6" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="O68" s="6" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="P68" s="6" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="Q68" s="5">
         <v>46065</v>
@@ -5572,12 +5575,12 @@
         <v>0</v>
       </c>
       <c r="U68" s="10" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="69" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A69" s="7" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="B69" s="8">
         <v>46073.699948865746</v>
@@ -5587,7 +5590,7 @@
         <v>46213.56641354167</v>
       </c>
       <c r="E69" s="9" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="F69" s="9" t="s">
         <v>25</v>
@@ -5611,7 +5614,7 @@
         <v>26</v>
       </c>
       <c r="O69" s="9" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="P69" s="9" t="s">
         <v>26</v>
@@ -5624,7 +5627,7 @@
     </row>
     <row r="70" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A70" s="4" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="B70" s="5">
         <v>46073.69995097222</v>
@@ -5634,16 +5637,16 @@
         <v>46213.56641027778</v>
       </c>
       <c r="E70" s="6" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="F70" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G70" s="6" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="H70" s="6" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="I70" s="5">
         <v>46097</v>
@@ -5661,13 +5664,13 @@
         <v>26</v>
       </c>
       <c r="N70" s="6" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="O70" s="6" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="P70" s="6" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="Q70" s="5">
         <v>46097</v>
@@ -5682,12 +5685,12 @@
         <v>0</v>
       </c>
       <c r="U70" s="10" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="71" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A71" s="7" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="B71" s="8">
         <v>46073.69994640046</v>
@@ -5697,16 +5700,16 @@
         <v>46121.187778182866</v>
       </c>
       <c r="E71" s="9" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="F71" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G71" s="9" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="H71" s="9" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="I71" s="8">
         <v>46119</v>
@@ -5724,13 +5727,13 @@
         <v>26</v>
       </c>
       <c r="N71" s="9" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="O71" s="9" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="P71" s="9" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="Q71" s="8">
         <v>46119</v>
@@ -5745,12 +5748,12 @@
         <v>0</v>
       </c>
       <c r="U71" s="10" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="72" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A72" s="4" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="B72" s="5">
         <v>46073.699946782406</v>
@@ -5760,16 +5763,16 @@
         <v>46199.82646660879</v>
       </c>
       <c r="E72" s="6" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="F72" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G72" s="6" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="H72" s="6" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="I72" s="5">
         <v>46132</v>
@@ -5787,13 +5790,13 @@
         <v>26</v>
       </c>
       <c r="N72" s="6" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="O72" s="6" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="P72" s="6" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="Q72" s="5">
         <v>46132</v>
@@ -5808,12 +5811,12 @@
         <v>0</v>
       </c>
       <c r="U72" s="10" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="73" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A73" s="7" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="B73" s="8">
         <v>46073.69994708333</v>
@@ -5825,16 +5828,16 @@
         <v>46195.603959687505</v>
       </c>
       <c r="E73" s="9" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="F73" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G73" s="9" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="H73" s="9" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="I73" s="8">
         <v>46147</v>
@@ -5852,13 +5855,13 @@
         <v>26</v>
       </c>
       <c r="N73" s="9" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="O73" s="9" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="P73" s="9" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="Q73" s="8">
         <v>46147</v>
@@ -5867,18 +5870,18 @@
         <v>46148</v>
       </c>
       <c r="S73" s="11" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="T73" s="9">
         <v>0</v>
       </c>
       <c r="U73" s="12" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
     </row>
     <row r="74" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A74" s="4" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="B74" s="5">
         <v>46076.88127923611</v>
@@ -5890,16 +5893,16 @@
         <v>46195.60422127315</v>
       </c>
       <c r="E74" s="6" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="F74" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G74" s="6" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="H74" s="6" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="I74" s="5">
         <v>46121</v>
@@ -5917,13 +5920,13 @@
         <v>26</v>
       </c>
       <c r="N74" s="6" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="O74" s="6" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="P74" s="6" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="Q74" s="5">
         <v>46121</v>
@@ -5938,12 +5941,12 @@
         <v>0</v>
       </c>
       <c r="U74" s="12" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
     </row>
     <row r="75" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A75" s="7" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="B75" s="8">
         <v>46077.57961084491</v>
@@ -5955,16 +5958,16 @@
         <v>46195.60466490741</v>
       </c>
       <c r="E75" s="9" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="F75" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G75" s="9" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="H75" s="9" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="I75" s="8">
         <v>46104</v>
@@ -5982,13 +5985,13 @@
         <v>26</v>
       </c>
       <c r="N75" s="9" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="O75" s="9" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="P75" s="9" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="Q75" s="8">
         <v>46104</v>
@@ -6003,12 +6006,12 @@
         <v>0</v>
       </c>
       <c r="U75" s="10" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="76" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A76" s="4" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="B76" s="5">
         <v>46077.57965403935</v>
@@ -6018,16 +6021,16 @@
         <v>46182.692112696765</v>
       </c>
       <c r="E76" s="6" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="F76" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G76" s="6" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="H76" s="6" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="I76" s="5">
         <v>46098</v>
@@ -6045,13 +6048,13 @@
         <v>26</v>
       </c>
       <c r="N76" s="6" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="O76" s="6" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="P76" s="6" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="Q76" s="5">
         <v>46098</v>
@@ -6066,12 +6069,12 @@
         <v>0</v>
       </c>
       <c r="U76" s="10" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="77" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A77" s="7" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="B77" s="8">
         <v>46073.69994733796</v>
@@ -6081,7 +6084,7 @@
         <v>46078.621237141204</v>
       </c>
       <c r="E77" s="9" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="F77" s="9" t="s">
         <v>25</v>
@@ -6105,7 +6108,7 @@
         <v>26</v>
       </c>
       <c r="O77" s="9" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="P77" s="9" t="s">
         <v>26</v>
@@ -6118,7 +6121,7 @@
     </row>
     <row r="78" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A78" s="4" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="B78" s="5">
         <v>46073.69994759259</v>
@@ -6128,16 +6131,16 @@
         <v>46210.861684930554</v>
       </c>
       <c r="E78" s="6" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="F78" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G78" s="6" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="H78" s="6" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="I78" s="5">
         <v>46111</v>
@@ -6155,13 +6158,13 @@
         <v>26</v>
       </c>
       <c r="N78" s="6" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="O78" s="6" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="P78" s="6" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="Q78" s="5">
         <v>46111</v>
@@ -6176,12 +6179,12 @@
         <v>0</v>
       </c>
       <c r="U78" s="10" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="79" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A79" s="7" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="B79" s="8">
         <v>46073.69994784722</v>
@@ -6191,16 +6194,16 @@
         <v>46198.59349042824</v>
       </c>
       <c r="E79" s="9" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="F79" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G79" s="9" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="H79" s="9" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="I79" s="8">
         <v>46149</v>
@@ -6218,13 +6221,13 @@
         <v>26</v>
       </c>
       <c r="N79" s="9" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="O79" s="9" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="P79" s="9" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="Q79" s="8">
         <v>46149</v>
@@ -6233,18 +6236,18 @@
         <v>46150</v>
       </c>
       <c r="S79" s="11" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="T79" s="9">
         <v>0</v>
       </c>
       <c r="U79" s="10" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="80" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A80" s="4" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="B80" s="5">
         <v>46073.69994813658</v>
@@ -6254,16 +6257,16 @@
         <v>46198.592367060184</v>
       </c>
       <c r="E80" s="6" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="F80" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G80" s="6" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="H80" s="6" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="I80" s="5">
         <v>46134</v>
@@ -6281,13 +6284,13 @@
         <v>26</v>
       </c>
       <c r="N80" s="6" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="O80" s="6" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="P80" s="6" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="Q80" s="5">
         <v>46134</v>
@@ -6302,12 +6305,12 @@
         <v>0</v>
       </c>
       <c r="U80" s="10" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="81" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A81" s="7" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="B81" s="8">
         <v>46073.699948368056</v>
@@ -6317,16 +6320,16 @@
         <v>46213.56641375</v>
       </c>
       <c r="E81" s="9" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="F81" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G81" s="9" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="H81" s="9" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="I81" s="8">
         <v>46136</v>
@@ -6344,13 +6347,13 @@
         <v>26</v>
       </c>
       <c r="N81" s="9" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="O81" s="9" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="P81" s="9" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="Q81" s="8">
         <v>46136</v>
@@ -6359,18 +6362,18 @@
         <v>46139</v>
       </c>
       <c r="S81" s="12" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="T81" s="9">
         <v>0.5</v>
       </c>
       <c r="U81" s="10" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="82" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A82" s="4" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="B82" s="5">
         <v>46076.88137268518</v>
@@ -6380,16 +6383,16 @@
         <v>46195.60422616898</v>
       </c>
       <c r="E82" s="6" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="F82" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G82" s="6" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="H82" s="6" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="I82" s="5">
         <v>46129</v>
@@ -6407,13 +6410,13 @@
         <v>26</v>
       </c>
       <c r="N82" s="6" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="O82" s="6" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="P82" s="6" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="Q82" s="5">
         <v>46129</v>
@@ -6428,12 +6431,12 @@
         <v>0</v>
       </c>
       <c r="U82" s="10" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="83" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A83" s="7" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="B83" s="8">
         <v>46073.69994864584</v>
@@ -6443,16 +6446,16 @@
         <v>46153.16811694445</v>
       </c>
       <c r="E83" s="9" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="F83" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G83" s="9" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="H83" s="9" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="I83" s="8">
         <v>46153</v>
@@ -6470,13 +6473,13 @@
         <v>26</v>
       </c>
       <c r="N83" s="9" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="O83" s="9" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="P83" s="9" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="Q83" s="8">
         <v>46153</v>
@@ -6485,18 +6488,18 @@
         <v>46153</v>
       </c>
       <c r="S83" s="11" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="T83" s="9">
         <v>0</v>
       </c>
       <c r="U83" s="10" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="84" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A84" s="4" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="B84" s="5">
         <v>46073.699948912035</v>
@@ -6506,16 +6509,16 @@
         <v>46154.16785564815</v>
       </c>
       <c r="E84" s="6" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="F84" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G84" s="6" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="H84" s="6" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="I84" s="5">
         <v>46154</v>
@@ -6533,13 +6536,13 @@
         <v>26</v>
       </c>
       <c r="N84" s="6" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="O84" s="6" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="P84" s="6" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="Q84" s="5">
         <v>46154</v>
@@ -6548,18 +6551,18 @@
         <v>46154</v>
       </c>
       <c r="S84" s="11" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="T84" s="6">
         <v>0</v>
       </c>
       <c r="U84" s="10" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="85" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A85" s="7" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="B85" s="8">
         <v>46073.69994572917</v>
@@ -6569,7 +6572,7 @@
         <v>46077.638347245374</v>
       </c>
       <c r="E85" s="9" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="F85" s="9" t="s">
         <v>25</v>
@@ -6593,7 +6596,7 @@
         <v>26</v>
       </c>
       <c r="O85" s="9" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="P85" s="9" t="s">
         <v>26</v>
@@ -6606,7 +6609,7 @@
     </row>
     <row r="86" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A86" s="4" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="B86" s="5">
         <v>46073.699946099536</v>
@@ -6616,16 +6619,16 @@
         <v>46210.60325569444</v>
       </c>
       <c r="E86" s="6" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="F86" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G86" s="6" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="H86" s="6" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="I86" s="5">
         <v>46155</v>
@@ -6643,13 +6646,13 @@
         <v>26</v>
       </c>
       <c r="N86" s="6" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="O86" s="6" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="P86" s="6" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="Q86" s="5">
         <v>46155</v>
@@ -6658,18 +6661,18 @@
         <v>46155</v>
       </c>
       <c r="S86" s="11" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="T86" s="6">
         <v>0</v>
       </c>
       <c r="U86" s="10" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="87" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A87" s="7" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="B87" s="8">
         <v>46073.69994638889</v>
@@ -6679,16 +6682,16 @@
         <v>46195.604670092594</v>
       </c>
       <c r="E87" s="9" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="F87" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G87" s="9" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="H87" s="9" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="I87" s="8">
         <v>46156</v>
@@ -6706,13 +6709,13 @@
         <v>26</v>
       </c>
       <c r="N87" s="9" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="O87" s="9" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="P87" s="9" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="Q87" s="8">
         <v>46156</v>
@@ -6721,18 +6724,18 @@
         <v>46160</v>
       </c>
       <c r="S87" s="11" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="T87" s="9">
         <v>0</v>
       </c>
       <c r="U87" s="10" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="88" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A88" s="4" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="B88" s="5">
         <v>46073.69994668981</v>
@@ -6742,16 +6745,16 @@
         <v>46161.25032122685</v>
       </c>
       <c r="E88" s="6" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="F88" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G88" s="6" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="H88" s="6" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="I88" s="5">
         <v>46161</v>
@@ -6769,13 +6772,13 @@
         <v>26</v>
       </c>
       <c r="N88" s="6" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="O88" s="6" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="P88" s="6" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="Q88" s="5">
         <v>46161</v>
@@ -6784,18 +6787,18 @@
         <v>46161</v>
       </c>
       <c r="S88" s="11" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="T88" s="6">
         <v>0</v>
       </c>
       <c r="U88" s="10" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="89" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A89" s="7" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="B89" s="8">
         <v>46073.69994695602</v>
@@ -6805,16 +6808,16 @@
         <v>46162.25040996527</v>
       </c>
       <c r="E89" s="9" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="F89" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G89" s="9" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="H89" s="9" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="I89" s="8">
         <v>46162</v>
@@ -6832,13 +6835,13 @@
         <v>26</v>
       </c>
       <c r="N89" s="9" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="O89" s="9" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="P89" s="9" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="Q89" s="8">
         <v>46162</v>
@@ -6847,18 +6850,18 @@
         <v>46162</v>
       </c>
       <c r="S89" s="11" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="T89" s="9">
         <v>0</v>
       </c>
       <c r="U89" s="10" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="90" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A90" s="4" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="B90" s="5">
         <v>46073.699947245375</v>
@@ -6868,7 +6871,7 @@
         <v>46077.6387968287</v>
       </c>
       <c r="E90" s="6" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="F90" s="6" t="s">
         <v>25</v>
@@ -6892,7 +6895,7 @@
         <v>26</v>
       </c>
       <c r="O90" s="6" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="P90" s="6" t="s">
         <v>26</v>
@@ -6905,7 +6908,7 @@
     </row>
     <row r="91" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A91" s="7" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="B91" s="8">
         <v>46073.699947500005</v>
@@ -6915,16 +6918,16 @@
         <v>46174.16833755787</v>
       </c>
       <c r="E91" s="9" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="F91" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G91" s="9" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="H91" s="9" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="I91" s="8">
         <v>46164</v>
@@ -6942,13 +6945,13 @@
         <v>26</v>
       </c>
       <c r="N91" s="9" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="O91" s="9" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="P91" s="9" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="Q91" s="8">
         <v>46164</v>
@@ -6957,18 +6960,18 @@
         <v>46174</v>
       </c>
       <c r="S91" s="11" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="T91" s="9">
         <v>0</v>
       </c>
       <c r="U91" s="10" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="92" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A92" s="4" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="B92" s="5">
         <v>46073.699947789355</v>
@@ -6978,16 +6981,16 @@
         <v>46174.168340185184</v>
       </c>
       <c r="E92" s="6" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="F92" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G92" s="6" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="H92" s="6" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="I92" s="5">
         <v>46164</v>
@@ -7005,13 +7008,13 @@
         <v>26</v>
       </c>
       <c r="N92" s="6" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="O92" s="6" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="P92" s="6" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="Q92" s="5">
         <v>46164</v>
@@ -7020,18 +7023,18 @@
         <v>46174</v>
       </c>
       <c r="S92" s="11" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="T92" s="6">
         <v>0</v>
       </c>
       <c r="U92" s="10" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="93" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A93" s="7" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="B93" s="8">
         <v>46092.48971385417</v>
@@ -7041,7 +7044,7 @@
         <v>46092.497058946756</v>
       </c>
       <c r="E93" s="9" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="F93" s="9" t="s">
         <v>25</v>
@@ -7065,7 +7068,7 @@
         <v>26</v>
       </c>
       <c r="O93" s="9" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="P93" s="9" t="s">
         <v>26</v>
@@ -7073,18 +7076,18 @@
       <c r="Q93" s="9"/>
       <c r="R93" s="9"/>
       <c r="S93" s="11" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="T93" s="9">
         <v>0</v>
       </c>
       <c r="U93" s="10" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="94" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A94" s="4" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="B94" s="5">
         <v>46092.49161491898</v>
@@ -7094,16 +7097,16 @@
         <v>46171.168742951384</v>
       </c>
       <c r="E94" s="6" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="F94" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G94" s="6" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="H94" s="6" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="I94" s="5">
         <v>46164</v>
@@ -7121,13 +7124,13 @@
         <v>26</v>
       </c>
       <c r="N94" s="6" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="O94" s="6" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="P94" s="6" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="Q94" s="5">
         <v>46164</v>
@@ -7136,18 +7139,18 @@
         <v>46171</v>
       </c>
       <c r="S94" s="11" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="T94" s="6">
         <v>0</v>
       </c>
       <c r="U94" s="10" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="95" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A95" s="7" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="B95" s="8">
         <v>46092.491661747685</v>
@@ -7157,16 +7160,16 @@
         <v>46181.16820616898</v>
       </c>
       <c r="E95" s="9" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="F95" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G95" s="9" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="H95" s="9" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="I95" s="8">
         <v>46174</v>
@@ -7184,13 +7187,13 @@
         <v>26</v>
       </c>
       <c r="N95" s="9" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="O95" s="9" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="P95" s="9" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="Q95" s="8">
         <v>46174</v>
@@ -7199,13 +7202,13 @@
         <v>46181</v>
       </c>
       <c r="S95" s="11" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="T95" s="9">
         <v>0</v>
       </c>
       <c r="U95" s="10" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualiza portafolio 2026-07-14 14:09 UTC
</commit_message>
<xml_diff>
--- a/data/50001490 - ZITRON PERU METRO LIMA PV04-PV05.xlsx
+++ b/data/50001490 - ZITRON PERU METRO LIMA PV04-PV05.xlsx
@@ -3551,7 +3551,7 @@
       </c>
       <c r="C35" s="9"/>
       <c r="D35" s="8">
-        <v>46174.65273861111</v>
+        <v>46217.58160621527</v>
       </c>
       <c r="E35" s="9" t="s">
         <v>134</v>
@@ -5056,7 +5056,7 @@
       </c>
       <c r="C60" s="6"/>
       <c r="D60" s="5">
-        <v>46213.85753734954</v>
+        <v>46217.57588326389</v>
       </c>
       <c r="E60" s="6" t="s">
         <v>208</v>

</xml_diff>

<commit_message>
KPI actualizado 2026-07-15 14:54 UTC
</commit_message>
<xml_diff>
--- a/data/50001490 - ZITRON PERU METRO LIMA PV04-PV05.xlsx
+++ b/data/50001490 - ZITRON PERU METRO LIMA PV04-PV05.xlsx
@@ -3551,7 +3551,7 @@
       </c>
       <c r="C35" s="9"/>
       <c r="D35" s="8">
-        <v>46217.58160621527</v>
+        <v>46218.59376659722</v>
       </c>
       <c r="E35" s="9" t="s">
         <v>134</v>
@@ -5056,7 +5056,7 @@
       </c>
       <c r="C60" s="6"/>
       <c r="D60" s="5">
-        <v>46217.57588326389</v>
+        <v>46218.58775554398</v>
       </c>
       <c r="E60" s="6" t="s">
         <v>208</v>

</xml_diff>

<commit_message>
Curva S actualizada 2026-08-01 17:10 Chile
</commit_message>
<xml_diff>
--- a/data/50001490 - ZITRON PERU METRO LIMA PV04-PV05.xlsx
+++ b/data/50001490 - ZITRON PERU METRO LIMA PV04-PV05.xlsx
@@ -2678,7 +2678,7 @@
         <v>46093.87454615741</v>
       </c>
       <c r="D21" s="8">
-        <v>46139.54278021991</v>
+        <v>46235.71759233796</v>
       </c>
       <c r="E21" s="9" t="s">
         <v>88</v>
@@ -4880,7 +4880,7 @@
         <v>46191.840089791665</v>
       </c>
       <c r="D57" s="8">
-        <v>46205.80892784722</v>
+        <v>46235.717934444445</v>
       </c>
       <c r="E57" s="9" t="s">
         <v>199</v>

</xml_diff>

<commit_message>
Actualiza portafolio 2026-08-28 23:04 UTC
</commit_message>
<xml_diff>
--- a/data/50001490 - ZITRON PERU METRO LIMA PV04-PV05.xlsx
+++ b/data/50001490 - ZITRON PERU METRO LIMA PV04-PV05.xlsx
@@ -6056,7 +6056,7 @@
       </c>
       <c r="C77" s="9"/>
       <c r="D77" s="8">
-        <v>46247.53022914352</v>
+        <v>46262.80759832176</v>
       </c>
       <c r="E77" s="9" t="s">
         <v>264</v>
@@ -6168,7 +6168,7 @@
       </c>
       <c r="C79" s="9"/>
       <c r="D79" s="8">
-        <v>46260.56856410879</v>
+        <v>46262.808263865736</v>
       </c>
       <c r="E79" s="9" t="s">
         <v>269</v>
@@ -6218,8 +6218,8 @@
       <c r="T79" s="9">
         <v>0</v>
       </c>
-      <c r="U79" s="12" t="s">
-        <v>202</v>
+      <c r="U79" s="11" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="80" spans="1:21" x14ac:dyDescent="0.25">
@@ -6296,7 +6296,7 @@
       </c>
       <c r="C81" s="9"/>
       <c r="D81" s="8">
-        <v>46237.5541136574</v>
+        <v>46262.80775383102</v>
       </c>
       <c r="E81" s="9" t="s">
         <v>276</v>
@@ -6346,8 +6346,8 @@
       <c r="T81" s="9">
         <v>0.5</v>
       </c>
-      <c r="U81" s="12" t="s">
-        <v>202</v>
+      <c r="U81" s="11" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="82" spans="1:21" x14ac:dyDescent="0.25">
@@ -6357,9 +6357,11 @@
       <c r="B82" s="5">
         <v>46076.88137268518</v>
       </c>
-      <c r="C82" s="6"/>
+      <c r="C82" s="5">
+        <v>46262.80759297454</v>
+      </c>
       <c r="D82" s="5">
-        <v>46237.554114976854</v>
+        <v>46262.80759458333</v>
       </c>
       <c r="E82" s="6" t="s">
         <v>280</v>
@@ -6409,8 +6411,8 @@
       <c r="T82" s="6">
         <v>0</v>
       </c>
-      <c r="U82" s="12" t="s">
-        <v>202</v>
+      <c r="U82" s="11" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="83" spans="1:21" x14ac:dyDescent="0.25">
@@ -6422,7 +6424,7 @@
       </c>
       <c r="C83" s="9"/>
       <c r="D83" s="8">
-        <v>46237.55404603009</v>
+        <v>46262.80759803241</v>
       </c>
       <c r="E83" s="9" t="s">
         <v>231</v>
@@ -6548,7 +6550,7 @@
       </c>
       <c r="C85" s="9"/>
       <c r="D85" s="8">
-        <v>46077.638347245374</v>
+        <v>46262.80754692129</v>
       </c>
       <c r="E85" s="9" t="s">
         <v>290</v>
@@ -6719,9 +6721,11 @@
       <c r="B88" s="5">
         <v>46073.69994668981</v>
       </c>
-      <c r="C88" s="6"/>
+      <c r="C88" s="5">
+        <v>46262.80753832176</v>
+      </c>
       <c r="D88" s="5">
-        <v>46161.25032122685</v>
+        <v>46262.807540567126</v>
       </c>
       <c r="E88" s="6" t="s">
         <v>301</v>
@@ -6771,8 +6775,8 @@
       <c r="T88" s="6">
         <v>0</v>
       </c>
-      <c r="U88" s="10" t="s">
-        <v>59</v>
+      <c r="U88" s="11" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="89" spans="1:21" x14ac:dyDescent="0.25">
@@ -6784,7 +6788,7 @@
       </c>
       <c r="C89" s="9"/>
       <c r="D89" s="8">
-        <v>46240.72176880787</v>
+        <v>46262.80754540509</v>
       </c>
       <c r="E89" s="9" t="s">
         <v>306</v>

</xml_diff>

<commit_message>
Actualizacion automatica 2026-08-31 15:24 UTC
</commit_message>
<xml_diff>
--- a/data/50001490 - ZITRON PERU METRO LIMA PV04-PV05.xlsx
+++ b/data/50001490 - ZITRON PERU METRO LIMA PV04-PV05.xlsx
@@ -5562,7 +5562,7 @@
       </c>
       <c r="C69" s="9"/>
       <c r="D69" s="8">
-        <v>46213.56641354167</v>
+        <v>46265.58197266204</v>
       </c>
       <c r="E69" s="9" t="s">
         <v>234</v>
@@ -5607,9 +5607,11 @@
       <c r="B70" s="5">
         <v>46073.69995097222</v>
       </c>
-      <c r="C70" s="6"/>
+      <c r="C70" s="5">
+        <v>46265.581966122685</v>
+      </c>
       <c r="D70" s="5">
-        <v>46213.56641027778</v>
+        <v>46265.58196802084</v>
       </c>
       <c r="E70" s="6" t="s">
         <v>246</v>
@@ -5733,9 +5735,11 @@
       <c r="B72" s="5">
         <v>46073.699946782406</v>
       </c>
-      <c r="C72" s="6"/>
+      <c r="C72" s="5">
+        <v>46265.58195543982</v>
+      </c>
       <c r="D72" s="5">
-        <v>46199.82646660879</v>
+        <v>46265.58195854167</v>
       </c>
       <c r="E72" s="6" t="s">
         <v>251</v>
@@ -6056,7 +6060,7 @@
       </c>
       <c r="C77" s="9"/>
       <c r="D77" s="8">
-        <v>46262.80759832176</v>
+        <v>46265.58240835648</v>
       </c>
       <c r="E77" s="9" t="s">
         <v>264</v>
@@ -6166,9 +6170,11 @@
       <c r="B79" s="8">
         <v>46073.69994784722</v>
       </c>
-      <c r="C79" s="9"/>
+      <c r="C79" s="8">
+        <v>46265.58239951389</v>
+      </c>
       <c r="D79" s="8">
-        <v>46262.808263865736</v>
+        <v>46265.582400960644</v>
       </c>
       <c r="E79" s="9" t="s">
         <v>269</v>
@@ -6233,7 +6239,7 @@
         <v>46237.554038807866</v>
       </c>
       <c r="D80" s="5">
-        <v>46237.55411311342</v>
+        <v>46265.58196423611</v>
       </c>
       <c r="E80" s="6" t="s">
         <v>273</v>
@@ -6294,9 +6300,11 @@
       <c r="B81" s="8">
         <v>46073.699948368056</v>
       </c>
-      <c r="C81" s="9"/>
+      <c r="C81" s="8">
+        <v>46265.5822203125</v>
+      </c>
       <c r="D81" s="8">
-        <v>46262.80775383102</v>
+        <v>46265.58222244213</v>
       </c>
       <c r="E81" s="9" t="s">
         <v>276</v>
@@ -6424,7 +6432,7 @@
       </c>
       <c r="C83" s="9"/>
       <c r="D83" s="8">
-        <v>46262.80759803241</v>
+        <v>46265.58240677083</v>
       </c>
       <c r="E83" s="9" t="s">
         <v>231</v>

</xml_diff>

<commit_message>
Actualizacion automatica 2026-09-03 22:39 UTC
</commit_message>
<xml_diff>
--- a/data/50001490 - ZITRON PERU METRO LIMA PV04-PV05.xlsx
+++ b/data/50001490 - ZITRON PERU METRO LIMA PV04-PV05.xlsx
@@ -6558,7 +6558,7 @@
       </c>
       <c r="C85" s="9"/>
       <c r="D85" s="8">
-        <v>46262.80754692129</v>
+        <v>46268.828274328705</v>
       </c>
       <c r="E85" s="9" t="s">
         <v>290</v>
@@ -6666,9 +6666,11 @@
       <c r="B87" s="8">
         <v>46073.69994638889</v>
       </c>
-      <c r="C87" s="9"/>
+      <c r="C87" s="8">
+        <v>46268.828154664356</v>
+      </c>
       <c r="D87" s="8">
-        <v>46237.53257923611</v>
+        <v>46268.82815729167</v>
       </c>
       <c r="E87" s="9" t="s">
         <v>261</v>
@@ -6733,7 +6735,7 @@
         <v>46262.80753832176</v>
       </c>
       <c r="D88" s="5">
-        <v>46262.807540567126</v>
+        <v>46268.828162418984</v>
       </c>
       <c r="E88" s="6" t="s">
         <v>301</v>
@@ -6794,9 +6796,11 @@
       <c r="B89" s="8">
         <v>46073.69994695602</v>
       </c>
-      <c r="C89" s="9"/>
+      <c r="C89" s="8">
+        <v>46268.82826504629</v>
+      </c>
       <c r="D89" s="8">
-        <v>46262.80754540509</v>
+        <v>46268.82826701389</v>
       </c>
       <c r="E89" s="9" t="s">
         <v>306</v>
@@ -6906,7 +6910,7 @@
       </c>
       <c r="C91" s="9"/>
       <c r="D91" s="8">
-        <v>46174.16833755787</v>
+        <v>46268.82827175926</v>
       </c>
       <c r="E91" s="9" t="s">
         <v>312</v>
@@ -6969,7 +6973,7 @@
       </c>
       <c r="C92" s="6"/>
       <c r="D92" s="5">
-        <v>46174.168340185184</v>
+        <v>46268.82827357639</v>
       </c>
       <c r="E92" s="6" t="s">
         <v>316</v>

</xml_diff>